<commit_message>
Added recruitment CRM competitor analysis and daily progress
</commit_message>
<xml_diff>
--- a/Defining ICP/Defined Leads.xlsx
+++ b/Defining ICP/Defined Leads.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\R E E M\Documents\EVA Ops Training\Defining ICP\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4C574FF4-F632-4B60-BC64-45BD5821391F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FAE49A41-7974-48EE-98E7-BABE72BB8C29}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{DAB7335F-B748-4A40-8146-0BCBFC1873B2}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="336" uniqueCount="240">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="391" uniqueCount="283">
   <si>
     <t>Name</t>
   </si>
@@ -745,6 +745,135 @@
   </si>
   <si>
     <t>https://tawazunuae.com/</t>
+  </si>
+  <si>
+    <t>Pacific Recruitment Services</t>
+  </si>
+  <si>
+    <t>https://pacificrts.com/</t>
+  </si>
+  <si>
+    <t>Staffing and Recruiting</t>
+  </si>
+  <si>
+    <t>Recruitment Agencies</t>
+  </si>
+  <si>
+    <t>11~50</t>
+  </si>
+  <si>
+    <t>Syed Benazeer Ghani | LinkedIn</t>
+  </si>
+  <si>
+    <t>Syed Benazeer Ghani</t>
+  </si>
+  <si>
+    <t>Head of Recruitment </t>
+  </si>
+  <si>
+    <t>benazeer@pacificrts.com</t>
+  </si>
+  <si>
+    <t>Handles recruitment and client coordination workflows for industrial hiring operations.</t>
+  </si>
+  <si>
+    <t>Abdel Rahman Yousif</t>
+  </si>
+  <si>
+    <t>Quickplus Recruitment Services</t>
+  </si>
+  <si>
+    <t>Abdel Rahman Yousif | LinkedIn</t>
+  </si>
+  <si>
+    <t>abdulrahman@quickplus-recruitment.com</t>
+  </si>
+  <si>
+    <t>+971 4 408 9000</t>
+  </si>
+  <si>
+    <t>quickplus-recruitment.com</t>
+  </si>
+  <si>
+    <t>Handles recruitment and staffing workflows for hiring operations.</t>
+  </si>
+  <si>
+    <t>Recruitment Manager</t>
+  </si>
+  <si>
+    <t>rabia.altunay@recruitithub.com</t>
+  </si>
+  <si>
+    <t>Rabia Altunay</t>
+  </si>
+  <si>
+    <t>HR &amp; Recruitment Manager</t>
+  </si>
+  <si>
+    <t> Recruit IT - IT Recruitment &amp; HR Consultancy</t>
+  </si>
+  <si>
+    <t>Rabia Altunay | LinkedIn</t>
+  </si>
+  <si>
+    <t>http://www.recruitithub.com</t>
+  </si>
+  <si>
+    <t>0850 441 08 43</t>
+  </si>
+  <si>
+    <t>Manages talent acquisition, sourcing, and recruitment workflows for IT and HR consulting operations.</t>
+  </si>
+  <si>
+    <t>Abdurrahman Ansari</t>
+  </si>
+  <si>
+    <t>Arbete Careers</t>
+  </si>
+  <si>
+    <t>Abdurrahman Ansari | LinkedIn</t>
+  </si>
+  <si>
+    <t>Recruitment Head</t>
+  </si>
+  <si>
+    <t>Manages recruitment and talent acquisition operations for corporate hiring.</t>
+  </si>
+  <si>
+    <t>ansari@arbetecareers.com</t>
+  </si>
+  <si>
+    <t>https://arbetecareers.com/</t>
+  </si>
+  <si>
+    <t>Human Resources</t>
+  </si>
+  <si>
+    <t>Headhunter</t>
+  </si>
+  <si>
+    <t>Stream Recruitment</t>
+  </si>
+  <si>
+    <t>Jawaher Al Jneibi | LinkedIn</t>
+  </si>
+  <si>
+    <t>Jawaher Al Jneibi</t>
+  </si>
+  <si>
+    <t>Works in recruitment and talent sourcing with experience using ATS and hiring workflows.</t>
+  </si>
+  <si>
+    <t>jawaher@streamrecruitment.ae</t>
+  </si>
+  <si>
+    <t>https://streamrecruitment.ae/</t>
+  </si>
+  <si>
+    <t>+971 2 444 4405</t>
+  </si>
+  <si>
+    <t>Abu Dhabi</t>
   </si>
 </sst>
 </file>
@@ -806,12 +935,18 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8"/>
+        <bgColor indexed="64"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -837,8 +972,6 @@
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="1" applyFont="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -846,20 +979,30 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
+      <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="17" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="16" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="left"/>
+    <xf numFmtId="17" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1" applyAlignment="1">
-      <alignment horizontal="left"/>
+    <xf numFmtId="16" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -1176,73 +1319,73 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3B2D820C-3568-45BE-99C1-F7479358E85B}">
-  <dimension ref="A1:M31"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <dimension ref="A1:M36"/>
+  <sheetFormatPr defaultRowHeight="15.6" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="19.21875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="25.88671875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="21.88671875" style="2" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="25.88671875" style="1" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="47.6640625" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="67.77734375" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="94.21875" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="12.77734375" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="32.5546875" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="17.33203125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="12.77734375" style="1" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="36.33203125" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="17.33203125" style="11" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="42.109375" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="25.77734375" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="11.77734375" customWidth="1"/>
-    <col min="12" max="12" width="11" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="16.6640625" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="25.77734375" style="1" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="11.77734375" style="1" customWidth="1"/>
+    <col min="12" max="12" width="11" style="1" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="18.88671875" style="1" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:13" s="3" customFormat="1" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A1" s="2" t="s">
+    <row r="1" spans="1:13" s="10" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A1" s="9" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="2" t="s">
+      <c r="B1" s="9" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="2" t="s">
+      <c r="C1" s="9" t="s">
         <v>3</v>
       </c>
-      <c r="D1" s="2" t="s">
+      <c r="D1" s="9" t="s">
         <v>2</v>
       </c>
-      <c r="E1" s="2" t="s">
+      <c r="E1" s="9" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="2" t="s">
+      <c r="F1" s="9" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="2" t="s">
+      <c r="G1" s="9" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="2" t="s">
+      <c r="H1" s="9" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="2" t="s">
+      <c r="I1" s="9" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="2" t="s">
+      <c r="J1" s="9" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="2" t="s">
+      <c r="K1" s="9" t="s">
         <v>10</v>
       </c>
-      <c r="L1" s="2" t="s">
+      <c r="L1" s="9" t="s">
         <v>11</v>
       </c>
-      <c r="M1" s="2" t="s">
+      <c r="M1" s="9" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="2" spans="1:13" ht="16.8" x14ac:dyDescent="0.4">
-      <c r="A2" s="12" t="s">
+    <row r="2" spans="1:13" ht="16.8" x14ac:dyDescent="0.3">
+      <c r="A2" s="2" t="s">
         <v>14</v>
       </c>
       <c r="B2" s="6" t="s">
         <v>15</v>
       </c>
-      <c r="C2" s="8" t="s">
+      <c r="C2" s="6" t="s">
         <v>16</v>
       </c>
       <c r="D2" s="4" t="s">
@@ -1254,30 +1397,30 @@
       <c r="F2" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="I2" s="7" t="s">
+      <c r="I2" s="5" t="s">
         <v>20</v>
       </c>
-      <c r="J2" s="3" t="s">
+      <c r="J2" s="2" t="s">
         <v>18</v>
       </c>
       <c r="K2" s="1">
         <v>1976</v>
       </c>
-      <c r="L2" s="5" t="s">
+      <c r="L2" s="14" t="s">
         <v>21</v>
       </c>
-      <c r="M2" t="s">
+      <c r="M2" s="1" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="3" spans="1:13" ht="16.8" x14ac:dyDescent="0.35">
-      <c r="A3" s="12" t="s">
+    <row r="3" spans="1:13" ht="16.8" x14ac:dyDescent="0.3">
+      <c r="A3" s="2" t="s">
         <v>23</v>
       </c>
-      <c r="B3" s="3" t="s">
+      <c r="B3" s="2" t="s">
         <v>24</v>
       </c>
-      <c r="C3" s="8" t="s">
+      <c r="C3" s="6" t="s">
         <v>25</v>
       </c>
       <c r="D3" s="4" t="s">
@@ -1295,27 +1438,27 @@
       <c r="I3" s="4" t="s">
         <v>27</v>
       </c>
-      <c r="J3" t="s">
+      <c r="J3" s="1" t="s">
         <v>30</v>
       </c>
       <c r="K3" s="1">
         <v>1964</v>
       </c>
-      <c r="L3" s="5" t="s">
+      <c r="L3" s="14" t="s">
         <v>26</v>
       </c>
-      <c r="M3" t="s">
+      <c r="M3" s="1" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="4" spans="1:13" ht="16.8" x14ac:dyDescent="0.35">
-      <c r="A4" t="s">
+    <row r="4" spans="1:13" ht="16.8" x14ac:dyDescent="0.3">
+      <c r="A4" s="2" t="s">
         <v>35</v>
       </c>
-      <c r="B4" t="s">
+      <c r="B4" s="1" t="s">
         <v>33</v>
       </c>
-      <c r="C4" s="8" t="s">
+      <c r="C4" s="6" t="s">
         <v>36</v>
       </c>
       <c r="D4" s="4" t="s">
@@ -1330,33 +1473,33 @@
       <c r="G4" t="s">
         <v>41</v>
       </c>
-      <c r="H4" s="4" t="s">
+      <c r="H4" s="12" t="s">
         <v>40</v>
       </c>
       <c r="I4" s="4" t="s">
         <v>39</v>
       </c>
-      <c r="J4" t="s">
+      <c r="J4" s="1" t="s">
         <v>38</v>
       </c>
       <c r="K4" s="1">
         <v>1981</v>
       </c>
-      <c r="L4" s="5" t="s">
+      <c r="L4" s="14" t="s">
         <v>26</v>
       </c>
-      <c r="M4" t="s">
+      <c r="M4" s="1" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="5" spans="1:13" ht="16.8" x14ac:dyDescent="0.35">
-      <c r="A5" t="s">
+    <row r="5" spans="1:13" ht="16.8" x14ac:dyDescent="0.3">
+      <c r="A5" s="2" t="s">
         <v>42</v>
       </c>
-      <c r="B5" t="s">
+      <c r="B5" s="1" t="s">
         <v>43</v>
       </c>
-      <c r="C5" s="8" t="s">
+      <c r="C5" s="6" t="s">
         <v>45</v>
       </c>
       <c r="D5" s="4" t="s">
@@ -1371,27 +1514,27 @@
       <c r="I5" s="4" t="s">
         <v>46</v>
       </c>
-      <c r="J5" t="s">
+      <c r="J5" s="1" t="s">
         <v>30</v>
       </c>
       <c r="K5" s="1">
         <v>1952</v>
       </c>
-      <c r="L5" s="5" t="s">
+      <c r="L5" s="14" t="s">
         <v>47</v>
       </c>
-      <c r="M5" t="s">
+      <c r="M5" s="1" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="6" spans="1:13" ht="16.8" x14ac:dyDescent="0.35">
-      <c r="A6" t="s">
+    <row r="6" spans="1:13" ht="16.8" x14ac:dyDescent="0.3">
+      <c r="A6" s="2" t="s">
         <v>54</v>
       </c>
-      <c r="B6" t="s">
+      <c r="B6" s="1" t="s">
         <v>53</v>
       </c>
-      <c r="C6" s="8" t="s">
+      <c r="C6" s="6" t="s">
         <v>52</v>
       </c>
       <c r="D6" s="4" t="s">
@@ -1406,31 +1549,31 @@
       <c r="G6" t="s">
         <v>58</v>
       </c>
-      <c r="H6" s="10"/>
+      <c r="H6" s="13"/>
       <c r="I6" s="4" t="s">
         <v>50</v>
       </c>
-      <c r="J6" t="s">
+      <c r="J6" s="1" t="s">
         <v>56</v>
       </c>
       <c r="K6" s="1">
         <v>2008</v>
       </c>
-      <c r="L6" s="5" t="s">
+      <c r="L6" s="14" t="s">
         <v>51</v>
       </c>
-      <c r="M6" t="s">
+      <c r="M6" s="1" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="7" spans="1:13" ht="16.8" x14ac:dyDescent="0.35">
-      <c r="A7" t="s">
+    <row r="7" spans="1:13" ht="16.8" x14ac:dyDescent="0.3">
+      <c r="A7" s="2" t="s">
         <v>62</v>
       </c>
-      <c r="B7" t="s">
+      <c r="B7" s="1" t="s">
         <v>64</v>
       </c>
-      <c r="C7" s="8" t="s">
+      <c r="C7" s="6" t="s">
         <v>59</v>
       </c>
       <c r="D7" s="4" t="s">
@@ -1442,33 +1585,33 @@
       <c r="F7" s="2" t="s">
         <v>49</v>
       </c>
-      <c r="H7" s="4" t="s">
+      <c r="H7" s="12" t="s">
         <v>61</v>
       </c>
       <c r="I7" s="4" t="s">
         <v>60</v>
       </c>
-      <c r="J7" t="s">
+      <c r="J7" s="1" t="s">
         <v>30</v>
       </c>
       <c r="K7" s="1">
         <v>1967</v>
       </c>
-      <c r="L7" s="5" t="s">
+      <c r="L7" s="14" t="s">
         <v>51</v>
       </c>
-      <c r="M7" t="s">
+      <c r="M7" s="1" t="s">
         <v>22</v>
       </c>
     </row>
     <row r="8" spans="1:13" ht="16.8" x14ac:dyDescent="0.3">
-      <c r="A8" t="s">
+      <c r="A8" s="2" t="s">
         <v>66</v>
       </c>
-      <c r="B8" t="s">
+      <c r="B8" s="1" t="s">
         <v>53</v>
       </c>
-      <c r="C8" s="8" t="s">
+      <c r="C8" s="6" t="s">
         <v>67</v>
       </c>
       <c r="D8" s="4" t="s">
@@ -1483,33 +1626,33 @@
       <c r="G8" t="s">
         <v>69</v>
       </c>
-      <c r="H8" s="4" t="s">
+      <c r="H8" s="12" t="s">
         <v>71</v>
       </c>
       <c r="I8" s="4" t="s">
         <v>70</v>
       </c>
-      <c r="J8" t="s">
+      <c r="J8" s="1" t="s">
         <v>56</v>
       </c>
       <c r="K8" s="1">
         <v>2004</v>
       </c>
-      <c r="L8" s="11">
+      <c r="L8" s="14">
         <v>23</v>
       </c>
-      <c r="M8" t="s">
+      <c r="M8" s="1" t="s">
         <v>22</v>
       </c>
     </row>
     <row r="9" spans="1:13" ht="16.8" x14ac:dyDescent="0.3">
-      <c r="A9" t="s">
+      <c r="A9" s="2" t="s">
         <v>80</v>
       </c>
-      <c r="B9" t="s">
+      <c r="B9" s="1" t="s">
         <v>53</v>
       </c>
-      <c r="C9" s="8" t="s">
+      <c r="C9" s="6" t="s">
         <v>74</v>
       </c>
       <c r="D9" s="4" t="s">
@@ -1524,33 +1667,33 @@
       <c r="G9" t="s">
         <v>81</v>
       </c>
-      <c r="H9" s="4" t="s">
+      <c r="H9" s="12" t="s">
         <v>76</v>
       </c>
       <c r="I9" s="4" t="s">
         <v>75</v>
       </c>
-      <c r="J9" t="s">
+      <c r="J9" s="1" t="s">
         <v>82</v>
       </c>
       <c r="K9" s="1">
         <v>1976</v>
       </c>
-      <c r="L9" t="s">
+      <c r="L9" s="1" t="s">
         <v>77</v>
       </c>
-      <c r="M9" t="s">
+      <c r="M9" s="1" t="s">
         <v>22</v>
       </c>
     </row>
     <row r="10" spans="1:13" ht="16.8" x14ac:dyDescent="0.3">
-      <c r="A10" t="s">
+      <c r="A10" s="2" t="s">
         <v>89</v>
       </c>
-      <c r="B10" t="s">
+      <c r="B10" s="1" t="s">
         <v>84</v>
       </c>
-      <c r="C10" s="8" t="s">
+      <c r="C10" s="6" t="s">
         <v>85</v>
       </c>
       <c r="D10" s="4" t="s">
@@ -1565,33 +1708,33 @@
       <c r="G10" s="4" t="s">
         <v>90</v>
       </c>
-      <c r="H10" s="4" t="s">
+      <c r="H10" s="12" t="s">
         <v>91</v>
       </c>
       <c r="I10" s="4" t="s">
         <v>86</v>
       </c>
-      <c r="J10" t="s">
+      <c r="J10" s="1" t="s">
         <v>87</v>
       </c>
       <c r="K10" s="1">
         <v>2022</v>
       </c>
-      <c r="L10" s="11">
+      <c r="L10" s="14">
         <v>21</v>
       </c>
-      <c r="M10" t="s">
+      <c r="M10" s="1" t="s">
         <v>22</v>
       </c>
     </row>
     <row r="11" spans="1:13" ht="16.8" x14ac:dyDescent="0.3">
-      <c r="A11" t="s">
+      <c r="A11" s="2" t="s">
         <v>92</v>
       </c>
-      <c r="B11" t="s">
+      <c r="B11" s="1" t="s">
         <v>93</v>
       </c>
-      <c r="C11" s="8" t="s">
+      <c r="C11" s="6" t="s">
         <v>94</v>
       </c>
       <c r="D11" s="4" t="s">
@@ -1606,33 +1749,33 @@
       <c r="G11" t="s">
         <v>98</v>
       </c>
-      <c r="H11" t="s">
+      <c r="H11" s="11" t="s">
         <v>99</v>
       </c>
       <c r="I11" s="4" t="s">
         <v>95</v>
       </c>
-      <c r="J11" t="s">
+      <c r="J11" s="1" t="s">
         <v>97</v>
       </c>
       <c r="K11" s="1">
         <v>2024</v>
       </c>
-      <c r="L11" s="13" t="s">
+      <c r="L11" s="15" t="s">
         <v>96</v>
       </c>
-      <c r="M11" t="s">
+      <c r="M11" s="1" t="s">
         <v>22</v>
       </c>
     </row>
     <row r="12" spans="1:13" ht="16.8" x14ac:dyDescent="0.3">
-      <c r="A12" t="s">
+      <c r="A12" s="2" t="s">
         <v>102</v>
       </c>
-      <c r="B12" t="s">
+      <c r="B12" s="1" t="s">
         <v>103</v>
       </c>
-      <c r="C12" s="8" t="s">
+      <c r="C12" s="6" t="s">
         <v>104</v>
       </c>
       <c r="D12" s="4" t="s">
@@ -1650,27 +1793,27 @@
       <c r="I12" s="4" t="s">
         <v>108</v>
       </c>
-      <c r="J12" t="s">
+      <c r="J12" s="1" t="s">
         <v>107</v>
       </c>
       <c r="K12" s="1">
         <v>2017</v>
       </c>
-      <c r="L12" s="14" t="s">
+      <c r="L12" s="16" t="s">
         <v>106</v>
       </c>
-      <c r="M12" t="s">
+      <c r="M12" s="1" t="s">
         <v>116</v>
       </c>
     </row>
     <row r="13" spans="1:13" ht="16.8" x14ac:dyDescent="0.3">
-      <c r="A13" t="s">
+      <c r="A13" s="2" t="s">
         <v>111</v>
       </c>
-      <c r="B13" t="s">
+      <c r="B13" s="1" t="s">
         <v>112</v>
       </c>
-      <c r="C13" s="8" t="s">
+      <c r="C13" s="6" t="s">
         <v>113</v>
       </c>
       <c r="D13" s="4" t="s">
@@ -1682,30 +1825,30 @@
       <c r="F13" s="2" t="s">
         <v>49</v>
       </c>
-      <c r="H13" s="4" t="s">
+      <c r="H13" s="12" t="s">
         <v>114</v>
       </c>
-      <c r="J13" t="s">
+      <c r="J13" s="1" t="s">
         <v>107</v>
       </c>
       <c r="K13" s="1">
         <v>2023</v>
       </c>
-      <c r="L13" s="13" t="s">
+      <c r="L13" s="15" t="s">
         <v>96</v>
       </c>
-      <c r="M13" t="s">
+      <c r="M13" s="1" t="s">
         <v>116</v>
       </c>
     </row>
     <row r="14" spans="1:13" ht="16.8" x14ac:dyDescent="0.3">
-      <c r="A14" t="s">
+      <c r="A14" s="2" t="s">
         <v>121</v>
       </c>
-      <c r="B14" t="s">
+      <c r="B14" s="1" t="s">
         <v>122</v>
       </c>
-      <c r="C14" s="8" t="s">
+      <c r="C14" s="6" t="s">
         <v>123</v>
       </c>
       <c r="D14" s="4" t="s">
@@ -1717,33 +1860,33 @@
       <c r="F14" s="2" t="s">
         <v>49</v>
       </c>
-      <c r="H14" s="4">
+      <c r="H14" s="12">
         <v>966535669887</v>
       </c>
       <c r="I14" s="4" t="s">
         <v>120</v>
       </c>
-      <c r="J14" t="s">
+      <c r="J14" s="1" t="s">
         <v>107</v>
       </c>
       <c r="K14" s="1">
         <v>2010</v>
       </c>
-      <c r="L14" t="s">
+      <c r="L14" s="1" t="s">
         <v>96</v>
       </c>
-      <c r="M14" t="s">
+      <c r="M14" s="1" t="s">
         <v>116</v>
       </c>
     </row>
     <row r="15" spans="1:13" ht="16.8" x14ac:dyDescent="0.3">
-      <c r="A15" t="s">
+      <c r="A15" s="2" t="s">
         <v>124</v>
       </c>
-      <c r="B15" t="s">
+      <c r="B15" s="1" t="s">
         <v>122</v>
       </c>
-      <c r="C15" s="8" t="s">
+      <c r="C15" s="6" t="s">
         <v>125</v>
       </c>
       <c r="D15" s="4" t="s">
@@ -1758,24 +1901,24 @@
       <c r="G15" t="s">
         <v>128</v>
       </c>
-      <c r="J15" t="s">
+      <c r="J15" s="1" t="s">
         <v>107</v>
       </c>
-      <c r="L15" s="15">
+      <c r="L15" s="1">
         <v>18</v>
       </c>
-      <c r="M15" t="s">
+      <c r="M15" s="1" t="s">
         <v>116</v>
       </c>
     </row>
     <row r="16" spans="1:13" ht="16.8" x14ac:dyDescent="0.3">
-      <c r="A16" t="s">
+      <c r="A16" s="2" t="s">
         <v>129</v>
       </c>
-      <c r="B16" t="s">
+      <c r="B16" s="1" t="s">
         <v>131</v>
       </c>
-      <c r="C16" s="8" t="s">
+      <c r="C16" s="6" t="s">
         <v>132</v>
       </c>
       <c r="D16" s="4" t="s">
@@ -1790,33 +1933,33 @@
       <c r="G16" t="s">
         <v>130</v>
       </c>
-      <c r="H16" s="4" t="s">
+      <c r="H16" s="12" t="s">
         <v>134</v>
       </c>
       <c r="I16" s="4" t="s">
         <v>133</v>
       </c>
-      <c r="J16" t="s">
+      <c r="J16" s="1" t="s">
         <v>107</v>
       </c>
       <c r="K16" s="1">
         <v>2006</v>
       </c>
-      <c r="L16" s="15">
+      <c r="L16" s="1">
         <v>19</v>
       </c>
-      <c r="M16" t="s">
+      <c r="M16" s="1" t="s">
         <v>116</v>
       </c>
     </row>
     <row r="17" spans="1:13" ht="16.8" x14ac:dyDescent="0.3">
-      <c r="A17" t="s">
+      <c r="A17" s="2" t="s">
         <v>137</v>
       </c>
-      <c r="B17" t="s">
+      <c r="B17" s="1" t="s">
         <v>138</v>
       </c>
-      <c r="C17" s="8" t="s">
+      <c r="C17" s="6" t="s">
         <v>142</v>
       </c>
       <c r="D17" s="4" t="s">
@@ -1831,33 +1974,33 @@
       <c r="G17" t="s">
         <v>139</v>
       </c>
-      <c r="H17" t="s">
+      <c r="H17" s="11" t="s">
         <v>140</v>
       </c>
       <c r="I17" s="4" t="s">
         <v>143</v>
       </c>
-      <c r="J17" t="s">
+      <c r="J17" s="1" t="s">
         <v>107</v>
       </c>
       <c r="K17" s="1">
         <v>2016</v>
       </c>
-      <c r="L17" s="15">
+      <c r="L17" s="1">
         <v>16</v>
       </c>
-      <c r="M17" t="s">
+      <c r="M17" s="1" t="s">
         <v>116</v>
       </c>
     </row>
     <row r="18" spans="1:13" ht="16.8" x14ac:dyDescent="0.3">
-      <c r="A18" t="s">
+      <c r="A18" s="2" t="s">
         <v>145</v>
       </c>
-      <c r="B18" t="s">
+      <c r="B18" s="1" t="s">
         <v>131</v>
       </c>
-      <c r="C18" s="8" t="s">
+      <c r="C18" s="6" t="s">
         <v>132</v>
       </c>
       <c r="D18" s="4" t="s">
@@ -1872,33 +2015,33 @@
       <c r="G18" t="s">
         <v>147</v>
       </c>
-      <c r="H18" s="4" t="s">
+      <c r="H18" s="12" t="s">
         <v>134</v>
       </c>
-      <c r="I18" s="9" t="s">
+      <c r="I18" s="7" t="s">
         <v>133</v>
       </c>
-      <c r="J18" t="s">
+      <c r="J18" s="1" t="s">
         <v>107</v>
       </c>
       <c r="K18" s="1">
         <v>2006</v>
       </c>
-      <c r="L18" s="15">
+      <c r="L18" s="1">
         <v>19</v>
       </c>
-      <c r="M18" t="s">
+      <c r="M18" s="1" t="s">
         <v>116</v>
       </c>
     </row>
     <row r="19" spans="1:13" ht="16.8" x14ac:dyDescent="0.3">
-      <c r="A19" t="s">
+      <c r="A19" s="2" t="s">
         <v>149</v>
       </c>
-      <c r="B19" t="s">
+      <c r="B19" s="1" t="s">
         <v>131</v>
       </c>
-      <c r="C19" s="8" t="s">
+      <c r="C19" s="6" t="s">
         <v>151</v>
       </c>
       <c r="D19" s="4" t="s">
@@ -1913,33 +2056,33 @@
       <c r="G19" t="s">
         <v>154</v>
       </c>
-      <c r="H19" s="4" t="s">
+      <c r="H19" s="12" t="s">
         <v>153</v>
       </c>
       <c r="I19" s="4" t="s">
         <v>152</v>
       </c>
-      <c r="J19" t="s">
+      <c r="J19" s="1" t="s">
         <v>107</v>
       </c>
       <c r="K19" s="1">
         <v>2006</v>
       </c>
-      <c r="L19" s="15">
+      <c r="L19" s="1">
         <v>16</v>
       </c>
-      <c r="M19" t="s">
+      <c r="M19" s="1" t="s">
         <v>116</v>
       </c>
     </row>
     <row r="20" spans="1:13" ht="16.8" x14ac:dyDescent="0.3">
-      <c r="A20" t="s">
+      <c r="A20" s="2" t="s">
         <v>156</v>
       </c>
-      <c r="B20" t="s">
+      <c r="B20" s="1" t="s">
         <v>131</v>
       </c>
-      <c r="C20" s="8" t="s">
+      <c r="C20" s="6" t="s">
         <v>158</v>
       </c>
       <c r="D20" s="4" t="s">
@@ -1954,33 +2097,33 @@
       <c r="G20" t="s">
         <v>159</v>
       </c>
-      <c r="H20" s="4" t="s">
+      <c r="H20" s="12" t="s">
         <v>161</v>
       </c>
       <c r="I20" s="4" t="s">
         <v>160</v>
       </c>
-      <c r="J20" t="s">
+      <c r="J20" s="1" t="s">
         <v>107</v>
       </c>
       <c r="K20" s="1">
         <v>2017</v>
       </c>
-      <c r="L20" s="15">
+      <c r="L20" s="1">
         <v>5</v>
       </c>
-      <c r="M20" t="s">
+      <c r="M20" s="1" t="s">
         <v>116</v>
       </c>
     </row>
     <row r="21" spans="1:13" ht="16.8" x14ac:dyDescent="0.3">
-      <c r="A21" t="s">
+      <c r="A21" s="2" t="s">
         <v>167</v>
       </c>
-      <c r="B21" t="s">
+      <c r="B21" s="1" t="s">
         <v>131</v>
       </c>
-      <c r="C21" s="8" t="s">
+      <c r="C21" s="6" t="s">
         <v>163</v>
       </c>
       <c r="D21" s="4" t="s">
@@ -1995,27 +2138,27 @@
       <c r="G21" t="s">
         <v>165</v>
       </c>
-      <c r="I21" s="9" t="s">
+      <c r="I21" s="7" t="s">
         <v>164</v>
       </c>
-      <c r="J21" t="s">
+      <c r="J21" s="1" t="s">
         <v>107</v>
       </c>
-      <c r="L21" t="s">
+      <c r="L21" s="1" t="s">
         <v>106</v>
       </c>
-      <c r="M21" t="s">
+      <c r="M21" s="1" t="s">
         <v>116</v>
       </c>
     </row>
     <row r="22" spans="1:13" ht="16.8" x14ac:dyDescent="0.3">
-      <c r="A22" t="s">
+      <c r="A22" s="2" t="s">
         <v>169</v>
       </c>
-      <c r="B22" t="s">
+      <c r="B22" s="1" t="s">
         <v>170</v>
       </c>
-      <c r="C22" s="8" t="s">
+      <c r="C22" s="6" t="s">
         <v>172</v>
       </c>
       <c r="D22" s="4" t="s">
@@ -2030,33 +2173,33 @@
       <c r="G22" t="s">
         <v>173</v>
       </c>
-      <c r="H22" s="4" t="s">
+      <c r="H22" s="12" t="s">
         <v>178</v>
       </c>
       <c r="I22" s="4" t="s">
         <v>174</v>
       </c>
-      <c r="J22" t="s">
+      <c r="J22" s="1" t="s">
         <v>175</v>
       </c>
       <c r="K22" s="1">
         <v>2018</v>
       </c>
-      <c r="L22" t="s">
+      <c r="L22" s="1" t="s">
         <v>176</v>
       </c>
-      <c r="M22" t="s">
+      <c r="M22" s="1" t="s">
         <v>177</v>
       </c>
     </row>
     <row r="23" spans="1:13" ht="16.8" x14ac:dyDescent="0.3">
-      <c r="A23" t="s">
+      <c r="A23" s="2" t="s">
         <v>180</v>
       </c>
-      <c r="B23" t="s">
+      <c r="B23" s="1" t="s">
         <v>181</v>
       </c>
-      <c r="C23" s="8" t="s">
+      <c r="C23" s="6" t="s">
         <v>183</v>
       </c>
       <c r="D23" s="4" t="s">
@@ -2071,33 +2214,33 @@
       <c r="G23" t="s">
         <v>184</v>
       </c>
-      <c r="H23" s="4" t="s">
+      <c r="H23" s="12" t="s">
         <v>185</v>
       </c>
       <c r="I23" s="4" t="s">
         <v>186</v>
       </c>
-      <c r="J23" t="s">
+      <c r="J23" s="1" t="s">
         <v>175</v>
       </c>
       <c r="K23" s="1">
         <v>2018</v>
       </c>
-      <c r="L23" s="15">
+      <c r="L23" s="1">
         <v>8</v>
       </c>
-      <c r="M23" t="s">
+      <c r="M23" s="1" t="s">
         <v>177</v>
       </c>
     </row>
     <row r="24" spans="1:13" ht="16.8" x14ac:dyDescent="0.3">
-      <c r="A24" t="s">
+      <c r="A24" s="2" t="s">
         <v>188</v>
       </c>
-      <c r="B24" t="s">
+      <c r="B24" s="1" t="s">
         <v>181</v>
       </c>
-      <c r="C24" s="8" t="s">
+      <c r="C24" s="6" t="s">
         <v>189</v>
       </c>
       <c r="D24" s="4" t="s">
@@ -2112,33 +2255,33 @@
       <c r="G24" t="s">
         <v>193</v>
       </c>
-      <c r="H24" s="16">
+      <c r="H24" s="12">
         <v>26222318</v>
       </c>
       <c r="I24" s="4" t="s">
         <v>190</v>
       </c>
-      <c r="J24" t="s">
+      <c r="J24" s="1" t="s">
         <v>191</v>
       </c>
       <c r="K24" s="1">
         <v>2004</v>
       </c>
-      <c r="L24" s="15">
+      <c r="L24" s="1">
         <v>10</v>
       </c>
-      <c r="M24" t="s">
+      <c r="M24" s="1" t="s">
         <v>177</v>
       </c>
     </row>
     <row r="25" spans="1:13" ht="16.8" x14ac:dyDescent="0.3">
-      <c r="A25" t="s">
+      <c r="A25" s="2" t="s">
         <v>195</v>
       </c>
-      <c r="B25" t="s">
+      <c r="B25" s="1" t="s">
         <v>181</v>
       </c>
-      <c r="C25" s="8" t="s">
+      <c r="C25" s="6" t="s">
         <v>196</v>
       </c>
       <c r="D25" s="4" t="s">
@@ -2153,30 +2296,30 @@
       <c r="G25" t="s">
         <v>198</v>
       </c>
-      <c r="H25" s="4" t="s">
+      <c r="H25" s="12" t="s">
         <v>200</v>
       </c>
       <c r="I25" s="4" t="s">
         <v>199</v>
       </c>
-      <c r="J25" t="s">
+      <c r="J25" s="1" t="s">
         <v>175</v>
       </c>
-      <c r="L25" s="15">
+      <c r="L25" s="1">
         <v>10</v>
       </c>
-      <c r="M25" t="s">
+      <c r="M25" s="1" t="s">
         <v>177</v>
       </c>
     </row>
     <row r="26" spans="1:13" ht="16.8" x14ac:dyDescent="0.3">
-      <c r="A26" t="s">
+      <c r="A26" s="2" t="s">
         <v>202</v>
       </c>
-      <c r="B26" t="s">
+      <c r="B26" s="1" t="s">
         <v>181</v>
       </c>
-      <c r="C26" s="8" t="s">
+      <c r="C26" s="6" t="s">
         <v>203</v>
       </c>
       <c r="D26" s="4" t="s">
@@ -2191,33 +2334,33 @@
       <c r="G26" t="s">
         <v>205</v>
       </c>
-      <c r="H26" s="16">
+      <c r="H26" s="12">
         <v>554488862</v>
       </c>
       <c r="I26" s="4" t="s">
         <v>206</v>
       </c>
-      <c r="J26" t="s">
+      <c r="J26" s="1" t="s">
         <v>175</v>
       </c>
       <c r="K26" s="1">
         <v>2020</v>
       </c>
-      <c r="L26" s="15">
+      <c r="L26" s="1">
         <v>13</v>
       </c>
-      <c r="M26" t="s">
+      <c r="M26" s="1" t="s">
         <v>177</v>
       </c>
     </row>
     <row r="27" spans="1:13" ht="16.8" x14ac:dyDescent="0.3">
-      <c r="A27" t="s">
+      <c r="A27" s="2" t="s">
         <v>208</v>
       </c>
-      <c r="B27" t="s">
+      <c r="B27" s="1" t="s">
         <v>170</v>
       </c>
-      <c r="C27" s="8" t="s">
+      <c r="C27" s="6" t="s">
         <v>209</v>
       </c>
       <c r="D27" s="4" t="s">
@@ -2232,33 +2375,33 @@
       <c r="G27" t="s">
         <v>212</v>
       </c>
-      <c r="H27" s="16" t="s">
+      <c r="H27" s="12" t="s">
         <v>213</v>
       </c>
       <c r="I27" s="4" t="s">
         <v>211</v>
       </c>
-      <c r="J27" t="s">
+      <c r="J27" s="1" t="s">
         <v>175</v>
       </c>
       <c r="K27" s="1">
         <v>2018</v>
       </c>
-      <c r="L27" s="15">
+      <c r="L27" s="1">
         <v>18</v>
       </c>
-      <c r="M27" t="s">
+      <c r="M27" s="1" t="s">
         <v>177</v>
       </c>
     </row>
     <row r="28" spans="1:13" ht="16.8" x14ac:dyDescent="0.3">
-      <c r="A28" t="s">
+      <c r="A28" s="2" t="s">
         <v>217</v>
       </c>
-      <c r="B28" t="s">
+      <c r="B28" s="1" t="s">
         <v>170</v>
       </c>
-      <c r="C28" s="8" t="s">
+      <c r="C28" s="6" t="s">
         <v>216</v>
       </c>
       <c r="D28" s="4" t="s">
@@ -2273,33 +2416,33 @@
       <c r="G28" t="s">
         <v>218</v>
       </c>
-      <c r="H28" s="16">
+      <c r="H28" s="12">
         <v>97142566675</v>
       </c>
       <c r="I28" s="4" t="s">
         <v>219</v>
       </c>
-      <c r="J28" t="s">
+      <c r="J28" s="1" t="s">
         <v>175</v>
       </c>
       <c r="K28" s="1">
         <v>2020</v>
       </c>
-      <c r="L28" s="15">
+      <c r="L28" s="1">
         <v>11</v>
       </c>
-      <c r="M28" t="s">
+      <c r="M28" s="1" t="s">
         <v>177</v>
       </c>
     </row>
     <row r="29" spans="1:13" ht="16.8" x14ac:dyDescent="0.3">
-      <c r="A29" t="s">
+      <c r="A29" s="2" t="s">
         <v>222</v>
       </c>
-      <c r="B29" t="s">
+      <c r="B29" s="1" t="s">
         <v>181</v>
       </c>
-      <c r="C29" s="8" t="s">
+      <c r="C29" s="6" t="s">
         <v>223</v>
       </c>
       <c r="D29" s="4" t="s">
@@ -2314,33 +2457,33 @@
       <c r="G29" t="s">
         <v>224</v>
       </c>
-      <c r="H29" s="4" t="s">
+      <c r="H29" s="12" t="s">
         <v>226</v>
       </c>
       <c r="I29" s="4" t="s">
         <v>225</v>
       </c>
-      <c r="J29" t="s">
+      <c r="J29" s="1" t="s">
         <v>191</v>
       </c>
       <c r="K29" s="1">
         <v>2021</v>
       </c>
-      <c r="L29" s="15">
+      <c r="L29" s="1">
         <v>4</v>
       </c>
-      <c r="M29" t="s">
+      <c r="M29" s="1" t="s">
         <v>177</v>
       </c>
     </row>
     <row r="30" spans="1:13" ht="16.8" x14ac:dyDescent="0.3">
-      <c r="A30" t="s">
+      <c r="A30" s="2" t="s">
         <v>229</v>
       </c>
-      <c r="B30" t="s">
+      <c r="B30" s="1" t="s">
         <v>170</v>
       </c>
-      <c r="C30" s="8" t="s">
+      <c r="C30" s="6" t="s">
         <v>230</v>
       </c>
       <c r="D30" s="4" t="s">
@@ -2355,61 +2498,269 @@
       <c r="G30" t="s">
         <v>231</v>
       </c>
-      <c r="H30" s="4" t="s">
+      <c r="H30" s="12" t="s">
         <v>233</v>
       </c>
       <c r="I30" s="4" t="s">
         <v>232</v>
       </c>
-      <c r="J30" t="s">
+      <c r="J30" s="1" t="s">
         <v>175</v>
       </c>
       <c r="K30" s="1">
         <v>2013</v>
       </c>
-      <c r="L30" s="15">
+      <c r="L30" s="1">
         <v>20</v>
       </c>
-      <c r="M30" t="s">
+      <c r="M30" s="1" t="s">
         <v>177</v>
       </c>
     </row>
     <row r="31" spans="1:13" ht="16.8" x14ac:dyDescent="0.3">
-      <c r="A31" t="s">
+      <c r="A31" s="2" t="s">
         <v>236</v>
       </c>
-      <c r="B31" t="s">
+      <c r="B31" s="1" t="s">
         <v>170</v>
       </c>
-      <c r="C31" s="8" t="s">
+      <c r="C31" s="6" t="s">
         <v>237</v>
       </c>
       <c r="D31" s="4" t="s">
         <v>235</v>
       </c>
+      <c r="E31" t="s">
+        <v>234</v>
+      </c>
       <c r="F31" s="2" t="s">
         <v>17</v>
       </c>
       <c r="G31" t="s">
         <v>238</v>
       </c>
-      <c r="H31" s="16">
+      <c r="H31" s="12">
         <v>586784488</v>
       </c>
       <c r="I31" s="4" t="s">
         <v>239</v>
       </c>
-      <c r="J31" t="s">
+      <c r="J31" s="1" t="s">
         <v>175</v>
       </c>
       <c r="K31" s="1">
         <v>2023</v>
       </c>
-      <c r="L31" s="15">
+      <c r="L31" s="1">
         <v>8</v>
       </c>
-      <c r="M31" t="s">
+      <c r="M31" s="1" t="s">
         <v>177</v>
+      </c>
+    </row>
+    <row r="32" spans="1:13" ht="16.8" x14ac:dyDescent="0.3">
+      <c r="A32" s="2" t="s">
+        <v>246</v>
+      </c>
+      <c r="B32" s="1" t="s">
+        <v>247</v>
+      </c>
+      <c r="C32" s="6" t="s">
+        <v>240</v>
+      </c>
+      <c r="D32" s="4" t="s">
+        <v>245</v>
+      </c>
+      <c r="E32" t="s">
+        <v>249</v>
+      </c>
+      <c r="F32" s="2" t="s">
+        <v>49</v>
+      </c>
+      <c r="G32" t="s">
+        <v>248</v>
+      </c>
+      <c r="H32" s="12">
+        <v>2652993869</v>
+      </c>
+      <c r="I32" s="4" t="s">
+        <v>241</v>
+      </c>
+      <c r="J32" s="14" t="s">
+        <v>242</v>
+      </c>
+      <c r="K32" s="1">
+        <v>2014</v>
+      </c>
+      <c r="L32" s="15" t="s">
+        <v>244</v>
+      </c>
+      <c r="M32" s="1" t="s">
+        <v>243</v>
+      </c>
+    </row>
+    <row r="33" spans="1:13" ht="16.8" x14ac:dyDescent="0.3">
+      <c r="A33" s="2" t="s">
+        <v>250</v>
+      </c>
+      <c r="B33" s="1" t="s">
+        <v>257</v>
+      </c>
+      <c r="C33" s="6" t="s">
+        <v>251</v>
+      </c>
+      <c r="D33" s="4" t="s">
+        <v>252</v>
+      </c>
+      <c r="E33" t="s">
+        <v>256</v>
+      </c>
+      <c r="F33" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="G33" t="s">
+        <v>253</v>
+      </c>
+      <c r="H33" s="11" t="s">
+        <v>254</v>
+      </c>
+      <c r="I33" s="4" t="s">
+        <v>255</v>
+      </c>
+      <c r="J33" s="14" t="s">
+        <v>242</v>
+      </c>
+      <c r="K33" s="1">
+        <v>2017</v>
+      </c>
+      <c r="L33" s="1">
+        <v>13</v>
+      </c>
+      <c r="M33" s="1" t="s">
+        <v>243</v>
+      </c>
+    </row>
+    <row r="34" spans="1:13" ht="16.8" x14ac:dyDescent="0.3">
+      <c r="A34" s="2" t="s">
+        <v>259</v>
+      </c>
+      <c r="B34" s="1" t="s">
+        <v>260</v>
+      </c>
+      <c r="C34" s="6" t="s">
+        <v>261</v>
+      </c>
+      <c r="D34" s="4" t="s">
+        <v>262</v>
+      </c>
+      <c r="E34" t="s">
+        <v>265</v>
+      </c>
+      <c r="F34" s="2" t="s">
+        <v>79</v>
+      </c>
+      <c r="G34" t="s">
+        <v>258</v>
+      </c>
+      <c r="H34" s="12" t="s">
+        <v>264</v>
+      </c>
+      <c r="I34" s="4" t="s">
+        <v>263</v>
+      </c>
+      <c r="J34" s="14" t="s">
+        <v>242</v>
+      </c>
+      <c r="K34" s="1">
+        <v>2017</v>
+      </c>
+      <c r="L34" s="1">
+        <v>12</v>
+      </c>
+      <c r="M34" s="1" t="s">
+        <v>243</v>
+      </c>
+    </row>
+    <row r="35" spans="1:13" ht="16.8" x14ac:dyDescent="0.3">
+      <c r="A35" s="2" t="s">
+        <v>266</v>
+      </c>
+      <c r="B35" s="1" t="s">
+        <v>269</v>
+      </c>
+      <c r="C35" s="6" t="s">
+        <v>267</v>
+      </c>
+      <c r="D35" s="4" t="s">
+        <v>268</v>
+      </c>
+      <c r="E35" t="s">
+        <v>270</v>
+      </c>
+      <c r="F35" s="1" t="s">
+        <v>49</v>
+      </c>
+      <c r="G35" t="s">
+        <v>271</v>
+      </c>
+      <c r="H35" s="8">
+        <v>966539182585</v>
+      </c>
+      <c r="I35" s="4" t="s">
+        <v>272</v>
+      </c>
+      <c r="J35" s="14" t="s">
+        <v>273</v>
+      </c>
+      <c r="K35" s="1">
+        <v>2019</v>
+      </c>
+      <c r="L35" s="1">
+        <v>13</v>
+      </c>
+      <c r="M35" s="1" t="s">
+        <v>243</v>
+      </c>
+    </row>
+    <row r="36" spans="1:13" ht="16.8" x14ac:dyDescent="0.3">
+      <c r="A36" s="2" t="s">
+        <v>277</v>
+      </c>
+      <c r="B36" s="1" t="s">
+        <v>274</v>
+      </c>
+      <c r="C36" s="6" t="s">
+        <v>275</v>
+      </c>
+      <c r="D36" s="4" t="s">
+        <v>276</v>
+      </c>
+      <c r="E36" t="s">
+        <v>278</v>
+      </c>
+      <c r="F36" s="1" t="s">
+        <v>282</v>
+      </c>
+      <c r="G36" t="s">
+        <v>279</v>
+      </c>
+      <c r="H36" s="11" t="s">
+        <v>281</v>
+      </c>
+      <c r="I36" s="4" t="s">
+        <v>280</v>
+      </c>
+      <c r="J36" s="14" t="s">
+        <v>242</v>
+      </c>
+      <c r="K36" s="1">
+        <v>2013</v>
+      </c>
+      <c r="L36" s="1">
+        <v>19</v>
+      </c>
+      <c r="M36" s="1" t="s">
+        <v>243</v>
       </c>
     </row>
   </sheetData>
@@ -2490,6 +2841,20 @@
     <hyperlink ref="D31" r:id="rId73" display="https://www.linkedin.com/in/ahmadrazaa155/" xr:uid="{A46B9262-BDDB-403C-A25D-2635AEE15617}"/>
     <hyperlink ref="H31" r:id="rId74" display="tel:0586784488" xr:uid="{43C0779E-0AEE-4C85-A7AA-CFDD9A3B15AA}"/>
     <hyperlink ref="I31" r:id="rId75" xr:uid="{D36C2BEA-A49D-441F-A17D-B26E7319C1FC}"/>
+    <hyperlink ref="I32" r:id="rId76" xr:uid="{2A9A480F-53AA-4220-BEB0-6DB71C19F5F3}"/>
+    <hyperlink ref="H32" r:id="rId77" display="tel:02652993869" xr:uid="{D5072072-A8B6-4625-8424-AE3F4FCEC6F8}"/>
+    <hyperlink ref="D32" r:id="rId78" display="https://www.linkedin.com/in/syed-benazeer-ghani-56ab1a90/" xr:uid="{68726B44-B116-47CC-BCD2-491997F7CD56}"/>
+    <hyperlink ref="D33" r:id="rId79" display="https://www.linkedin.com/in/abdulrahman-abd/" xr:uid="{AF76796A-0165-47EB-9910-C1F81B1C4079}"/>
+    <hyperlink ref="I33" r:id="rId80" display="https://quickplus-recruitment.com/" xr:uid="{6A689384-3EE0-4C0F-ACCE-4625C41567A6}"/>
+    <hyperlink ref="C34" r:id="rId81" location="/contacts/6a078bc6120ac8001174aa11?accountId=6a078bc6120ac8001174aa13" display="https://app.apollo.io/?_gl=1*q36ca5*_gcl_au*MTUxMjc4Mjc5LjE3NzgwNzQ1NTY.*_ga*NjAyNDkwODczLjE3NzgwNzQ1NTY.*_ga_76XXTC73SP*czE3Nzg4NDMwNDMkbzYkZzAkdDE3Nzg4NDMwNDMkajYwJGwwJGgzNDcxMjAyMg.. - /contacts/6a078bc6120ac8001174aa11?accountId=6a078bc6120ac8001174aa13" xr:uid="{B934623B-B73F-474D-BA43-0638F32F9825}"/>
+    <hyperlink ref="D34" r:id="rId82" display="https://www.linkedin.com/in/rabiaaltunay/" xr:uid="{97A3DD26-9512-41FB-9C5B-5CF06E863C0B}"/>
+    <hyperlink ref="I34" r:id="rId83" display="http://www.recruitithub.com/" xr:uid="{6758E700-6F8A-4972-9D82-4852F07D823B}"/>
+    <hyperlink ref="H34" r:id="rId84" display="tel:0850 441 08 43" xr:uid="{5F516FF0-673A-4F67-B26E-984198CE54D8}"/>
+    <hyperlink ref="D35" r:id="rId85" display="https://www.linkedin.com/in/abdurrahman-ansari/" xr:uid="{8DFE1422-30E9-4B55-B437-44EFE0DA9541}"/>
+    <hyperlink ref="I35" r:id="rId86" xr:uid="{9DD91332-7FA0-450C-BE6C-2C4BF5FB54A1}"/>
+    <hyperlink ref="H35" r:id="rId87" display="tel:+966539182585" xr:uid="{62810195-C7B8-4AFE-9C50-323A5BC98036}"/>
+    <hyperlink ref="D36" r:id="rId88" display="https://www.linkedin.com/in/jawaher-al-jneibi-535a16216/" xr:uid="{7C0EA381-C75D-481A-8FCA-C46402431C34}"/>
+    <hyperlink ref="I36" r:id="rId89" xr:uid="{F3E9733A-E5A8-4F6A-A96C-562C92D3D820}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Add Day 5 recruitment CRM research progress
</commit_message>
<xml_diff>
--- a/Defining ICP/Defined Leads.xlsx
+++ b/Defining ICP/Defined Leads.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\R E E M\Documents\EVA Ops Training\Defining ICP\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FAE49A41-7974-48EE-98E7-BABE72BB8C29}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0C56EBC8-A8FD-4887-A83F-F7F4D9A06188}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{DAB7335F-B748-4A40-8146-0BCBFC1873B2}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="391" uniqueCount="283">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="564" uniqueCount="392">
   <si>
     <t>Name</t>
   </si>
@@ -874,13 +874,353 @@
   </si>
   <si>
     <t>Abu Dhabi</t>
+  </si>
+  <si>
+    <t>Riddhi Parekh</t>
+  </si>
+  <si>
+    <r>
+      <t>HR Manager</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="8"/>
+        <color rgb="FFB8B6B9"/>
+        <rFont val="Segoe UI"/>
+        <family val="2"/>
+      </rPr>
+      <t> </t>
+    </r>
+  </si>
+  <si>
+    <t>Elite HR Consultancy</t>
+  </si>
+  <si>
+    <t>Riddhi Parekh | LinkedIn</t>
+  </si>
+  <si>
+    <t>Strong recruitment lead involved in GCC talent acquisition, executive search, and HR consulting.</t>
+  </si>
+  <si>
+    <t>riddhi@elitehrconsultancy.com</t>
+  </si>
+  <si>
+    <t>+971 55 122 6879</t>
+  </si>
+  <si>
+    <t>www.elitehrconsultancy.com</t>
+  </si>
+  <si>
+    <t>Sam Mazzotta</t>
+  </si>
+  <si>
+    <t>SELECTED RECRUITMENT</t>
+  </si>
+  <si>
+    <t>https://www.selected.ae</t>
+  </si>
+  <si>
+    <t>sam@selected.ae</t>
+  </si>
+  <si>
+    <t>Strong recruitment lead focused on headhunting, placements, and UAE talent acquisition.</t>
+  </si>
+  <si>
+    <t>Sam Mazzotta | LinkedIn</t>
+  </si>
+  <si>
+    <t>Ceni Venugopalan | LinkedIn</t>
+  </si>
+  <si>
+    <t>Recruitment leadership professional managing hiring and talent acquisition activities.</t>
+  </si>
+  <si>
+    <t>Ceni Venugopalan</t>
+  </si>
+  <si>
+    <t>HIRE HEAD</t>
+  </si>
+  <si>
+    <t>https://hirehead.me/</t>
+  </si>
+  <si>
+    <t>ceni.v@hirehead.me</t>
+  </si>
+  <si>
+    <t>+1 517-316-2860</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2~10 </t>
+  </si>
+  <si>
+    <t>Bharat Fulwani</t>
+  </si>
+  <si>
+    <t>Recruitment manager focused on candidate sourcing and recruitment operations in the UAE market.</t>
+  </si>
+  <si>
+    <t>Bharat F. | LinkedIn</t>
+  </si>
+  <si>
+    <t>Elkho Group</t>
+  </si>
+  <si>
+    <t>b.fulwani@elkho-group.com</t>
+  </si>
+  <si>
+    <t>+33 4 74 07 89 40</t>
+  </si>
+  <si>
+    <t>http://www.elkho-group.com</t>
+  </si>
+  <si>
+    <t>51~200</t>
+  </si>
+  <si>
+    <t xml:space="preserve">
+Yeshma Fernandes</t>
+  </si>
+  <si>
+    <t>Yeshma Fernandes | LinkedIn</t>
+  </si>
+  <si>
+    <t>Strong recruitment lead focused on HR management and talent acquisition in the UAE market.</t>
+  </si>
+  <si>
+    <t>HR Manager </t>
+  </si>
+  <si>
+    <t>Global ME Recruitment Network</t>
+  </si>
+  <si>
+    <t>yeshma.fernandes@globalmerecruitmentnetwork.com</t>
+  </si>
+  <si>
+    <t>https://globalmerecruitmentnetwork.com/</t>
+  </si>
+  <si>
+    <t>+90 212 274 4749</t>
+  </si>
+  <si>
+    <t>Yasmin McKeon | LinkedIn</t>
+  </si>
+  <si>
+    <t>Yasmin McKeon</t>
+  </si>
+  <si>
+    <t>Head of Interim Recruitment</t>
+  </si>
+  <si>
+    <t>Collins Search</t>
+  </si>
+  <si>
+    <t>www.collins-search.com</t>
+  </si>
+  <si>
+    <t>Executive Search Services</t>
+  </si>
+  <si>
+    <t>Strong recruitment lead focused on legal and compliance talent acquisition in the Middle East.</t>
+  </si>
+  <si>
+    <t>yasmin@collins-search.com</t>
+  </si>
+  <si>
+    <t>Giby George</t>
+  </si>
+  <si>
+    <t>Assistant Recruitment Manager</t>
+  </si>
+  <si>
+    <t>BuildWell HR Solutions LLC</t>
+  </si>
+  <si>
+    <t>Giby George | LinkedIn</t>
+  </si>
+  <si>
+    <t>Recruitment professional working in HR and hiring operations within the UAE market.</t>
+  </si>
+  <si>
+    <t>giby.george@buildwellhrs.com</t>
+  </si>
+  <si>
+    <t>https://buildwellhrs.com/</t>
+  </si>
+  <si>
+    <t>Jasmine Sagai</t>
+  </si>
+  <si>
+    <t>Jasmine Sagai | LinkedIn</t>
+  </si>
+  <si>
+    <t>Senior recruitment professional handling executive search and international talent sourcing for healthcare roles.</t>
+  </si>
+  <si>
+    <t>DAVIDSON MANAGEMENT CONSULTANTS</t>
+  </si>
+  <si>
+    <t>jasmine@davidsondubai.com</t>
+  </si>
+  <si>
+    <t>http://www.davidsondubai.net</t>
+  </si>
+  <si>
+    <t>https://www.andrewvinell.com/</t>
+  </si>
+  <si>
+    <t>+44 (0)20 3926 7603</t>
+  </si>
+  <si>
+    <t>2~10</t>
+  </si>
+  <si>
+    <t>AVTR</t>
+  </si>
+  <si>
+    <t>Specialized recruiter focused on tax and legal talent acquisition and international recruitment opportunities.</t>
+  </si>
+  <si>
+    <t>Daniela Madden | LinkedIn</t>
+  </si>
+  <si>
+    <t>dm@andrewvinell.com</t>
+  </si>
+  <si>
+    <t>Daniela Madden</t>
+  </si>
+  <si>
+    <t>Head of UK and International Recruitment</t>
+  </si>
+  <si>
+    <t>Head of Recruitment handling international executive and healthcare leadership hiring across GCC markets.</t>
+  </si>
+  <si>
+    <t>Rajiv D D. | LinkedIn</t>
+  </si>
+  <si>
+    <t>Rajiv D</t>
+  </si>
+  <si>
+    <t>rajiv@davidsondubai.com</t>
+  </si>
+  <si>
+    <t>Masooda Khan</t>
+  </si>
+  <si>
+    <t>TASC Outsourcing</t>
+  </si>
+  <si>
+    <t>Masooda Khan | LinkedIn</t>
+  </si>
+  <si>
+    <t>recruitment leader specializing in global talent acquisition and headhunting at a major outsourcing and staffing company.</t>
+  </si>
+  <si>
+    <t>masooda@tascoutsourcing.com</t>
+  </si>
+  <si>
+    <t>+971 4 358 8500</t>
+  </si>
+  <si>
+    <t>https://tascoutsourcing.com/en</t>
+  </si>
+  <si>
+    <t>1000+</t>
+  </si>
+  <si>
+    <t>Recruitment Consulting Manager specializing in GCC hiring, strategic talent acquisition, and end-to-end recruitment operations.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">
+Sinduja V</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Recruitment Consulting Manager </t>
+  </si>
+  <si>
+    <t>Sinduja V | LinkedIn</t>
+  </si>
+  <si>
+    <t>sinduja@business-umbrella.com</t>
+  </si>
+  <si>
+    <t>+971 55 442 6831</t>
+  </si>
+  <si>
+    <t>https://www.business-umbrella.com</t>
+  </si>
+  <si>
+    <t>Recruitment Consulting Manager</t>
+  </si>
+  <si>
+    <t>Turki Al Otaibi</t>
+  </si>
+  <si>
+    <t>turki.otaibi@eramgroup.com</t>
+  </si>
+  <si>
+    <t>Turki Al Otaibi | LinkedIn</t>
+  </si>
+  <si>
+    <t>Talent acquisition and recruitment professional managing large-scale hiring and mobilization workflows in Saudi Arabia.</t>
+  </si>
+  <si>
+    <t>Eram Talent</t>
+  </si>
+  <si>
+    <t>http://eramtalent.com/</t>
+  </si>
+  <si>
+    <t>+966 13 8493777</t>
+  </si>
+  <si>
+    <t>Recruitment and executive search professional managing end-to-end talent acquisition and RPO solutions across global markets.</t>
+  </si>
+  <si>
+    <t>Nadeem Amjad</t>
+  </si>
+  <si>
+    <t>M. Nadeem Amjad | LinkedIn</t>
+  </si>
+  <si>
+    <t>RFS HR CONSULTANCY</t>
+  </si>
+  <si>
+    <t>http://www.rfsonshr.com</t>
+  </si>
+  <si>
+    <t>971 50 434 4675</t>
+  </si>
+  <si>
+    <t>nadeem@rfsonshr.com</t>
+  </si>
+  <si>
+    <t>Talent acquisition and recruitment operations professional managing HR outsourcing and recruitment workflows.</t>
+  </si>
+  <si>
+    <t>Stivan Quadros</t>
+  </si>
+  <si>
+    <t>Stivan Quadros | LinkedIn</t>
+  </si>
+  <si>
+    <t>Tadbeer Recruitment</t>
+  </si>
+  <si>
+    <t>stivan@tadbeerco.com</t>
+  </si>
+  <si>
+    <t>+966 92 002 9279</t>
+  </si>
+  <si>
+    <t>https://tadbeerco.com/</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="8" x14ac:knownFonts="1">
+  <fonts count="9" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -934,6 +1274,12 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="8"/>
+      <color rgb="FFB8B6B9"/>
+      <name val="Segoe UI"/>
+      <family val="2"/>
+    </font>
   </fonts>
   <fills count="3">
     <fill>
@@ -962,7 +1308,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="17">
+  <cellXfs count="18">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -1004,6 +1350,7 @@
     <xf numFmtId="16" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -1319,17 +1666,17 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3B2D820C-3568-45BE-99C1-F7479358E85B}">
-  <dimension ref="A1:M36"/>
+  <dimension ref="A1:M51"/>
   <sheetFormatPr defaultRowHeight="15.6" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="21.88671875" style="2" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="25.88671875" style="1" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="35.88671875" style="1" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="47.6640625" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="67.77734375" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="94.21875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="110.88671875" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="12.77734375" style="1" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="36.33203125" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="17.33203125" style="11" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="46.5546875" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="18.44140625" style="11" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="42.109375" bestFit="1" customWidth="1"/>
     <col min="10" max="10" width="25.77734375" style="1" bestFit="1" customWidth="1"/>
     <col min="11" max="11" width="11.77734375" style="1" customWidth="1"/>
@@ -2760,6 +3107,600 @@
         <v>19</v>
       </c>
       <c r="M36" s="1" t="s">
+        <v>243</v>
+      </c>
+    </row>
+    <row r="37" spans="1:13" ht="16.8" x14ac:dyDescent="0.3">
+      <c r="A37" s="2" t="s">
+        <v>283</v>
+      </c>
+      <c r="B37" s="1" t="s">
+        <v>284</v>
+      </c>
+      <c r="C37" s="6" t="s">
+        <v>285</v>
+      </c>
+      <c r="D37" s="4" t="s">
+        <v>286</v>
+      </c>
+      <c r="E37" t="s">
+        <v>287</v>
+      </c>
+      <c r="F37" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="G37" t="s">
+        <v>288</v>
+      </c>
+      <c r="H37" s="11" t="s">
+        <v>289</v>
+      </c>
+      <c r="I37" s="4" t="s">
+        <v>290</v>
+      </c>
+      <c r="J37" s="14" t="s">
+        <v>242</v>
+      </c>
+      <c r="L37" s="1">
+        <v>12</v>
+      </c>
+      <c r="M37" s="1" t="s">
+        <v>243</v>
+      </c>
+    </row>
+    <row r="38" spans="1:13" ht="16.8" x14ac:dyDescent="0.3">
+      <c r="A38" s="2" t="s">
+        <v>291</v>
+      </c>
+      <c r="B38" s="1" t="s">
+        <v>269</v>
+      </c>
+      <c r="C38" s="6" t="s">
+        <v>292</v>
+      </c>
+      <c r="D38" s="4" t="s">
+        <v>296</v>
+      </c>
+      <c r="E38" t="s">
+        <v>295</v>
+      </c>
+      <c r="F38" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="G38" t="s">
+        <v>294</v>
+      </c>
+      <c r="I38" s="4" t="s">
+        <v>293</v>
+      </c>
+      <c r="J38" s="14" t="s">
+        <v>242</v>
+      </c>
+      <c r="K38" s="1">
+        <v>2024</v>
+      </c>
+      <c r="L38" s="1">
+        <v>6</v>
+      </c>
+      <c r="M38" s="1" t="s">
+        <v>243</v>
+      </c>
+    </row>
+    <row r="39" spans="1:13" ht="16.8" x14ac:dyDescent="0.3">
+      <c r="A39" s="2" t="s">
+        <v>299</v>
+      </c>
+      <c r="B39" s="1" t="s">
+        <v>269</v>
+      </c>
+      <c r="C39" s="6" t="s">
+        <v>300</v>
+      </c>
+      <c r="D39" s="4" t="s">
+        <v>297</v>
+      </c>
+      <c r="E39" t="s">
+        <v>298</v>
+      </c>
+      <c r="F39" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="G39" t="s">
+        <v>302</v>
+      </c>
+      <c r="H39" s="11" t="s">
+        <v>303</v>
+      </c>
+      <c r="I39" s="4" t="s">
+        <v>301</v>
+      </c>
+      <c r="J39" s="14" t="s">
+        <v>242</v>
+      </c>
+      <c r="L39" s="1" t="s">
+        <v>304</v>
+      </c>
+      <c r="M39" s="1" t="s">
+        <v>243</v>
+      </c>
+    </row>
+    <row r="40" spans="1:13" ht="16.8" x14ac:dyDescent="0.3">
+      <c r="A40" s="2" t="s">
+        <v>305</v>
+      </c>
+      <c r="B40" s="1" t="s">
+        <v>257</v>
+      </c>
+      <c r="C40" s="6" t="s">
+        <v>308</v>
+      </c>
+      <c r="D40" s="4" t="s">
+        <v>307</v>
+      </c>
+      <c r="E40" t="s">
+        <v>306</v>
+      </c>
+      <c r="F40" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="G40" t="s">
+        <v>309</v>
+      </c>
+      <c r="H40" s="11" t="s">
+        <v>310</v>
+      </c>
+      <c r="I40" s="4" t="s">
+        <v>311</v>
+      </c>
+      <c r="J40" s="14" t="s">
+        <v>242</v>
+      </c>
+      <c r="K40" s="1">
+        <v>2008</v>
+      </c>
+      <c r="L40" s="1" t="s">
+        <v>312</v>
+      </c>
+      <c r="M40" s="1" t="s">
+        <v>243</v>
+      </c>
+    </row>
+    <row r="41" spans="1:13" ht="16.8" x14ac:dyDescent="0.3">
+      <c r="A41" s="2" t="s">
+        <v>313</v>
+      </c>
+      <c r="B41" s="1" t="s">
+        <v>316</v>
+      </c>
+      <c r="C41" s="6" t="s">
+        <v>317</v>
+      </c>
+      <c r="D41" s="4" t="s">
+        <v>314</v>
+      </c>
+      <c r="E41" t="s">
+        <v>315</v>
+      </c>
+      <c r="F41" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="G41" t="s">
+        <v>318</v>
+      </c>
+      <c r="H41" s="11" t="s">
+        <v>320</v>
+      </c>
+      <c r="I41" s="4" t="s">
+        <v>319</v>
+      </c>
+      <c r="J41" s="14" t="s">
+        <v>242</v>
+      </c>
+      <c r="L41" s="1" t="s">
+        <v>304</v>
+      </c>
+      <c r="M41" s="1" t="s">
+        <v>243</v>
+      </c>
+    </row>
+    <row r="42" spans="1:13" ht="16.8" x14ac:dyDescent="0.3">
+      <c r="A42" s="2" t="s">
+        <v>322</v>
+      </c>
+      <c r="B42" s="1" t="s">
+        <v>323</v>
+      </c>
+      <c r="C42" s="6" t="s">
+        <v>324</v>
+      </c>
+      <c r="D42" s="4" t="s">
+        <v>321</v>
+      </c>
+      <c r="E42" t="s">
+        <v>327</v>
+      </c>
+      <c r="F42" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="G42" t="s">
+        <v>328</v>
+      </c>
+      <c r="I42" s="4" t="s">
+        <v>325</v>
+      </c>
+      <c r="J42" s="14" t="s">
+        <v>326</v>
+      </c>
+      <c r="L42" s="1" t="s">
+        <v>304</v>
+      </c>
+      <c r="M42" s="1" t="s">
+        <v>243</v>
+      </c>
+    </row>
+    <row r="43" spans="1:13" ht="16.8" x14ac:dyDescent="0.35">
+      <c r="A43" s="2" t="s">
+        <v>329</v>
+      </c>
+      <c r="B43" s="17" t="s">
+        <v>330</v>
+      </c>
+      <c r="C43" s="6" t="s">
+        <v>331</v>
+      </c>
+      <c r="D43" s="4" t="s">
+        <v>332</v>
+      </c>
+      <c r="E43" t="s">
+        <v>333</v>
+      </c>
+      <c r="F43" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="G43" t="s">
+        <v>334</v>
+      </c>
+      <c r="H43" s="11">
+        <v>971585850831</v>
+      </c>
+      <c r="I43" s="4" t="s">
+        <v>335</v>
+      </c>
+      <c r="J43" s="14" t="s">
+        <v>273</v>
+      </c>
+      <c r="K43" s="1">
+        <v>2018</v>
+      </c>
+      <c r="L43" s="1" t="s">
+        <v>244</v>
+      </c>
+      <c r="M43" s="1" t="s">
+        <v>243</v>
+      </c>
+    </row>
+    <row r="44" spans="1:13" ht="16.8" x14ac:dyDescent="0.3">
+      <c r="A44" s="2" t="s">
+        <v>336</v>
+      </c>
+      <c r="B44" s="1" t="s">
+        <v>257</v>
+      </c>
+      <c r="C44" s="6" t="s">
+        <v>339</v>
+      </c>
+      <c r="D44" s="4" t="s">
+        <v>337</v>
+      </c>
+      <c r="E44" t="s">
+        <v>338</v>
+      </c>
+      <c r="F44" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="G44" t="s">
+        <v>340</v>
+      </c>
+      <c r="H44" s="11">
+        <v>43555961</v>
+      </c>
+      <c r="I44" s="4" t="s">
+        <v>341</v>
+      </c>
+      <c r="J44" s="14" t="s">
+        <v>242</v>
+      </c>
+      <c r="K44" s="1">
+        <v>2011</v>
+      </c>
+      <c r="L44" s="1" t="s">
+        <v>244</v>
+      </c>
+      <c r="M44" s="1" t="s">
+        <v>243</v>
+      </c>
+    </row>
+    <row r="45" spans="1:13" ht="16.8" x14ac:dyDescent="0.3">
+      <c r="A45" s="2" t="s">
+        <v>349</v>
+      </c>
+      <c r="B45" s="1" t="s">
+        <v>350</v>
+      </c>
+      <c r="C45" s="6" t="s">
+        <v>345</v>
+      </c>
+      <c r="D45" s="4" t="s">
+        <v>347</v>
+      </c>
+      <c r="E45" t="s">
+        <v>346</v>
+      </c>
+      <c r="F45" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="G45" t="s">
+        <v>348</v>
+      </c>
+      <c r="H45" s="4" t="s">
+        <v>343</v>
+      </c>
+      <c r="I45" s="4" t="s">
+        <v>342</v>
+      </c>
+      <c r="J45" s="14" t="s">
+        <v>242</v>
+      </c>
+      <c r="K45" s="1">
+        <v>2018</v>
+      </c>
+      <c r="L45" s="1" t="s">
+        <v>344</v>
+      </c>
+      <c r="M45" s="1" t="s">
+        <v>243</v>
+      </c>
+    </row>
+    <row r="46" spans="1:13" ht="16.8" x14ac:dyDescent="0.3">
+      <c r="A46" s="2" t="s">
+        <v>353</v>
+      </c>
+      <c r="B46" s="1" t="s">
+        <v>269</v>
+      </c>
+      <c r="C46" s="6" t="s">
+        <v>339</v>
+      </c>
+      <c r="D46" s="4" t="s">
+        <v>352</v>
+      </c>
+      <c r="E46" t="s">
+        <v>351</v>
+      </c>
+      <c r="F46" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="G46" t="s">
+        <v>354</v>
+      </c>
+      <c r="H46" s="8">
+        <v>43555961</v>
+      </c>
+      <c r="I46" s="4" t="s">
+        <v>341</v>
+      </c>
+      <c r="J46" s="14" t="s">
+        <v>242</v>
+      </c>
+      <c r="K46" s="1">
+        <v>2011</v>
+      </c>
+      <c r="L46" s="1" t="s">
+        <v>244</v>
+      </c>
+      <c r="M46" s="1" t="s">
+        <v>243</v>
+      </c>
+    </row>
+    <row r="47" spans="1:13" ht="16.8" x14ac:dyDescent="0.3">
+      <c r="A47" s="2" t="s">
+        <v>355</v>
+      </c>
+      <c r="B47" s="1" t="s">
+        <v>257</v>
+      </c>
+      <c r="C47" s="6" t="s">
+        <v>356</v>
+      </c>
+      <c r="D47" s="4" t="s">
+        <v>357</v>
+      </c>
+      <c r="E47" t="s">
+        <v>358</v>
+      </c>
+      <c r="F47" s="1" t="s">
+        <v>49</v>
+      </c>
+      <c r="G47" t="s">
+        <v>359</v>
+      </c>
+      <c r="H47" s="11" t="s">
+        <v>360</v>
+      </c>
+      <c r="I47" s="4" t="s">
+        <v>361</v>
+      </c>
+      <c r="J47" s="14" t="s">
+        <v>242</v>
+      </c>
+      <c r="K47" s="1">
+        <v>2007</v>
+      </c>
+      <c r="L47" s="1" t="s">
+        <v>362</v>
+      </c>
+      <c r="M47" s="1" t="s">
+        <v>243</v>
+      </c>
+    </row>
+    <row r="48" spans="1:13" ht="16.8" x14ac:dyDescent="0.3">
+      <c r="A48" s="1" t="s">
+        <v>364</v>
+      </c>
+      <c r="B48" s="6" t="s">
+        <v>365</v>
+      </c>
+      <c r="C48" s="6" t="s">
+        <v>370</v>
+      </c>
+      <c r="D48" s="4" t="s">
+        <v>366</v>
+      </c>
+      <c r="E48" t="s">
+        <v>363</v>
+      </c>
+      <c r="F48" s="1" t="s">
+        <v>49</v>
+      </c>
+      <c r="G48" t="s">
+        <v>367</v>
+      </c>
+      <c r="H48" s="11" t="s">
+        <v>368</v>
+      </c>
+      <c r="I48" s="4" t="s">
+        <v>369</v>
+      </c>
+      <c r="J48" s="14" t="s">
+        <v>242</v>
+      </c>
+      <c r="K48" s="1">
+        <v>2016</v>
+      </c>
+      <c r="L48" s="1" t="s">
+        <v>312</v>
+      </c>
+      <c r="M48" s="1" t="s">
+        <v>243</v>
+      </c>
+    </row>
+    <row r="49" spans="1:13" ht="16.8" x14ac:dyDescent="0.3">
+      <c r="A49" s="1" t="s">
+        <v>371</v>
+      </c>
+      <c r="B49" s="1" t="s">
+        <v>257</v>
+      </c>
+      <c r="C49" s="6" t="s">
+        <v>375</v>
+      </c>
+      <c r="D49" s="4" t="s">
+        <v>373</v>
+      </c>
+      <c r="E49" t="s">
+        <v>374</v>
+      </c>
+      <c r="F49" s="1" t="s">
+        <v>49</v>
+      </c>
+      <c r="G49" t="s">
+        <v>372</v>
+      </c>
+      <c r="H49" s="4" t="s">
+        <v>377</v>
+      </c>
+      <c r="I49" s="4" t="s">
+        <v>376</v>
+      </c>
+      <c r="J49" s="14" t="s">
+        <v>242</v>
+      </c>
+      <c r="L49" s="1" t="s">
+        <v>362</v>
+      </c>
+      <c r="M49" s="1" t="s">
+        <v>243</v>
+      </c>
+    </row>
+    <row r="50" spans="1:13" ht="16.8" x14ac:dyDescent="0.3">
+      <c r="A50" s="1" t="s">
+        <v>379</v>
+      </c>
+      <c r="B50" s="1" t="s">
+        <v>257</v>
+      </c>
+      <c r="C50" s="6" t="s">
+        <v>381</v>
+      </c>
+      <c r="D50" s="4" t="s">
+        <v>380</v>
+      </c>
+      <c r="E50" t="s">
+        <v>378</v>
+      </c>
+      <c r="F50" s="1" t="s">
+        <v>49</v>
+      </c>
+      <c r="G50" t="s">
+        <v>384</v>
+      </c>
+      <c r="H50" s="4" t="s">
+        <v>383</v>
+      </c>
+      <c r="I50" s="4" t="s">
+        <v>382</v>
+      </c>
+      <c r="J50" s="14" t="s">
+        <v>242</v>
+      </c>
+      <c r="K50" s="1">
+        <v>2016</v>
+      </c>
+      <c r="L50" s="1" t="s">
+        <v>244</v>
+      </c>
+      <c r="M50" s="1" t="s">
+        <v>243</v>
+      </c>
+    </row>
+    <row r="51" spans="1:13" ht="16.8" x14ac:dyDescent="0.3">
+      <c r="A51" s="1" t="s">
+        <v>386</v>
+      </c>
+      <c r="B51" s="1" t="s">
+        <v>257</v>
+      </c>
+      <c r="C51" s="6" t="s">
+        <v>388</v>
+      </c>
+      <c r="D51" s="4" t="s">
+        <v>387</v>
+      </c>
+      <c r="E51" t="s">
+        <v>385</v>
+      </c>
+      <c r="F51" s="1" t="s">
+        <v>49</v>
+      </c>
+      <c r="G51" t="s">
+        <v>389</v>
+      </c>
+      <c r="H51" s="4" t="s">
+        <v>390</v>
+      </c>
+      <c r="I51" s="4" t="s">
+        <v>391</v>
+      </c>
+      <c r="J51" s="14" t="s">
+        <v>273</v>
+      </c>
+      <c r="K51" s="1">
+        <v>2019</v>
+      </c>
+      <c r="L51" s="1" t="s">
+        <v>51</v>
+      </c>
+      <c r="M51" s="1" t="s">
         <v>243</v>
       </c>
     </row>
@@ -2855,6 +3796,46 @@
     <hyperlink ref="H35" r:id="rId87" display="tel:+966539182585" xr:uid="{62810195-C7B8-4AFE-9C50-323A5BC98036}"/>
     <hyperlink ref="D36" r:id="rId88" display="https://www.linkedin.com/in/jawaher-al-jneibi-535a16216/" xr:uid="{7C0EA381-C75D-481A-8FCA-C46402431C34}"/>
     <hyperlink ref="I36" r:id="rId89" xr:uid="{F3E9733A-E5A8-4F6A-A96C-562C92D3D820}"/>
+    <hyperlink ref="D37" r:id="rId90" display="https://www.linkedin.com/in/riddhi-parekh-612907329/" xr:uid="{47CE4792-6485-4D6E-90B9-C397D0803946}"/>
+    <hyperlink ref="I37" r:id="rId91" display="https://www.elitehrconsultancy.com/" xr:uid="{6461BF70-84BB-4BFC-BE10-2BDF148499A5}"/>
+    <hyperlink ref="D38" r:id="rId92" display="https://www.linkedin.com/in/sam-mazzotta/" xr:uid="{2360BAA8-518D-4328-8F90-FD05A9236727}"/>
+    <hyperlink ref="D39" r:id="rId93" display="https://www.linkedin.com/in/ceni-venugopalan-40408690/" xr:uid="{0FF628D8-E925-41C9-AF72-28E45C02F58F}"/>
+    <hyperlink ref="A39" r:id="rId94" display="https://www.linkedin.com/in/ceni-venugopalan-40408690/" xr:uid="{10039B58-FBAB-4899-B45A-65E8095701BE}"/>
+    <hyperlink ref="I39" r:id="rId95" xr:uid="{2B975F24-0248-4E6B-A6B6-BBF636EB10A0}"/>
+    <hyperlink ref="D40" r:id="rId96" display="https://www.linkedin.com/in/bharat-f-0b9b3145/" xr:uid="{AE62925B-9FEF-420F-ADD8-BD519E7A4A41}"/>
+    <hyperlink ref="I40" r:id="rId97" display="http://www.elkho-group.com/" xr:uid="{308A3A0E-03D3-4C84-AFBE-2FE4591599FB}"/>
+    <hyperlink ref="D41" r:id="rId98" display="https://www.linkedin.com/in/yeshma-fernandes/" xr:uid="{98A51B9B-4E83-4E36-9A6E-7B1E80AE4B08}"/>
+    <hyperlink ref="I41" r:id="rId99" xr:uid="{67134D0F-06D9-44C5-A744-3F075902E5D4}"/>
+    <hyperlink ref="D42" r:id="rId100" display="https://www.linkedin.com/in/yasmin-mckeon/" xr:uid="{C09AAA2E-2D1D-4465-ABDB-CE4C6465ED06}"/>
+    <hyperlink ref="I42" r:id="rId101" display="https://www.collins-search.com/" xr:uid="{ACE06A3B-62F2-4360-BD99-0092D704F499}"/>
+    <hyperlink ref="D43" r:id="rId102" display="https://www.linkedin.com/in/giby-george-404b388/" xr:uid="{7BDBF524-EAD9-4811-A1BF-109236848390}"/>
+    <hyperlink ref="I43" r:id="rId103" xr:uid="{DADA0788-937C-414F-B1F7-E8991FC8A1FE}"/>
+    <hyperlink ref="H43" r:id="rId104" display="tel:00971585850831" xr:uid="{8AB1710D-5FC6-4853-98D8-789B11657428}"/>
+    <hyperlink ref="D44" r:id="rId105" display="https://www.linkedin.com/in/jasmine-sagai-831ab5105/" xr:uid="{49385D95-A015-497C-BBD7-2DD196A9645F}"/>
+    <hyperlink ref="I44" r:id="rId106" display="http://www.davidsondubai.net/" xr:uid="{A1274F9D-EB09-43DD-9941-DBF78275C196}"/>
+    <hyperlink ref="H44" r:id="rId107" display="tel:043555961" xr:uid="{E4E91E96-FC0C-4972-A0B4-BD2E458B8D1F}"/>
+    <hyperlink ref="I45" r:id="rId108" xr:uid="{EC35330C-DE5C-49D1-AB26-8D751110C156}"/>
+    <hyperlink ref="H45" r:id="rId109" display="tel:+44 (0)20 3926 7603" xr:uid="{A7DDB436-ED69-4536-8BF4-941B7D7468EB}"/>
+    <hyperlink ref="D45" r:id="rId110" display="https://www.linkedin.com/in/daniela-madden-04851427b/" xr:uid="{B4F621AF-390E-47C9-AD5F-813651AFBA58}"/>
+    <hyperlink ref="D46" r:id="rId111" display="https://www.linkedin.com/in/rajiv-d-d-52908117a/" xr:uid="{BC5567D8-13F4-49E2-BA68-DD5FEFD17F3E}"/>
+    <hyperlink ref="I46" r:id="rId112" display="http://www.davidsondubai.net/" xr:uid="{6169CE20-AE5D-4BB8-A71D-003BB7773C91}"/>
+    <hyperlink ref="H46" r:id="rId113" display="tel:043555961" xr:uid="{9DE80C9C-6AD9-4C3E-BA13-68E3A2C25E46}"/>
+    <hyperlink ref="A47" r:id="rId114" display="https://www.linkedin.com/in/asmaa-sad-941023196/" xr:uid="{82B3E83E-A86D-4E13-8B6D-D75B645A3102}"/>
+    <hyperlink ref="D47" r:id="rId115" display="https://www.linkedin.com/in/masoodamkhan/" xr:uid="{AC1766F3-9C98-41E9-8646-283D608F6BB2}"/>
+    <hyperlink ref="I47" r:id="rId116" xr:uid="{DD509087-6DEE-4B3F-85AA-F84CD6E39D91}"/>
+    <hyperlink ref="D48" r:id="rId117" display="https://www.linkedin.com/in/sindujav/" xr:uid="{68ED95F2-A4FD-4BD2-B35D-E47C27F6A84B}"/>
+    <hyperlink ref="I48" r:id="rId118" display="https://www.business-umbrella.com/" xr:uid="{1C361BD6-FC4D-4880-B2CC-72721E3DB86A}"/>
+    <hyperlink ref="A49" r:id="rId119" display="https://www.linkedin.com/in/turki-al-otaibi-95b5a9244/" xr:uid="{1D14A056-F79C-42A7-808F-E741DE7017DF}"/>
+    <hyperlink ref="D49" r:id="rId120" display="https://www.linkedin.com/in/turki-al-otaibi-95b5a9244/" xr:uid="{E6AD25CA-2886-47AD-AD7C-9E798C8A4BD4}"/>
+    <hyperlink ref="I49" r:id="rId121" xr:uid="{00EDE74A-8C6A-4840-B7A1-DD8DB9355A6F}"/>
+    <hyperlink ref="H49" r:id="rId122" display="tel:+966 13 8493777" xr:uid="{685BE368-BBD1-4838-A11E-6EEACAF1E7E2}"/>
+    <hyperlink ref="D50" r:id="rId123" display="https://www.linkedin.com/in/m-nadeem-amjad-5664098a/" xr:uid="{BEF22B56-5399-4574-A1F7-C4E957358F3E}"/>
+    <hyperlink ref="I50" r:id="rId124" display="http://www.rfsonshr.com/" xr:uid="{B13F1D29-D5A3-4233-B672-333871A2E48D}"/>
+    <hyperlink ref="H50" r:id="rId125" display="tel:971 50 434 4675" xr:uid="{C997CCFF-69A0-4521-B026-CB0D11B7251F}"/>
+    <hyperlink ref="A51" r:id="rId126" display="https://www.linkedin.com/in/stivan-quadros-ksa/" xr:uid="{FADA9964-DB09-45D3-93BD-FA395C99183F}"/>
+    <hyperlink ref="D51" r:id="rId127" display="https://www.linkedin.com/in/stivan-quadros-ksa/" xr:uid="{FC7EF43B-25D7-46B4-89E4-AB03AFF16612}"/>
+    <hyperlink ref="H51" r:id="rId128" display="tel:+966 92 002 9279" xr:uid="{FE02768F-59E0-47FF-A628-A21E5277C800}"/>
+    <hyperlink ref="I51" r:id="rId129" xr:uid="{01106064-EC7F-4724-9969-36C95B08DB90}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Add day 27 progress
</commit_message>
<xml_diff>
--- a/Defining ICP/Defined Leads.xlsx
+++ b/Defining ICP/Defined Leads.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\R E E M\Documents\EVA Ops Training\Defining ICP\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0C56EBC8-A8FD-4887-A83F-F7F4D9A06188}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9B69AEC7-3AB6-408F-9365-768C662E8156}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{DAB7335F-B748-4A40-8146-0BCBFC1873B2}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="564" uniqueCount="392">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="675" uniqueCount="462">
   <si>
     <t>Name</t>
   </si>
@@ -1214,6 +1214,216 @@
   </si>
   <si>
     <t>https://tadbeerco.com/</t>
+  </si>
+  <si>
+    <t>ismael@rawafed.ae</t>
+  </si>
+  <si>
+    <t>linkedin.com/in/jay-mar-ismael-phri-chrm-chrp-uk-22384128</t>
+  </si>
+  <si>
+    <t>Jay-Mar Ismael</t>
+  </si>
+  <si>
+    <t>Head of Recruitment</t>
+  </si>
+  <si>
+    <t>Rawafed Recruitment</t>
+  </si>
+  <si>
+    <t>http://rawafed.ae/</t>
+  </si>
+  <si>
+    <t>Recruitment leader managing talent acquisition, executive search, and recruitment workflows for staffing and hiring operations.</t>
+  </si>
+  <si>
+    <t>Saif Msc</t>
+  </si>
+  <si>
+    <t>saif@resmodtec.com</t>
+  </si>
+  <si>
+    <t>ResModTec</t>
+  </si>
+  <si>
+    <t>Recruitment leader managing talent acquisition, workforce strategy, and end-to-end hiring operations within recruitment and consulting services.</t>
+  </si>
+  <si>
+    <t>http://www.resmodtec.com</t>
+  </si>
+  <si>
+    <t>https://www.linkedin.com/in/saif-abdali-150a3b4a/</t>
+  </si>
+  <si>
+    <t>+971 2 667 4666</t>
+  </si>
+  <si>
+    <t>Shalu Roshni</t>
+  </si>
+  <si>
+    <t>Fast HR Solutions</t>
+  </si>
+  <si>
+    <t>Shalu Roshni | LinkedIn</t>
+  </si>
+  <si>
+    <t>Manages recruitment operations, talent acquisition, and hiring workflows for staffing and HR solutions services.</t>
+  </si>
+  <si>
+    <t>sroshni@cisco.com</t>
+  </si>
+  <si>
+    <t>(4) Fast HR Solutions: Overview | LinkedIn</t>
+  </si>
+  <si>
+    <t>Yohannes Getachew</t>
+  </si>
+  <si>
+    <t>Veretin Recruitment</t>
+  </si>
+  <si>
+    <t>Yohannes Getachew | LinkedIn</t>
+  </si>
+  <si>
+    <t>Head of Recruitment managing technical talent acquisition, candidate sourcing, and end-to-end recruitment workflows for Web3 and AI hiring operations.</t>
+  </si>
+  <si>
+    <t>+62 823 4180442</t>
+  </si>
+  <si>
+    <t>veretin.com/recruitment</t>
+  </si>
+  <si>
+    <t>yohannes@veretin.com</t>
+  </si>
+  <si>
+    <t>Veena Lalwani</t>
+  </si>
+  <si>
+    <t>ADIV Human Resources Consultancies LLC</t>
+  </si>
+  <si>
+    <t>Veena Lalwani | LinkedIn</t>
+  </si>
+  <si>
+    <t>Recruitment leader specializing in executive search, talent acquisition, headhunting, and recruitment operations for consulting and technology sectors.</t>
+  </si>
+  <si>
+    <t>veena@adivhr.com</t>
+  </si>
+  <si>
+    <t>+971 55 136 2753</t>
+  </si>
+  <si>
+    <t>http://www.adivhr.com</t>
+  </si>
+  <si>
+    <t>Talent Tap MENA</t>
+  </si>
+  <si>
+    <t>Daniel Soares</t>
+  </si>
+  <si>
+    <t>Daniel Soares | LinkedIn</t>
+  </si>
+  <si>
+    <t>Founder and recruitment leader managing executive search, talent acquisition, headhunting, and recruitment workflows across multiple industries in the MENA region.</t>
+  </si>
+  <si>
+    <t>www.talenttapmena.com</t>
+  </si>
+  <si>
+    <t>daniel@talenttapmena.com</t>
+  </si>
+  <si>
+    <t>Sirine Dahmen</t>
+  </si>
+  <si>
+    <t>Palm Springs Co.</t>
+  </si>
+  <si>
+    <t>Sirine Dahmen | LinkedIn</t>
+  </si>
+  <si>
+    <t>Recruitment professional specializing in executive search, headhunting, candidate sourcing, and recruitment workflows across multiple industries.</t>
+  </si>
+  <si>
+    <t>sirine@palmspringsarabia.com</t>
+  </si>
+  <si>
+    <t>+966 11 288 6575</t>
+  </si>
+  <si>
+    <t>http://www.palmspringsarabia.com</t>
+  </si>
+  <si>
+    <t>Gayathry Gireesh</t>
+  </si>
+  <si>
+    <t>Gayathry Gireesh (Nair) | LinkedIn</t>
+  </si>
+  <si>
+    <t>We Search</t>
+  </si>
+  <si>
+    <t>Recruitment leader specializing in talent acquisition, executive search, recruitment database management, and end-to-end hiring operations.</t>
+  </si>
+  <si>
+    <t>gayathry@wesearchinc.com</t>
+  </si>
+  <si>
+    <t>http://www.wesearchinc.com</t>
+  </si>
+  <si>
+    <t>Human Resources Services</t>
+  </si>
+  <si>
+    <t>200+</t>
+  </si>
+  <si>
+    <t>Shrawan Wosti</t>
+  </si>
+  <si>
+    <t>Managing Director</t>
+  </si>
+  <si>
+    <t>Aspire Global Human Resources</t>
+  </si>
+  <si>
+    <t>Shrawan Wosti | LinkedIn</t>
+  </si>
+  <si>
+    <t>Leads recruitment, talent acquisition, and HR consulting operations for hospitality and workforce solutions.</t>
+  </si>
+  <si>
+    <t>md@aspireglobal-hr.com</t>
+  </si>
+  <si>
+    <t>+971 56 509 8988</t>
+  </si>
+  <si>
+    <t>Hospitality</t>
+  </si>
+  <si>
+    <t>Lamya Aldossary</t>
+  </si>
+  <si>
+    <t>Human Resources Manager</t>
+  </si>
+  <si>
+    <t>NES Fircroft</t>
+  </si>
+  <si>
+    <t>Lamya Aldossary | LinkedIn</t>
+  </si>
+  <si>
+    <t>Handles recruitment, HR operations, and workforce management workflows for technical and engineering staffing.</t>
+  </si>
+  <si>
+    <t>lamya.aldossary@nesfircroft.com</t>
+  </si>
+  <si>
+    <t>https://www.nesfircroft.com/</t>
   </si>
 </sst>
 </file>
@@ -1666,14 +1876,14 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3B2D820C-3568-45BE-99C1-F7479358E85B}">
-  <dimension ref="A1:M51"/>
+  <dimension ref="A1:M61"/>
   <sheetFormatPr defaultRowHeight="15.6" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="21.88671875" style="2" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="35.88671875" style="1" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="47.6640625" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="67.77734375" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="110.88671875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="141.33203125" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="12.77734375" style="1" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="46.5546875" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="18.44140625" style="11" bestFit="1" customWidth="1"/>
@@ -3701,6 +3911,389 @@
         <v>51</v>
       </c>
       <c r="M51" s="1" t="s">
+        <v>243</v>
+      </c>
+    </row>
+    <row r="52" spans="1:13" ht="16.8" x14ac:dyDescent="0.3">
+      <c r="A52" s="1" t="s">
+        <v>394</v>
+      </c>
+      <c r="B52" s="1" t="s">
+        <v>395</v>
+      </c>
+      <c r="C52" s="6" t="s">
+        <v>396</v>
+      </c>
+      <c r="D52" s="4" t="s">
+        <v>393</v>
+      </c>
+      <c r="E52" t="s">
+        <v>398</v>
+      </c>
+      <c r="F52" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="G52" t="s">
+        <v>392</v>
+      </c>
+      <c r="I52" s="4" t="s">
+        <v>397</v>
+      </c>
+      <c r="J52" s="1" t="s">
+        <v>242</v>
+      </c>
+      <c r="L52" s="1" t="s">
+        <v>312</v>
+      </c>
+      <c r="M52" s="1" t="s">
+        <v>243</v>
+      </c>
+    </row>
+    <row r="53" spans="1:13" ht="16.8" x14ac:dyDescent="0.3">
+      <c r="A53" s="1" t="s">
+        <v>399</v>
+      </c>
+      <c r="B53" s="1" t="s">
+        <v>395</v>
+      </c>
+      <c r="C53" s="6" t="s">
+        <v>401</v>
+      </c>
+      <c r="D53" s="4" t="s">
+        <v>404</v>
+      </c>
+      <c r="E53" t="s">
+        <v>402</v>
+      </c>
+      <c r="F53" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="G53" t="s">
+        <v>400</v>
+      </c>
+      <c r="H53" s="11" t="s">
+        <v>405</v>
+      </c>
+      <c r="I53" s="4" t="s">
+        <v>403</v>
+      </c>
+      <c r="J53" s="1" t="s">
+        <v>242</v>
+      </c>
+      <c r="K53" s="1">
+        <v>2002</v>
+      </c>
+      <c r="L53" s="1" t="s">
+        <v>312</v>
+      </c>
+      <c r="M53" s="1" t="s">
+        <v>243</v>
+      </c>
+    </row>
+    <row r="54" spans="1:13" ht="16.8" x14ac:dyDescent="0.3">
+      <c r="A54" s="1" t="s">
+        <v>406</v>
+      </c>
+      <c r="B54" s="1" t="s">
+        <v>395</v>
+      </c>
+      <c r="C54" s="6" t="s">
+        <v>407</v>
+      </c>
+      <c r="D54" s="4" t="s">
+        <v>408</v>
+      </c>
+      <c r="E54" t="s">
+        <v>409</v>
+      </c>
+      <c r="F54" s="1" t="s">
+        <v>79</v>
+      </c>
+      <c r="G54" t="s">
+        <v>410</v>
+      </c>
+      <c r="I54" s="4" t="s">
+        <v>411</v>
+      </c>
+      <c r="J54" s="1" t="s">
+        <v>242</v>
+      </c>
+      <c r="K54" s="1">
+        <v>2017</v>
+      </c>
+      <c r="L54" s="1" t="s">
+        <v>244</v>
+      </c>
+      <c r="M54" s="1" t="s">
+        <v>243</v>
+      </c>
+    </row>
+    <row r="55" spans="1:13" ht="16.8" x14ac:dyDescent="0.3">
+      <c r="A55" s="1" t="s">
+        <v>412</v>
+      </c>
+      <c r="B55" s="1" t="s">
+        <v>395</v>
+      </c>
+      <c r="C55" s="6" t="s">
+        <v>413</v>
+      </c>
+      <c r="D55" s="4" t="s">
+        <v>414</v>
+      </c>
+      <c r="E55" t="s">
+        <v>415</v>
+      </c>
+      <c r="F55" s="1" t="s">
+        <v>79</v>
+      </c>
+      <c r="G55" t="s">
+        <v>418</v>
+      </c>
+      <c r="H55" s="11" t="s">
+        <v>416</v>
+      </c>
+      <c r="I55" s="4" t="s">
+        <v>417</v>
+      </c>
+      <c r="J55" s="1" t="s">
+        <v>242</v>
+      </c>
+      <c r="K55" s="1">
+        <v>2024</v>
+      </c>
+      <c r="L55" s="1">
+        <v>15</v>
+      </c>
+      <c r="M55" s="1" t="s">
+        <v>243</v>
+      </c>
+    </row>
+    <row r="56" spans="1:13" ht="16.8" x14ac:dyDescent="0.3">
+      <c r="A56" s="1" t="s">
+        <v>419</v>
+      </c>
+      <c r="B56" s="1" t="s">
+        <v>395</v>
+      </c>
+      <c r="C56" s="6" t="s">
+        <v>420</v>
+      </c>
+      <c r="D56" s="4" t="s">
+        <v>421</v>
+      </c>
+      <c r="E56" t="s">
+        <v>422</v>
+      </c>
+      <c r="F56" s="1" t="s">
+        <v>79</v>
+      </c>
+      <c r="G56" t="s">
+        <v>423</v>
+      </c>
+      <c r="H56" s="11" t="s">
+        <v>424</v>
+      </c>
+      <c r="I56" s="4" t="s">
+        <v>425</v>
+      </c>
+      <c r="J56" s="1" t="s">
+        <v>242</v>
+      </c>
+      <c r="L56" s="1">
+        <v>10</v>
+      </c>
+      <c r="M56" s="1" t="s">
+        <v>243</v>
+      </c>
+    </row>
+    <row r="57" spans="1:13" ht="16.8" x14ac:dyDescent="0.3">
+      <c r="A57" s="1" t="s">
+        <v>427</v>
+      </c>
+      <c r="B57" s="1" t="s">
+        <v>395</v>
+      </c>
+      <c r="C57" s="6" t="s">
+        <v>426</v>
+      </c>
+      <c r="D57" s="4" t="s">
+        <v>428</v>
+      </c>
+      <c r="E57" t="s">
+        <v>429</v>
+      </c>
+      <c r="F57" s="1" t="s">
+        <v>79</v>
+      </c>
+      <c r="G57" t="s">
+        <v>431</v>
+      </c>
+      <c r="I57" s="4" t="s">
+        <v>430</v>
+      </c>
+      <c r="J57" s="1" t="s">
+        <v>242</v>
+      </c>
+      <c r="K57" s="1">
+        <v>2019</v>
+      </c>
+      <c r="L57" s="1">
+        <v>10</v>
+      </c>
+      <c r="M57" s="1" t="s">
+        <v>243</v>
+      </c>
+    </row>
+    <row r="58" spans="1:13" ht="16.8" x14ac:dyDescent="0.3">
+      <c r="A58" s="1" t="s">
+        <v>432</v>
+      </c>
+      <c r="B58" s="1" t="s">
+        <v>395</v>
+      </c>
+      <c r="C58" s="6" t="s">
+        <v>433</v>
+      </c>
+      <c r="D58" s="4" t="s">
+        <v>434</v>
+      </c>
+      <c r="E58" t="s">
+        <v>435</v>
+      </c>
+      <c r="F58" s="1" t="s">
+        <v>49</v>
+      </c>
+      <c r="G58" t="s">
+        <v>436</v>
+      </c>
+      <c r="H58" s="11" t="s">
+        <v>437</v>
+      </c>
+      <c r="I58" s="4" t="s">
+        <v>438</v>
+      </c>
+      <c r="J58" s="1" t="s">
+        <v>242</v>
+      </c>
+      <c r="K58" s="1">
+        <v>2005</v>
+      </c>
+      <c r="L58" s="1" t="s">
+        <v>51</v>
+      </c>
+      <c r="M58" s="1" t="s">
+        <v>243</v>
+      </c>
+    </row>
+    <row r="59" spans="1:13" ht="16.8" x14ac:dyDescent="0.3">
+      <c r="A59" s="1" t="s">
+        <v>439</v>
+      </c>
+      <c r="B59" s="1" t="s">
+        <v>395</v>
+      </c>
+      <c r="C59" s="6" t="s">
+        <v>441</v>
+      </c>
+      <c r="D59" s="4" t="s">
+        <v>440</v>
+      </c>
+      <c r="E59" t="s">
+        <v>442</v>
+      </c>
+      <c r="F59" s="1" t="s">
+        <v>79</v>
+      </c>
+      <c r="G59" t="s">
+        <v>443</v>
+      </c>
+      <c r="I59" s="4" t="s">
+        <v>444</v>
+      </c>
+      <c r="J59" s="1" t="s">
+        <v>445</v>
+      </c>
+      <c r="K59" s="1">
+        <v>2008</v>
+      </c>
+      <c r="L59" s="1" t="s">
+        <v>446</v>
+      </c>
+      <c r="M59" s="1" t="s">
+        <v>243</v>
+      </c>
+    </row>
+    <row r="60" spans="1:13" ht="16.8" x14ac:dyDescent="0.3">
+      <c r="A60" s="1" t="s">
+        <v>447</v>
+      </c>
+      <c r="B60" s="1" t="s">
+        <v>448</v>
+      </c>
+      <c r="C60" s="6" t="s">
+        <v>449</v>
+      </c>
+      <c r="D60" s="4" t="s">
+        <v>450</v>
+      </c>
+      <c r="E60" t="s">
+        <v>451</v>
+      </c>
+      <c r="F60" s="1" t="s">
+        <v>79</v>
+      </c>
+      <c r="G60" t="s">
+        <v>452</v>
+      </c>
+      <c r="H60" s="11" t="s">
+        <v>453</v>
+      </c>
+      <c r="J60" s="1" t="s">
+        <v>454</v>
+      </c>
+      <c r="K60" s="1">
+        <v>2022</v>
+      </c>
+      <c r="L60" s="1" t="s">
+        <v>446</v>
+      </c>
+      <c r="M60" s="1" t="s">
+        <v>243</v>
+      </c>
+    </row>
+    <row r="61" spans="1:13" ht="16.8" x14ac:dyDescent="0.3">
+      <c r="A61" s="1" t="s">
+        <v>455</v>
+      </c>
+      <c r="B61" s="1" t="s">
+        <v>456</v>
+      </c>
+      <c r="C61" s="6" t="s">
+        <v>457</v>
+      </c>
+      <c r="D61" s="4" t="s">
+        <v>458</v>
+      </c>
+      <c r="E61" t="s">
+        <v>459</v>
+      </c>
+      <c r="F61" s="1" t="s">
+        <v>49</v>
+      </c>
+      <c r="G61" t="s">
+        <v>460</v>
+      </c>
+      <c r="I61" s="4" t="s">
+        <v>461</v>
+      </c>
+      <c r="J61" s="1" t="s">
+        <v>242</v>
+      </c>
+      <c r="L61" s="1" t="s">
+        <v>362</v>
+      </c>
+      <c r="M61" s="1" t="s">
         <v>243</v>
       </c>
     </row>
@@ -3836,6 +4429,25 @@
     <hyperlink ref="D51" r:id="rId127" display="https://www.linkedin.com/in/stivan-quadros-ksa/" xr:uid="{FC7EF43B-25D7-46B4-89E4-AB03AFF16612}"/>
     <hyperlink ref="H51" r:id="rId128" display="tel:+966 92 002 9279" xr:uid="{FE02768F-59E0-47FF-A628-A21E5277C800}"/>
     <hyperlink ref="I51" r:id="rId129" xr:uid="{01106064-EC7F-4724-9969-36C95B08DB90}"/>
+    <hyperlink ref="D52" r:id="rId130" display="https://www.linkedin.com/in/jay-mar-ismael-phri-chrm-chrp-uk-22384128/" xr:uid="{AFA10F6A-E0D1-45FD-A3EA-DDA698E33B81}"/>
+    <hyperlink ref="I52" r:id="rId131" xr:uid="{349B6D69-FD00-45B9-9979-979FB1A4379D}"/>
+    <hyperlink ref="I53" r:id="rId132" display="http://www.resmodtec.com/" xr:uid="{CF25AB71-BD87-4FFA-8E10-0CD30D2D2703}"/>
+    <hyperlink ref="D53" r:id="rId133" xr:uid="{7B3FB104-E758-4454-8F06-FD0494F701ED}"/>
+    <hyperlink ref="D54" r:id="rId134" display="https://www.linkedin.com/in/shalu-roshni-9b4478233/" xr:uid="{EB117998-BD17-439B-BFA4-23387F171CAB}"/>
+    <hyperlink ref="I54" r:id="rId135" display="https://www.linkedin.com/company/fasthrsolutions/" xr:uid="{FEA35606-3869-450A-9A77-EFBF084081D7}"/>
+    <hyperlink ref="D55" r:id="rId136" display="https://www.linkedin.com/in/yohannes-getachew-667a1b241/" xr:uid="{C1B72A1E-03B2-4C6A-8AD5-5D1B02E95FC1}"/>
+    <hyperlink ref="I55" r:id="rId137" display="https://veretin.com/recruitment" xr:uid="{998BAE98-B7F4-4152-A11A-2CF8D0C93303}"/>
+    <hyperlink ref="D56" r:id="rId138" display="https://www.linkedin.com/in/veenalalwani/" xr:uid="{8EDAED5F-A529-4B72-8A9F-098871973FF3}"/>
+    <hyperlink ref="I56" r:id="rId139" display="http://www.adivhr.com/" xr:uid="{ECDC9D3B-02A1-471C-9CF1-1D63D8598BE5}"/>
+    <hyperlink ref="D57" r:id="rId140" display="https://www.linkedin.com/in/danielsoares1/" xr:uid="{8BC89E79-37B5-4FBB-A41C-6187DFDB8AD5}"/>
+    <hyperlink ref="I57" r:id="rId141" display="https://www.talenttapmena.com/" xr:uid="{054C6189-EC52-4215-842E-255FDC15151E}"/>
+    <hyperlink ref="D58" r:id="rId142" display="https://www.linkedin.com/in/sirine-dahmen-ab331453/" xr:uid="{71C6F447-842A-4571-962A-88ECD1AC620D}"/>
+    <hyperlink ref="I58" r:id="rId143" display="http://www.palmspringsarabia.com/" xr:uid="{5C3CAFA0-ADE4-438E-8E38-9FCE9E71671E}"/>
+    <hyperlink ref="D59" r:id="rId144" display="https://www.linkedin.com/in/gayathry-gireesh-nair-b7175369/" xr:uid="{14058160-36A5-4CD5-B3A8-16B7E3330C81}"/>
+    <hyperlink ref="I59" r:id="rId145" display="http://www.wesearchinc.com/" xr:uid="{5C2DA1DD-5B4F-44F1-9006-4F0EC9CF7707}"/>
+    <hyperlink ref="D60" r:id="rId146" display="https://www.linkedin.com/in/shrawanwosti/" xr:uid="{21B41A97-B92E-405F-A312-DE8A093123E8}"/>
+    <hyperlink ref="D61" r:id="rId147" display="https://www.linkedin.com/in/lamya-aldossary-623190187/" xr:uid="{BF3B5748-10F8-4363-A1DA-353246EB81FE}"/>
+    <hyperlink ref="I61" r:id="rId148" xr:uid="{917910E4-A41B-4F77-B435-8358E4E69A0F}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Add day 28 progress
</commit_message>
<xml_diff>
--- a/Defining ICP/Defined Leads.xlsx
+++ b/Defining ICP/Defined Leads.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\R E E M\Documents\EVA Ops Training\Defining ICP\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9B69AEC7-3AB6-408F-9365-768C662E8156}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BF70B4B6-4267-49DD-AEB2-7F220B7CB9A0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{DAB7335F-B748-4A40-8146-0BCBFC1873B2}"/>
+    <workbookView xWindow="1152" yWindow="1284" windowWidth="17280" windowHeight="9960" xr2:uid="{DAB7335F-B748-4A40-8146-0BCBFC1873B2}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="675" uniqueCount="462">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="790" uniqueCount="532">
   <si>
     <t>Name</t>
   </si>
@@ -1424,6 +1424,216 @@
   </si>
   <si>
     <t>https://www.nesfircroft.com/</t>
+  </si>
+  <si>
+    <t>Mohammed Kafaween</t>
+  </si>
+  <si>
+    <t>Recriutment Manager</t>
+  </si>
+  <si>
+    <t>mohammed A kafaween | LinkedIn</t>
+  </si>
+  <si>
+    <t>TKAFU HR and Recruitment co.</t>
+  </si>
+  <si>
+    <t>Manages recruitment, staffing, candidate sourcing, and end-to-end hiring workflows within a recruitment agency.</t>
+  </si>
+  <si>
+    <t>Lebanon</t>
+  </si>
+  <si>
+    <t>mohammadk@tkafu.com</t>
+  </si>
+  <si>
+    <t>+962 6 437 9971</t>
+  </si>
+  <si>
+    <t>50+</t>
+  </si>
+  <si>
+    <t>Amr Abdelkarim</t>
+  </si>
+  <si>
+    <t>Black Pearl Consult</t>
+  </si>
+  <si>
+    <t>Amr AbdElKarim | LinkedIn</t>
+  </si>
+  <si>
+    <t>HR and recruitment leader managing talent acquisition, staffing, candidate sourcing, and end-to-end hiring workflows across recruitment and consulting services.</t>
+  </si>
+  <si>
+    <t>amr@blackpearlconsult.com</t>
+  </si>
+  <si>
+    <t>+971 2 622 5503</t>
+  </si>
+  <si>
+    <t>http://blackpearlconsult.com/</t>
+  </si>
+  <si>
+    <t>Upasana Arora</t>
+  </si>
+  <si>
+    <t>Upasana Arora | LinkedIn</t>
+  </si>
+  <si>
+    <t>Vision Staffing Solutions</t>
+  </si>
+  <si>
+    <t>Recruitment leader managing talent sourcing, client relations, staffing operations, and end-to-end hiring workflows within recruitment and staffing services.</t>
+  </si>
+  <si>
+    <t>upasana.arora@vssjobs.in</t>
+  </si>
+  <si>
+    <t>http://vssjobs.in/</t>
+  </si>
+  <si>
+    <t>20+</t>
+  </si>
+  <si>
+    <t>Nisha Mangalam</t>
+  </si>
+  <si>
+    <t>Nisha D.M. Deni Dennis Mangalam | LinkedIn</t>
+  </si>
+  <si>
+    <t>Terrafirma Solutions &amp; Fixit Manpower Supply</t>
+  </si>
+  <si>
+    <t>Recruitment manager specializing in talent acquisition, headhunting, candidate sourcing, and end-to-end recruitment workflows across GCC hiring operations.</t>
+  </si>
+  <si>
+    <t>https://terrafirmasolutions.ae</t>
+  </si>
+  <si>
+    <t>+971 4 548 1336</t>
+  </si>
+  <si>
+    <t>nisha@terrafirmasolutions.ae</t>
+  </si>
+  <si>
+    <t>Rita Najem</t>
+  </si>
+  <si>
+    <t>Vacancy Insider</t>
+  </si>
+  <si>
+    <t>Rita Najem | LinkedIn</t>
+  </si>
+  <si>
+    <t>Recruitment leader specializing in executive search, talent acquisition, headhunting, candidate sourcing, and end-to-end recruitment workflows across multiple industries.</t>
+  </si>
+  <si>
+    <t>rita@vacancyinsider.com</t>
+  </si>
+  <si>
+    <t>http://www.VacancyInsider.com</t>
+  </si>
+  <si>
+    <t>Faisal Banjar</t>
+  </si>
+  <si>
+    <t>Jobskey Search &amp; Selection</t>
+  </si>
+  <si>
+    <t>Faisal Banjar (ECRE) | LinkedIn</t>
+  </si>
+  <si>
+    <t>Recruitment leader managing executive search, talent acquisition, headhunting, candidate sourcing, and recruitment workflows for staffing and hiring operations across multiple industries.</t>
+  </si>
+  <si>
+    <t>faisal@jobskeysearch.com</t>
+  </si>
+  <si>
+    <t>http://www.jobskeysearch.com</t>
+  </si>
+  <si>
+    <t>+966 50 368 9803</t>
+  </si>
+  <si>
+    <t>Aya Makki</t>
+  </si>
+  <si>
+    <t>Aya Makki | LinkedIn</t>
+  </si>
+  <si>
+    <t>Kaizen Firm </t>
+  </si>
+  <si>
+    <t>Recruitment professional specializing in talent acquisition, headhunting, candidate sourcing, HR operations, and recruitment workflows for startup and corporate hiring.</t>
+  </si>
+  <si>
+    <t>http://www.kaizen-firm.com</t>
+  </si>
+  <si>
+    <t>aya.makki@kaizen-firm.com</t>
+  </si>
+  <si>
+    <t>+971 4 579 9489</t>
+  </si>
+  <si>
+    <t>Wendy Wang</t>
+  </si>
+  <si>
+    <t>WHR Solution</t>
+  </si>
+  <si>
+    <t>Wendy Wang | LinkedIn</t>
+  </si>
+  <si>
+    <t>Recruitment leader managing executive search, talent acquisition, candidate sourcing, workforce planning, and recruitment workflows for regional hiring operations across multiple industries.</t>
+  </si>
+  <si>
+    <t>wendy.wang@whr-solution.com</t>
+  </si>
+  <si>
+    <t>http://whr-solution.com/</t>
+  </si>
+  <si>
+    <t>10+</t>
+  </si>
+  <si>
+    <t>Samah AN</t>
+  </si>
+  <si>
+    <t>Samah AN | LinkedIn</t>
+  </si>
+  <si>
+    <t>Boundless</t>
+  </si>
+  <si>
+    <t>Head of recruitment managing talent acquisition, executive search, headhunting, strategic hiring, and end-to-end recruitment workflows</t>
+  </si>
+  <si>
+    <t>http://www.boundless.hr</t>
+  </si>
+  <si>
+    <t>samah@boundless.hr</t>
+  </si>
+  <si>
+    <t>+971 55 823 2944</t>
+  </si>
+  <si>
+    <t>Dannie Mhanna</t>
+  </si>
+  <si>
+    <t>Dannie Mhanna | LinkedIn</t>
+  </si>
+  <si>
+    <t>RemotelyX</t>
+  </si>
+  <si>
+    <t>Recruitment leader responsible for talent acquisition, sourcing, headhunting, hiring strategy, and managing full-cycle recruitment processes.</t>
+  </si>
+  <si>
+    <t>http://www.remotelyx.com</t>
+  </si>
+  <si>
+    <t>dannie@remotelyx.com</t>
   </si>
 </sst>
 </file>
@@ -1876,14 +2086,14 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3B2D820C-3568-45BE-99C1-F7479358E85B}">
-  <dimension ref="A1:M61"/>
+  <dimension ref="A1:M72"/>
   <sheetFormatPr defaultRowHeight="15.6" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="21.88671875" style="2" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="35.88671875" style="1" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="47.6640625" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="67.77734375" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="141.33203125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="161.109375" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="12.77734375" style="1" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="46.5546875" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="18.44140625" style="11" bestFit="1" customWidth="1"/>
@@ -4296,6 +4506,399 @@
       <c r="M61" s="1" t="s">
         <v>243</v>
       </c>
+    </row>
+    <row r="62" spans="1:13" ht="16.8" x14ac:dyDescent="0.3">
+      <c r="A62" s="1" t="s">
+        <v>462</v>
+      </c>
+      <c r="B62" s="1" t="s">
+        <v>463</v>
+      </c>
+      <c r="C62" s="6" t="s">
+        <v>465</v>
+      </c>
+      <c r="D62" s="4" t="s">
+        <v>464</v>
+      </c>
+      <c r="E62" t="s">
+        <v>466</v>
+      </c>
+      <c r="F62" s="1" t="s">
+        <v>467</v>
+      </c>
+      <c r="G62" t="s">
+        <v>468</v>
+      </c>
+      <c r="H62" s="11" t="s">
+        <v>469</v>
+      </c>
+      <c r="J62" s="1" t="s">
+        <v>242</v>
+      </c>
+      <c r="K62" s="1">
+        <v>2012</v>
+      </c>
+      <c r="L62" s="1" t="s">
+        <v>470</v>
+      </c>
+      <c r="M62" s="1" t="s">
+        <v>243</v>
+      </c>
+    </row>
+    <row r="63" spans="1:13" ht="16.8" x14ac:dyDescent="0.3">
+      <c r="A63" s="1" t="s">
+        <v>471</v>
+      </c>
+      <c r="B63" s="1" t="s">
+        <v>463</v>
+      </c>
+      <c r="C63" s="6" t="s">
+        <v>472</v>
+      </c>
+      <c r="D63" s="4" t="s">
+        <v>473</v>
+      </c>
+      <c r="E63" t="s">
+        <v>474</v>
+      </c>
+      <c r="F63" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="G63" t="s">
+        <v>475</v>
+      </c>
+      <c r="H63" s="11" t="s">
+        <v>476</v>
+      </c>
+      <c r="I63" s="4" t="s">
+        <v>477</v>
+      </c>
+      <c r="J63" s="1" t="s">
+        <v>242</v>
+      </c>
+      <c r="L63" s="1" t="s">
+        <v>470</v>
+      </c>
+      <c r="M63" s="1" t="s">
+        <v>243</v>
+      </c>
+    </row>
+    <row r="64" spans="1:13" ht="16.8" x14ac:dyDescent="0.3">
+      <c r="A64" s="1" t="s">
+        <v>478</v>
+      </c>
+      <c r="B64" s="1" t="s">
+        <v>463</v>
+      </c>
+      <c r="C64" s="6" t="s">
+        <v>480</v>
+      </c>
+      <c r="D64" s="4" t="s">
+        <v>479</v>
+      </c>
+      <c r="E64" t="s">
+        <v>481</v>
+      </c>
+      <c r="F64" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="G64" t="s">
+        <v>482</v>
+      </c>
+      <c r="I64" s="4" t="s">
+        <v>483</v>
+      </c>
+      <c r="J64" s="1" t="s">
+        <v>445</v>
+      </c>
+      <c r="K64" s="1">
+        <v>2012</v>
+      </c>
+      <c r="L64" s="1" t="s">
+        <v>484</v>
+      </c>
+      <c r="M64" s="1" t="s">
+        <v>243</v>
+      </c>
+    </row>
+    <row r="65" spans="1:13" ht="16.8" x14ac:dyDescent="0.3">
+      <c r="A65" s="1" t="s">
+        <v>485</v>
+      </c>
+      <c r="B65" s="1" t="s">
+        <v>463</v>
+      </c>
+      <c r="C65" s="6" t="s">
+        <v>487</v>
+      </c>
+      <c r="D65" s="4" t="s">
+        <v>486</v>
+      </c>
+      <c r="E65" t="s">
+        <v>488</v>
+      </c>
+      <c r="F65" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="G65" t="s">
+        <v>491</v>
+      </c>
+      <c r="H65" s="4" t="s">
+        <v>490</v>
+      </c>
+      <c r="I65" s="4" t="s">
+        <v>489</v>
+      </c>
+      <c r="J65" s="1" t="s">
+        <v>242</v>
+      </c>
+      <c r="L65" s="1" t="s">
+        <v>51</v>
+      </c>
+      <c r="M65" s="1" t="s">
+        <v>243</v>
+      </c>
+    </row>
+    <row r="66" spans="1:13" ht="16.8" x14ac:dyDescent="0.3">
+      <c r="A66" s="1" t="s">
+        <v>492</v>
+      </c>
+      <c r="B66" s="1" t="s">
+        <v>463</v>
+      </c>
+      <c r="C66" s="6" t="s">
+        <v>493</v>
+      </c>
+      <c r="D66" s="4" t="s">
+        <v>494</v>
+      </c>
+      <c r="E66" t="s">
+        <v>495</v>
+      </c>
+      <c r="F66" s="1" t="s">
+        <v>467</v>
+      </c>
+      <c r="G66" t="s">
+        <v>496</v>
+      </c>
+      <c r="I66" s="4" t="s">
+        <v>497</v>
+      </c>
+      <c r="J66" s="1" t="s">
+        <v>242</v>
+      </c>
+      <c r="K66" s="1">
+        <v>2017</v>
+      </c>
+      <c r="L66" s="1" t="s">
+        <v>484</v>
+      </c>
+      <c r="M66" s="1" t="s">
+        <v>243</v>
+      </c>
+    </row>
+    <row r="67" spans="1:13" ht="16.8" x14ac:dyDescent="0.3">
+      <c r="A67" s="1" t="s">
+        <v>498</v>
+      </c>
+      <c r="B67" s="1" t="s">
+        <v>463</v>
+      </c>
+      <c r="C67" s="6" t="s">
+        <v>499</v>
+      </c>
+      <c r="D67" s="4" t="s">
+        <v>500</v>
+      </c>
+      <c r="E67" t="s">
+        <v>501</v>
+      </c>
+      <c r="F67" s="1" t="s">
+        <v>49</v>
+      </c>
+      <c r="G67" t="s">
+        <v>502</v>
+      </c>
+      <c r="H67" s="11" t="s">
+        <v>504</v>
+      </c>
+      <c r="I67" s="4" t="s">
+        <v>503</v>
+      </c>
+      <c r="J67" s="1" t="s">
+        <v>242</v>
+      </c>
+      <c r="K67" s="1">
+        <v>2006</v>
+      </c>
+      <c r="L67" s="1" t="s">
+        <v>470</v>
+      </c>
+      <c r="M67" s="1" t="s">
+        <v>243</v>
+      </c>
+    </row>
+    <row r="68" spans="1:13" ht="16.8" x14ac:dyDescent="0.3">
+      <c r="A68" s="1" t="s">
+        <v>505</v>
+      </c>
+      <c r="B68" s="1" t="s">
+        <v>463</v>
+      </c>
+      <c r="C68" s="6" t="s">
+        <v>507</v>
+      </c>
+      <c r="D68" s="4" t="s">
+        <v>506</v>
+      </c>
+      <c r="E68" t="s">
+        <v>508</v>
+      </c>
+      <c r="F68" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="G68" t="s">
+        <v>510</v>
+      </c>
+      <c r="H68" s="4" t="s">
+        <v>511</v>
+      </c>
+      <c r="I68" s="4" t="s">
+        <v>509</v>
+      </c>
+      <c r="J68" s="1" t="s">
+        <v>242</v>
+      </c>
+      <c r="K68" s="1">
+        <v>2011</v>
+      </c>
+      <c r="L68" s="1" t="s">
+        <v>470</v>
+      </c>
+      <c r="M68" s="1" t="s">
+        <v>243</v>
+      </c>
+    </row>
+    <row r="69" spans="1:13" ht="16.8" x14ac:dyDescent="0.3">
+      <c r="A69" s="1" t="s">
+        <v>512</v>
+      </c>
+      <c r="B69" s="1" t="s">
+        <v>463</v>
+      </c>
+      <c r="C69" s="6" t="s">
+        <v>513</v>
+      </c>
+      <c r="D69" s="4" t="s">
+        <v>514</v>
+      </c>
+      <c r="E69" t="s">
+        <v>515</v>
+      </c>
+      <c r="F69" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="G69" t="s">
+        <v>516</v>
+      </c>
+      <c r="I69" s="4" t="s">
+        <v>517</v>
+      </c>
+      <c r="J69" s="1" t="s">
+        <v>242</v>
+      </c>
+      <c r="K69" s="1">
+        <v>2015</v>
+      </c>
+      <c r="L69" s="1" t="s">
+        <v>518</v>
+      </c>
+      <c r="M69" s="1" t="s">
+        <v>243</v>
+      </c>
+    </row>
+    <row r="70" spans="1:13" ht="16.8" x14ac:dyDescent="0.3">
+      <c r="A70" s="1" t="s">
+        <v>519</v>
+      </c>
+      <c r="B70" s="1" t="s">
+        <v>395</v>
+      </c>
+      <c r="C70" s="6" t="s">
+        <v>521</v>
+      </c>
+      <c r="D70" s="4" t="s">
+        <v>520</v>
+      </c>
+      <c r="E70" t="s">
+        <v>522</v>
+      </c>
+      <c r="F70" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="G70" t="s">
+        <v>524</v>
+      </c>
+      <c r="H70" s="11" t="s">
+        <v>525</v>
+      </c>
+      <c r="I70" s="4" t="s">
+        <v>523</v>
+      </c>
+      <c r="J70" s="1" t="s">
+        <v>242</v>
+      </c>
+      <c r="K70" s="1">
+        <v>2012</v>
+      </c>
+      <c r="L70" s="1" t="s">
+        <v>518</v>
+      </c>
+      <c r="M70" s="1" t="s">
+        <v>243</v>
+      </c>
+    </row>
+    <row r="71" spans="1:13" ht="16.8" x14ac:dyDescent="0.3">
+      <c r="A71" s="1" t="s">
+        <v>526</v>
+      </c>
+      <c r="B71" s="1" t="s">
+        <v>395</v>
+      </c>
+      <c r="C71" s="6" t="s">
+        <v>528</v>
+      </c>
+      <c r="D71" s="4" t="s">
+        <v>527</v>
+      </c>
+      <c r="E71" t="s">
+        <v>529</v>
+      </c>
+      <c r="F71" s="1" t="s">
+        <v>467</v>
+      </c>
+      <c r="G71" t="s">
+        <v>531</v>
+      </c>
+      <c r="I71" s="4" t="s">
+        <v>530</v>
+      </c>
+      <c r="J71" s="1" t="s">
+        <v>242</v>
+      </c>
+      <c r="K71" s="1">
+        <v>2023</v>
+      </c>
+      <c r="L71" s="1" t="s">
+        <v>470</v>
+      </c>
+      <c r="M71" s="1" t="s">
+        <v>243</v>
+      </c>
+    </row>
+    <row r="72" spans="1:13" ht="14.4" x14ac:dyDescent="0.3">
+      <c r="A72" s="1"/>
+      <c r="D72" s="4"/>
     </row>
   </sheetData>
   <phoneticPr fontId="7" type="noConversion"/>
@@ -4448,6 +5051,25 @@
     <hyperlink ref="D60" r:id="rId146" display="https://www.linkedin.com/in/shrawanwosti/" xr:uid="{21B41A97-B92E-405F-A312-DE8A093123E8}"/>
     <hyperlink ref="D61" r:id="rId147" display="https://www.linkedin.com/in/lamya-aldossary-623190187/" xr:uid="{BF3B5748-10F8-4363-A1DA-353246EB81FE}"/>
     <hyperlink ref="I61" r:id="rId148" xr:uid="{917910E4-A41B-4F77-B435-8358E4E69A0F}"/>
+    <hyperlink ref="D62" r:id="rId149" display="https://www.linkedin.com/in/mohammed-a-kafaween-6a391a87/" xr:uid="{39094149-0EB1-4555-AA75-FA8CF76BAADB}"/>
+    <hyperlink ref="D63" r:id="rId150" display="https://www.linkedin.com/in/amr-abdelkarim-76560438/" xr:uid="{0291B7CC-F26E-4B43-9BF7-EFB345DF63C9}"/>
+    <hyperlink ref="D64" r:id="rId151" display="https://www.linkedin.com/in/upasana-arora-56a494134/" xr:uid="{984FA937-D483-48F5-BC06-75AC49F744ED}"/>
+    <hyperlink ref="I64" r:id="rId152" xr:uid="{0B79FD60-8D29-479E-9C32-BF881A1F0B7E}"/>
+    <hyperlink ref="D65" r:id="rId153" display="https://www.linkedin.com/in/nishadeni/" xr:uid="{2C95EA26-D23A-4882-8B61-4074AB0AB0B2}"/>
+    <hyperlink ref="I65" r:id="rId154" display="https://terrafirmasolutions.ae/" xr:uid="{C142E67C-F6F9-4475-AFDD-11F4CBCF160B}"/>
+    <hyperlink ref="H65" r:id="rId155" display="tel:+971 4 548 1336" xr:uid="{AE09ABFC-89C1-483B-9CA7-2B027ACD6A1E}"/>
+    <hyperlink ref="D66" r:id="rId156" display="https://www.linkedin.com/in/rita-najem-73a46516/" xr:uid="{E83382C4-FE7F-4B2E-883B-C57633F10927}"/>
+    <hyperlink ref="I66" r:id="rId157" display="http://www.vacancyinsider.com/" xr:uid="{A279ACF6-5773-4A37-A295-9F095707EEBA}"/>
+    <hyperlink ref="D67" r:id="rId158" display="https://www.linkedin.com/in/fbanjar/" xr:uid="{BCF9FCA2-C441-4BA2-A3BC-91AE4D275330}"/>
+    <hyperlink ref="I67" r:id="rId159" display="http://www.jobskeysearch.com/" xr:uid="{E85F4689-6305-4F01-BF75-E98069E79E79}"/>
+    <hyperlink ref="D68" r:id="rId160" display="https://www.linkedin.com/in/aya-makki-5926a77b/" xr:uid="{4018F3EE-3294-4EF5-A797-E69B6212C16F}"/>
+    <hyperlink ref="I68" r:id="rId161" display="http://www.kaizen-firm.com/" xr:uid="{436EBCD6-CD15-41AF-A840-9316A38B2288}"/>
+    <hyperlink ref="D69" r:id="rId162" display="https://www.linkedin.com/in/wendy-wang-8457a059/" xr:uid="{B0D64574-B6F5-43A6-B40A-F769BC0B319F}"/>
+    <hyperlink ref="I69" r:id="rId163" xr:uid="{64A99209-E9B3-42B1-865D-16F5CB3FEF05}"/>
+    <hyperlink ref="D70" r:id="rId164" display="https://www.linkedin.com/in/samah-an-52990824b/" xr:uid="{9AB76211-2555-4AEE-809C-AF8D7AD57D1C}"/>
+    <hyperlink ref="I70" r:id="rId165" display="http://www.boundless.hr/" xr:uid="{BAF3FA68-CA69-4FF7-BDC9-F249194AB5C3}"/>
+    <hyperlink ref="D71" r:id="rId166" display="https://www.linkedin.com/in/dannie-mhanna/" xr:uid="{E4F90630-43BF-40DA-BD4C-698F2C85D431}"/>
+    <hyperlink ref="I71" r:id="rId167" display="http://www.remotelyx.com/" xr:uid="{0F1C3CC9-F4F2-41BB-B98A-870C9E2740F6}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Add day 29  progress
</commit_message>
<xml_diff>
--- a/Defining ICP/Defined Leads.xlsx
+++ b/Defining ICP/Defined Leads.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\R E E M\Documents\EVA Ops Training\Defining ICP\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BF70B4B6-4267-49DD-AEB2-7F220B7CB9A0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5EF6908E-9ECB-47DF-A41A-70DBB06279F9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="1152" yWindow="1284" windowWidth="17280" windowHeight="9960" xr2:uid="{DAB7335F-B748-4A40-8146-0BCBFC1873B2}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="790" uniqueCount="532">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="910" uniqueCount="610">
   <si>
     <t>Name</t>
   </si>
@@ -1634,6 +1634,240 @@
   </si>
   <si>
     <t>dannie@remotelyx.com</t>
+  </si>
+  <si>
+    <t>Albeena Shaji</t>
+  </si>
+  <si>
+    <t>HR Manager</t>
+  </si>
+  <si>
+    <t>Albeena Shaji - Assoc CIPD | LinkedIn</t>
+  </si>
+  <si>
+    <t>Descon</t>
+  </si>
+  <si>
+    <t>HR professional leading talent acquisition, workforce planning, and HR operations across engineering and construction projects.</t>
+  </si>
+  <si>
+    <t>albeena.shaji@descon.com</t>
+  </si>
+  <si>
+    <t>http://www.descon.com</t>
+  </si>
+  <si>
+    <t>+92 42 35990034</t>
+  </si>
+  <si>
+    <t>Hisham Obaid</t>
+  </si>
+  <si>
+    <t>Hisham Obaid | LinkedIn</t>
+  </si>
+  <si>
+    <t>Al-Ahlia Integrated General Trading &amp; Contracting Company</t>
+  </si>
+  <si>
+    <t>https://ahliainteg.net/?lang=ar</t>
+  </si>
+  <si>
+    <t>HR leader managing recruitment, staffing, workforce planning, and employee lifecycle operations across engineering and construction projects.</t>
+  </si>
+  <si>
+    <t>+(965)22254530</t>
+  </si>
+  <si>
+    <t>Kuwait</t>
+  </si>
+  <si>
+    <t>hisham.obaid@ahliainteg.com</t>
+  </si>
+  <si>
+    <t>1k+</t>
+  </si>
+  <si>
+    <t>Imad Hicham</t>
+  </si>
+  <si>
+    <t>Samsung C&amp;T Corporation</t>
+  </si>
+  <si>
+    <t>Imad Hicham | LinkedIn</t>
+  </si>
+  <si>
+    <t>Human Resources Manager overseeing recruitment, workforce planning, talent acquisition, employee relations, and HR operations within a large engineering and construction organization.</t>
+  </si>
+  <si>
+    <t>http://www.samsungcnt.com/</t>
+  </si>
+  <si>
+    <t>hicham.imad@samsung.com</t>
+  </si>
+  <si>
+    <t>South Korea</t>
+  </si>
+  <si>
+    <t>+82 22-145-2114</t>
+  </si>
+  <si>
+    <t>Nesrine Choumane</t>
+  </si>
+  <si>
+    <t>Ets. WAFIC IDRISS S.a.r.l.</t>
+  </si>
+  <si>
+    <t>Nesrine Choumane | LinkedIn</t>
+  </si>
+  <si>
+    <t>Human Resources Manager overseeing talent acquisition, employee relations, workforce planning, benefits administration, and HR operations within a retail and FMCG distribution organization.</t>
+  </si>
+  <si>
+    <t>n.choumane@widriss.com</t>
+  </si>
+  <si>
+    <t>http://www.widriss.com</t>
+  </si>
+  <si>
+    <t>+961 5 950 820</t>
+  </si>
+  <si>
+    <t>Manufacturing</t>
+  </si>
+  <si>
+    <t>100+</t>
+  </si>
+  <si>
+    <t>Retail</t>
+  </si>
+  <si>
+    <t>Jumana Kabli</t>
+  </si>
+  <si>
+    <t>Alesayi Holding</t>
+  </si>
+  <si>
+    <t>Jumana A. Kabli | LinkedIn</t>
+  </si>
+  <si>
+    <t>Human Resources Manager leading talent acquisition, employee relations, workforce planning, recruitment, and HR operations across a diversified retail and consumer goods organization.</t>
+  </si>
+  <si>
+    <t>j.kabli@alesayi.com</t>
+  </si>
+  <si>
+    <t>+966 12 644 8282</t>
+  </si>
+  <si>
+    <t>http://www.alesayi.com</t>
+  </si>
+  <si>
+    <t>5k+</t>
+  </si>
+  <si>
+    <t>Bandar Alhazza</t>
+  </si>
+  <si>
+    <t>Bait Al Mward Contracting Co.</t>
+  </si>
+  <si>
+    <t>bandar alhazza | LinkedIn</t>
+  </si>
+  <si>
+    <t>HR Manager responsible for recruitment, workforce planning, employee relations, and talent acquisition within a large construction and engineering company.</t>
+  </si>
+  <si>
+    <t>bandar@bmcc-ltd.com</t>
+  </si>
+  <si>
+    <t>https://www.baitalmward.com</t>
+  </si>
+  <si>
+    <t>+966 11 413 4442</t>
+  </si>
+  <si>
+    <t>Muhammad Ali Khan</t>
+  </si>
+  <si>
+    <t>Parsons Corporation</t>
+  </si>
+  <si>
+    <t>Muhammad Ali Khan | LinkedIn</t>
+  </si>
+  <si>
+    <t>Recruitment Manager responsible for hiring and workforce planning for large-scale engineering, construction, and infrastructure projects across the GCC region.</t>
+  </si>
+  <si>
+    <t>muhammad.a.khan@parsons.com</t>
+  </si>
+  <si>
+    <t>+1 703-988-8500</t>
+  </si>
+  <si>
+    <t>http://www.parsons.com</t>
+  </si>
+  <si>
+    <t>Nasser Alhamami</t>
+  </si>
+  <si>
+    <t>NEOM</t>
+  </si>
+  <si>
+    <t>Nasser Alhamami , Assoc CIPD | LinkedIn</t>
+  </si>
+  <si>
+    <t>Talent Acquisition Manager responsible for recruiting and onboarding professionals across large-scale engineering, infrastructure, construction, and development projects within NEOM.</t>
+  </si>
+  <si>
+    <t>http://NEOM.com</t>
+  </si>
+  <si>
+    <t>nasser.alhamami@neom.com</t>
+  </si>
+  <si>
+    <t>+1 303-546-7946</t>
+  </si>
+  <si>
+    <t>Faris Aloqalaa</t>
+  </si>
+  <si>
+    <t>Saudi Real Estate Infrastructure Company (BINIYAH)</t>
+  </si>
+  <si>
+    <t>Faris Aloqalaa, SHRM-ACHRM | LinkedIn</t>
+  </si>
+  <si>
+    <t>Recruitment Manager responsible for hiring talent across engineering, infrastructure, construction, and EPC projects within a large-scale Saudi infrastructure company.</t>
+  </si>
+  <si>
+    <t>faris.aloqalaa@binyah.com.sa</t>
+  </si>
+  <si>
+    <t>http://www.binyah.com.sa</t>
+  </si>
+  <si>
+    <t>+966 11 419 0728</t>
+  </si>
+  <si>
+    <t>Ryan Catani</t>
+  </si>
+  <si>
+    <t>Mace</t>
+  </si>
+  <si>
+    <t>Ryan Catani | LinkedIn</t>
+  </si>
+  <si>
+    <t>Recruitment Manager responsible for hiring engineering, construction, project management, and infrastructure talent for a global construction consultancy operating in Saudi Arabia.</t>
+  </si>
+  <si>
+    <t>ryan.catani@macegroup.com</t>
+  </si>
+  <si>
+    <t>http://www.macegroup.com</t>
+  </si>
+  <si>
+    <t>+44 20 3522 3081</t>
   </si>
 </sst>
 </file>
@@ -2086,12 +2320,12 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3B2D820C-3568-45BE-99C1-F7479358E85B}">
-  <dimension ref="A1:M72"/>
+  <dimension ref="A1:M81"/>
   <sheetFormatPr defaultRowHeight="15.6" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="21.88671875" style="2" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="35.88671875" style="1" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="47.6640625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="57.6640625" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="67.77734375" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="161.109375" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="12.77734375" style="1" bestFit="1" customWidth="1"/>
@@ -4896,9 +5130,412 @@
         <v>243</v>
       </c>
     </row>
-    <row r="72" spans="1:13" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A72" s="1"/>
-      <c r="D72" s="4"/>
+    <row r="72" spans="1:13" ht="16.8" x14ac:dyDescent="0.3">
+      <c r="A72" s="1" t="s">
+        <v>532</v>
+      </c>
+      <c r="B72" s="1" t="s">
+        <v>533</v>
+      </c>
+      <c r="C72" s="6" t="s">
+        <v>535</v>
+      </c>
+      <c r="D72" s="4" t="s">
+        <v>534</v>
+      </c>
+      <c r="E72" t="s">
+        <v>536</v>
+      </c>
+      <c r="F72" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="G72" t="s">
+        <v>537</v>
+      </c>
+      <c r="H72" s="11" t="s">
+        <v>539</v>
+      </c>
+      <c r="I72" s="4" t="s">
+        <v>538</v>
+      </c>
+      <c r="J72" s="1" t="s">
+        <v>82</v>
+      </c>
+      <c r="K72" s="1">
+        <v>1977</v>
+      </c>
+      <c r="L72" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="M72" s="1" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="73" spans="1:13" ht="16.8" x14ac:dyDescent="0.3">
+      <c r="A73" s="1" t="s">
+        <v>540</v>
+      </c>
+      <c r="B73" s="1" t="s">
+        <v>456</v>
+      </c>
+      <c r="C73" s="6" t="s">
+        <v>542</v>
+      </c>
+      <c r="D73" s="4" t="s">
+        <v>541</v>
+      </c>
+      <c r="E73" t="s">
+        <v>544</v>
+      </c>
+      <c r="F73" s="1" t="s">
+        <v>546</v>
+      </c>
+      <c r="G73" t="s">
+        <v>547</v>
+      </c>
+      <c r="H73" s="4" t="s">
+        <v>545</v>
+      </c>
+      <c r="I73" s="4" t="s">
+        <v>543</v>
+      </c>
+      <c r="J73" s="1" t="s">
+        <v>87</v>
+      </c>
+      <c r="K73" s="1">
+        <v>1977</v>
+      </c>
+      <c r="L73" s="1" t="s">
+        <v>548</v>
+      </c>
+      <c r="M73" s="1" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="74" spans="1:13" ht="16.8" x14ac:dyDescent="0.3">
+      <c r="A74" s="1" t="s">
+        <v>549</v>
+      </c>
+      <c r="B74" s="1" t="s">
+        <v>456</v>
+      </c>
+      <c r="C74" s="6" t="s">
+        <v>550</v>
+      </c>
+      <c r="D74" s="4" t="s">
+        <v>551</v>
+      </c>
+      <c r="E74" t="s">
+        <v>552</v>
+      </c>
+      <c r="F74" s="1" t="s">
+        <v>555</v>
+      </c>
+      <c r="G74" t="s">
+        <v>554</v>
+      </c>
+      <c r="H74" s="11" t="s">
+        <v>556</v>
+      </c>
+      <c r="I74" s="4" t="s">
+        <v>553</v>
+      </c>
+      <c r="J74" s="1" t="s">
+        <v>87</v>
+      </c>
+      <c r="K74" s="1">
+        <v>1938</v>
+      </c>
+      <c r="L74" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="M74" s="1" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="75" spans="1:13" ht="16.8" x14ac:dyDescent="0.3">
+      <c r="A75" s="1" t="s">
+        <v>557</v>
+      </c>
+      <c r="B75" s="1" t="s">
+        <v>456</v>
+      </c>
+      <c r="C75" s="6" t="s">
+        <v>558</v>
+      </c>
+      <c r="D75" s="4" t="s">
+        <v>559</v>
+      </c>
+      <c r="E75" t="s">
+        <v>560</v>
+      </c>
+      <c r="F75" s="1" t="s">
+        <v>467</v>
+      </c>
+      <c r="G75" t="s">
+        <v>561</v>
+      </c>
+      <c r="H75" s="11" t="s">
+        <v>563</v>
+      </c>
+      <c r="I75" s="4" t="s">
+        <v>562</v>
+      </c>
+      <c r="J75" s="1" t="s">
+        <v>564</v>
+      </c>
+      <c r="K75" s="1">
+        <v>1939</v>
+      </c>
+      <c r="L75" s="1" t="s">
+        <v>565</v>
+      </c>
+      <c r="M75" s="1" t="s">
+        <v>566</v>
+      </c>
+    </row>
+    <row r="76" spans="1:13" ht="16.8" x14ac:dyDescent="0.3">
+      <c r="A76" s="1" t="s">
+        <v>567</v>
+      </c>
+      <c r="B76" s="1" t="s">
+        <v>456</v>
+      </c>
+      <c r="C76" s="6" t="s">
+        <v>568</v>
+      </c>
+      <c r="D76" s="4" t="s">
+        <v>569</v>
+      </c>
+      <c r="E76" t="s">
+        <v>570</v>
+      </c>
+      <c r="F76" s="1" t="s">
+        <v>49</v>
+      </c>
+      <c r="G76" t="s">
+        <v>571</v>
+      </c>
+      <c r="H76" s="11" t="s">
+        <v>572</v>
+      </c>
+      <c r="I76" s="4" t="s">
+        <v>573</v>
+      </c>
+      <c r="J76" s="1" t="s">
+        <v>566</v>
+      </c>
+      <c r="K76" s="1">
+        <v>1945</v>
+      </c>
+      <c r="L76" s="1" t="s">
+        <v>574</v>
+      </c>
+      <c r="M76" s="1" t="s">
+        <v>566</v>
+      </c>
+    </row>
+    <row r="77" spans="1:13" ht="16.8" x14ac:dyDescent="0.3">
+      <c r="A77" s="1" t="s">
+        <v>575</v>
+      </c>
+      <c r="B77" s="1" t="s">
+        <v>456</v>
+      </c>
+      <c r="C77" s="6" t="s">
+        <v>576</v>
+      </c>
+      <c r="D77" s="4" t="s">
+        <v>577</v>
+      </c>
+      <c r="E77" t="s">
+        <v>578</v>
+      </c>
+      <c r="F77" s="1" t="s">
+        <v>49</v>
+      </c>
+      <c r="G77" t="s">
+        <v>579</v>
+      </c>
+      <c r="H77" s="11" t="s">
+        <v>581</v>
+      </c>
+      <c r="I77" s="4" t="s">
+        <v>580</v>
+      </c>
+      <c r="J77" s="1" t="s">
+        <v>87</v>
+      </c>
+      <c r="L77" s="1" t="s">
+        <v>470</v>
+      </c>
+      <c r="M77" s="1" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="78" spans="1:13" ht="16.8" x14ac:dyDescent="0.3">
+      <c r="A78" s="1" t="s">
+        <v>582</v>
+      </c>
+      <c r="B78" s="1" t="s">
+        <v>463</v>
+      </c>
+      <c r="C78" s="6" t="s">
+        <v>583</v>
+      </c>
+      <c r="D78" s="4" t="s">
+        <v>584</v>
+      </c>
+      <c r="E78" t="s">
+        <v>585</v>
+      </c>
+      <c r="F78" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="G78" t="s">
+        <v>586</v>
+      </c>
+      <c r="H78" s="11" t="s">
+        <v>587</v>
+      </c>
+      <c r="I78" s="4" t="s">
+        <v>588</v>
+      </c>
+      <c r="J78" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="K78" s="1">
+        <v>1944</v>
+      </c>
+      <c r="L78" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="M78" s="1" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="79" spans="1:13" ht="16.8" x14ac:dyDescent="0.3">
+      <c r="A79" s="1" t="s">
+        <v>589</v>
+      </c>
+      <c r="B79" s="1" t="s">
+        <v>463</v>
+      </c>
+      <c r="C79" s="6" t="s">
+        <v>590</v>
+      </c>
+      <c r="D79" s="4" t="s">
+        <v>591</v>
+      </c>
+      <c r="E79" t="s">
+        <v>592</v>
+      </c>
+      <c r="F79" s="1" t="s">
+        <v>49</v>
+      </c>
+      <c r="G79" t="s">
+        <v>594</v>
+      </c>
+      <c r="H79" s="11" t="s">
+        <v>595</v>
+      </c>
+      <c r="I79" s="4" t="s">
+        <v>593</v>
+      </c>
+      <c r="J79" s="1" t="s">
+        <v>87</v>
+      </c>
+      <c r="K79" s="1">
+        <v>2017</v>
+      </c>
+      <c r="L79" s="1" t="s">
+        <v>548</v>
+      </c>
+      <c r="M79" s="1" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="80" spans="1:13" ht="16.8" x14ac:dyDescent="0.3">
+      <c r="A80" s="1" t="s">
+        <v>596</v>
+      </c>
+      <c r="B80" s="1" t="s">
+        <v>463</v>
+      </c>
+      <c r="C80" s="6" t="s">
+        <v>597</v>
+      </c>
+      <c r="D80" s="4" t="s">
+        <v>598</v>
+      </c>
+      <c r="E80" t="s">
+        <v>599</v>
+      </c>
+      <c r="F80" s="1" t="s">
+        <v>49</v>
+      </c>
+      <c r="G80" t="s">
+        <v>600</v>
+      </c>
+      <c r="H80" s="11" t="s">
+        <v>602</v>
+      </c>
+      <c r="I80" s="4" t="s">
+        <v>601</v>
+      </c>
+      <c r="J80" s="1" t="s">
+        <v>87</v>
+      </c>
+      <c r="K80" s="1">
+        <v>2017</v>
+      </c>
+      <c r="L80" s="1" t="s">
+        <v>51</v>
+      </c>
+      <c r="M80" s="1" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="81" spans="1:13" ht="16.8" x14ac:dyDescent="0.3">
+      <c r="A81" s="1" t="s">
+        <v>603</v>
+      </c>
+      <c r="B81" s="1" t="s">
+        <v>463</v>
+      </c>
+      <c r="C81" s="6" t="s">
+        <v>604</v>
+      </c>
+      <c r="D81" s="4" t="s">
+        <v>605</v>
+      </c>
+      <c r="E81" t="s">
+        <v>606</v>
+      </c>
+      <c r="F81" s="1" t="s">
+        <v>49</v>
+      </c>
+      <c r="G81" t="s">
+        <v>607</v>
+      </c>
+      <c r="H81" s="11" t="s">
+        <v>609</v>
+      </c>
+      <c r="I81" s="4" t="s">
+        <v>608</v>
+      </c>
+      <c r="J81" s="1" t="s">
+        <v>87</v>
+      </c>
+      <c r="K81" s="1">
+        <v>1990</v>
+      </c>
+      <c r="L81" s="1" t="s">
+        <v>574</v>
+      </c>
+      <c r="M81" s="1" t="s">
+        <v>30</v>
+      </c>
     </row>
   </sheetData>
   <phoneticPr fontId="7" type="noConversion"/>
@@ -5070,6 +5707,27 @@
     <hyperlink ref="I70" r:id="rId165" display="http://www.boundless.hr/" xr:uid="{BAF3FA68-CA69-4FF7-BDC9-F249194AB5C3}"/>
     <hyperlink ref="D71" r:id="rId166" display="https://www.linkedin.com/in/dannie-mhanna/" xr:uid="{E4F90630-43BF-40DA-BD4C-698F2C85D431}"/>
     <hyperlink ref="I71" r:id="rId167" display="http://www.remotelyx.com/" xr:uid="{0F1C3CC9-F4F2-41BB-B98A-870C9E2740F6}"/>
+    <hyperlink ref="D72" r:id="rId168" display="https://www.linkedin.com/in/albeena/" xr:uid="{E213BE98-33F8-4686-A475-13BC62428094}"/>
+    <hyperlink ref="I72" r:id="rId169" display="http://www.descon.com/" xr:uid="{129E42EA-D2DF-4113-870B-1898D7F63B5A}"/>
+    <hyperlink ref="D73" r:id="rId170" display="https://www.linkedin.com/in/hisham-obaid-a0b80127b/" xr:uid="{733B3904-9EAA-49C0-BC7D-85B7E564959B}"/>
+    <hyperlink ref="I73" r:id="rId171" xr:uid="{E6881362-61A0-46A9-B60D-2382A1B97FD0}"/>
+    <hyperlink ref="H73" r:id="rId172" display="tel:+(965)22254530" xr:uid="{67599FB7-2E21-499A-9AF3-078F3118CAB6}"/>
+    <hyperlink ref="D74" r:id="rId173" display="https://www.linkedin.com/in/imad-hicham-b82a63330/" xr:uid="{826F1616-4AEF-4325-AADC-B53236930B15}"/>
+    <hyperlink ref="I74" r:id="rId174" xr:uid="{A64F0BB0-648B-429B-85FC-378B4D10492F}"/>
+    <hyperlink ref="D75" r:id="rId175" display="https://www.linkedin.com/in/nesrine-choumane-301978263/" xr:uid="{366A9712-9D4B-4485-B5F0-F707CF78E9D3}"/>
+    <hyperlink ref="I75" r:id="rId176" display="http://www.widriss.com/" xr:uid="{90043E00-5A55-4E62-BEB3-C238A0E1E019}"/>
+    <hyperlink ref="D76" r:id="rId177" display="https://www.linkedin.com/in/jumana-a-kabli-9aa788136/" xr:uid="{9B2877E5-57ED-4096-A44E-B8C8A62B8764}"/>
+    <hyperlink ref="I76" r:id="rId178" display="http://www.alesayi.com/" xr:uid="{1D52F418-9474-48DD-BC3B-91C149A34934}"/>
+    <hyperlink ref="D77" r:id="rId179" display="https://www.linkedin.com/in/bandar-alhazza-551a77214/" xr:uid="{C69AC3D6-BFD3-4CD7-8154-4D1E3725123F}"/>
+    <hyperlink ref="I77" r:id="rId180" display="https://www.baitalmward.com/" xr:uid="{B0C7B665-CCAB-49EC-A5DE-AE06959ABDF5}"/>
+    <hyperlink ref="D78" r:id="rId181" display="https://www.linkedin.com/in/muhammadalikhan/" xr:uid="{F7FB5122-FB98-4E5A-A767-9823B76470C7}"/>
+    <hyperlink ref="I78" r:id="rId182" display="http://www.parsons.com/" xr:uid="{FE8E8528-6491-4AD3-B86A-466E35D499CA}"/>
+    <hyperlink ref="D79" r:id="rId183" display="https://www.linkedin.com/in/nasser-alhamami-assoc-cipd-95b9b893/" xr:uid="{513EA06D-17BE-4A4D-BFF7-3D5A0E6BE73D}"/>
+    <hyperlink ref="I79" r:id="rId184" display="http://neom.com/" xr:uid="{2C3854C8-903A-4A82-90C9-7FDEC3C75B7E}"/>
+    <hyperlink ref="D80" r:id="rId185" display="https://www.linkedin.com/in/faris-aloqalaa/" xr:uid="{F00C123C-63F0-4CBF-9D3F-E208E6B5943F}"/>
+    <hyperlink ref="I80" r:id="rId186" display="http://www.binyah.com.sa/" xr:uid="{5D874C19-9D5D-45F2-9B6A-64F34B812C53}"/>
+    <hyperlink ref="D81" r:id="rId187" display="https://www.linkedin.com/in/ryan-catani-0a67317/" xr:uid="{18AC0A40-4DEB-4581-88F2-A1C0B96D42B6}"/>
+    <hyperlink ref="I81" r:id="rId188" display="http://www.macegroup.com/" xr:uid="{E1542C94-51DE-4F6B-9B92-6548EE80C9E4}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Add day 30  progress
</commit_message>
<xml_diff>
--- a/Defining ICP/Defined Leads.xlsx
+++ b/Defining ICP/Defined Leads.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\R E E M\Documents\EVA Ops Training\Defining ICP\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5EF6908E-9ECB-47DF-A41A-70DBB06279F9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E1BACC97-287E-4085-9118-13C0AF9CB401}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="1152" yWindow="1284" windowWidth="17280" windowHeight="9960" xr2:uid="{DAB7335F-B748-4A40-8146-0BCBFC1873B2}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="910" uniqueCount="610">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1085" uniqueCount="717">
   <si>
     <t>Name</t>
   </si>
@@ -1868,6 +1868,327 @@
   </si>
   <si>
     <t>+44 20 3522 3081</t>
+  </si>
+  <si>
+    <t>Leo Faelden</t>
+  </si>
+  <si>
+    <t>Talent Acquisition Manager</t>
+  </si>
+  <si>
+    <t>Dewan Architects &amp; Engineers</t>
+  </si>
+  <si>
+    <t>Leo Faelden | LinkedIn</t>
+  </si>
+  <si>
+    <t>Talent Acquisition Manager responsible for recruiting engineers, architects, designers, and project professionals</t>
+  </si>
+  <si>
+    <t>l.faelden@dewan-architects.com</t>
+  </si>
+  <si>
+    <t>http://www.dewan-architects.com</t>
+  </si>
+  <si>
+    <t>Akram Rafie</t>
+  </si>
+  <si>
+    <t>Abunayyan Holding</t>
+  </si>
+  <si>
+    <t>Akram Rafie | LinkedIn</t>
+  </si>
+  <si>
+    <t>Talent Acquisition Manager responsible for recruiting engineering, construction, industrial, infrastructure, and energy professionals across a large diversified group</t>
+  </si>
+  <si>
+    <t>akram-rafie@abunayyanholding.com</t>
+  </si>
+  <si>
+    <t>+966 11 477 9111</t>
+  </si>
+  <si>
+    <t>(2) Abunayyan Holding: Overview | LinkedIn</t>
+  </si>
+  <si>
+    <t>Mohammed Febin</t>
+  </si>
+  <si>
+    <t>Al Nasr Contracting</t>
+  </si>
+  <si>
+    <t>Mohammed Febin | LinkedIn</t>
+  </si>
+  <si>
+    <t>Talent Acquisition Manager responsible for recruiting engineering, construction, infrastructure, project management, and technical professionals for a large-scale contracting company</t>
+  </si>
+  <si>
+    <t>mohammed.febin@alnasruae.com</t>
+  </si>
+  <si>
+    <t>http://www.alnasruae.com</t>
+  </si>
+  <si>
+    <t>+971 2 642 0002</t>
+  </si>
+  <si>
+    <t>Anitha Ganesh</t>
+  </si>
+  <si>
+    <t>Talent Acquisition Manager MEA</t>
+  </si>
+  <si>
+    <t>Bechtel Corporation</t>
+  </si>
+  <si>
+    <t>Anitha Ganesh | LinkedIn</t>
+  </si>
+  <si>
+    <t>Talent Acquisition Manager leading recruitment across engineering, procurement, construction (EPC), infrastructure, and large-scale project delivery teams throughout the MEA region.</t>
+  </si>
+  <si>
+    <t>http://www.bechtel.com</t>
+  </si>
+  <si>
+    <t>aganesh1@bechtel.com</t>
+  </si>
+  <si>
+    <t>+1 571-392-6300</t>
+  </si>
+  <si>
+    <t>Mohammed Alqarni</t>
+  </si>
+  <si>
+    <t>SISCO</t>
+  </si>
+  <si>
+    <t>Mohammed Alqarni | LinkedIn</t>
+  </si>
+  <si>
+    <t>Talent Acquisition Manager responsible for recruiting engineering, construction, industrial services, infrastructure, and project-based professionals across Saudi Arabia.</t>
+  </si>
+  <si>
+    <t>m.qarni@siscosaudi.com</t>
+  </si>
+  <si>
+    <t>http://www.siscosaudi.com</t>
+  </si>
+  <si>
+    <t>+966 13 340 7999</t>
+  </si>
+  <si>
+    <t>Matthew Bennett</t>
+  </si>
+  <si>
+    <t>Arabian Construction Company (ACC)</t>
+  </si>
+  <si>
+    <t>Matthew Bennett, Assoc. CIPD | LinkedIn</t>
+  </si>
+  <si>
+    <t>Group Talent Acquisition Manager responsible for recruitment across large-scale construction, engineering, project management, and infrastructure projects</t>
+  </si>
+  <si>
+    <t>mbennett@accsal.com</t>
+  </si>
+  <si>
+    <t>http://www.accgroup.com</t>
+  </si>
+  <si>
+    <t>+971 2 644 5400</t>
+  </si>
+  <si>
+    <t>Iustina Blidariu</t>
+  </si>
+  <si>
+    <t>Mott MacDonald</t>
+  </si>
+  <si>
+    <t>Iustina Blidariu | LinkedIn</t>
+  </si>
+  <si>
+    <t>Middle East Talent Acquisition Manager responsible for regional recruitment across engineering, infrastructure, transportation, water, energy, and development consultancy projects.</t>
+  </si>
+  <si>
+    <t>iustina.blidariu@mottmac.com</t>
+  </si>
+  <si>
+    <t>+44 (0)20 7651 0300</t>
+  </si>
+  <si>
+    <t>https://mottmac.com</t>
+  </si>
+  <si>
+    <t>Sam Jordan</t>
+  </si>
+  <si>
+    <t>Jacobs</t>
+  </si>
+  <si>
+    <t>Sam Jordan | LinkedIn</t>
+  </si>
+  <si>
+    <t>Talent Acquisition Manager responsible for recruitment across infrastructure, utilities, environment, energy, and giga engineering projects throughout the MENA region.</t>
+  </si>
+  <si>
+    <t>sam.jordan@jacobs.com</t>
+  </si>
+  <si>
+    <t>http://www.jacobs.com</t>
+  </si>
+  <si>
+    <t>+1 214-638-0145</t>
+  </si>
+  <si>
+    <t>Engineering &amp; Construction</t>
+  </si>
+  <si>
+    <t>Areeba Yahya</t>
+  </si>
+  <si>
+    <t>Power On Building Contracting LLC</t>
+  </si>
+  <si>
+    <t>AREEBA YAHYA | LinkedIn</t>
+  </si>
+  <si>
+    <t>HR professional supporting recruitment, onboarding, workforce planning, and talent acquisition activities within an engineering and construction company.</t>
+  </si>
+  <si>
+    <t>areeba.y@poweron.ae</t>
+  </si>
+  <si>
+    <t>http://www.poweron.ae</t>
+  </si>
+  <si>
+    <t>Abdulla Nigil</t>
+  </si>
+  <si>
+    <t>Egis</t>
+  </si>
+  <si>
+    <t>Abdulla Nigil | LinkedIn</t>
+  </si>
+  <si>
+    <t>Talent Acquisition Manager supporting engineering, infrastructure, and construction hiring across a global engineering firm.</t>
+  </si>
+  <si>
+    <t>abdulla.nigil@egis-group.com</t>
+  </si>
+  <si>
+    <t>http://www.egis-group.com</t>
+  </si>
+  <si>
+    <t>+33 1 39 41 40 00</t>
+  </si>
+  <si>
+    <t>Ahmad Sanjar</t>
+  </si>
+  <si>
+    <t>Phoenicia University</t>
+  </si>
+  <si>
+    <t>Ahmad Sanjar | LinkedIn</t>
+  </si>
+  <si>
+    <t>Recruitment Manager in Higher Education with extensive talent acquisition experience.</t>
+  </si>
+  <si>
+    <t>ahmad.sanjar@pu.edu.lb</t>
+  </si>
+  <si>
+    <t>961-7-420720</t>
+  </si>
+  <si>
+    <t>http://www.pu.edu.lb</t>
+  </si>
+  <si>
+    <t>Higher Education</t>
+  </si>
+  <si>
+    <t>Educational Institutions</t>
+  </si>
+  <si>
+    <t>Fahad Al Fawaz</t>
+  </si>
+  <si>
+    <t>National Company for Learning &amp; Education (NCLE)</t>
+  </si>
+  <si>
+    <t>Fahad Al Fawaz | LinkedIn</t>
+  </si>
+  <si>
+    <t>Director of Talent Acquisition &amp; Onboarding at a leading education provider with direct recruitment decision-making authority.</t>
+  </si>
+  <si>
+    <t>f-alfawaz@edu.com.sa</t>
+  </si>
+  <si>
+    <t>http://www.edu.com.sa</t>
+  </si>
+  <si>
+    <t>Education</t>
+  </si>
+  <si>
+    <t>Emma Bedford</t>
+  </si>
+  <si>
+    <t>Cognita Schools</t>
+  </si>
+  <si>
+    <t>Emma Bedford | LinkedIn</t>
+  </si>
+  <si>
+    <t>Recruitment Manager at a global K-12 school group responsible for talent attraction and recruitment.</t>
+  </si>
+  <si>
+    <t>emma.bedford@cognita.com</t>
+  </si>
+  <si>
+    <t>http://www.cognita.com</t>
+  </si>
+  <si>
+    <t>+44 16 5678 2509</t>
+  </si>
+  <si>
+    <t>Caroline Habr</t>
+  </si>
+  <si>
+    <t>Gulf Education</t>
+  </si>
+  <si>
+    <t>Caroline Habr | LinkedIn</t>
+  </si>
+  <si>
+    <t>Recruitment Manager at an education consultancy specializing in teacher recruitment and educational services.</t>
+  </si>
+  <si>
+    <t>caroline@gulfeducation.ae</t>
+  </si>
+  <si>
+    <t>+971 2677 7708</t>
+  </si>
+  <si>
+    <t>http://www.gulfeducation.ae</t>
+  </si>
+  <si>
+    <t>Jaber Al Mallah</t>
+  </si>
+  <si>
+    <t>Australian University (Kuwait)</t>
+  </si>
+  <si>
+    <t>Jaber Al Mallah | LinkedIn</t>
+  </si>
+  <si>
+    <t>Recruitment Manager at a private university responsible for talent acquisition within the higher education sector.</t>
+  </si>
+  <si>
+    <t>j.mallah@au.edu.kw</t>
+  </si>
+  <si>
+    <t>http://www.au.edu.kw</t>
   </si>
 </sst>
 </file>
@@ -2320,7 +2641,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3B2D820C-3568-45BE-99C1-F7479358E85B}">
-  <dimension ref="A1:M81"/>
+  <dimension ref="A1:M96"/>
   <sheetFormatPr defaultRowHeight="15.6" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="21.88671875" style="2" bestFit="1" customWidth="1"/>
@@ -2335,7 +2656,7 @@
     <col min="10" max="10" width="25.77734375" style="1" bestFit="1" customWidth="1"/>
     <col min="11" max="11" width="11.77734375" style="1" customWidth="1"/>
     <col min="12" max="12" width="11" style="1" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="18.88671875" style="1" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="20.88671875" style="1" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:13" s="10" customFormat="1" x14ac:dyDescent="0.3">
@@ -5535,6 +5856,609 @@
       </c>
       <c r="M81" s="1" t="s">
         <v>30</v>
+      </c>
+    </row>
+    <row r="82" spans="1:13" ht="16.8" x14ac:dyDescent="0.3">
+      <c r="A82" s="1" t="s">
+        <v>610</v>
+      </c>
+      <c r="B82" s="1" t="s">
+        <v>611</v>
+      </c>
+      <c r="C82" s="6" t="s">
+        <v>612</v>
+      </c>
+      <c r="D82" s="4" t="s">
+        <v>613</v>
+      </c>
+      <c r="E82" t="s">
+        <v>614</v>
+      </c>
+      <c r="F82" s="1" t="s">
+        <v>79</v>
+      </c>
+      <c r="G82" t="s">
+        <v>615</v>
+      </c>
+      <c r="I82" s="4" t="s">
+        <v>616</v>
+      </c>
+      <c r="J82" s="1" t="s">
+        <v>87</v>
+      </c>
+      <c r="K82" s="1">
+        <v>1984</v>
+      </c>
+      <c r="L82" s="1" t="s">
+        <v>51</v>
+      </c>
+      <c r="M82" s="1" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="83" spans="1:13" ht="16.8" x14ac:dyDescent="0.3">
+      <c r="A83" s="1" t="s">
+        <v>617</v>
+      </c>
+      <c r="B83" s="1" t="s">
+        <v>611</v>
+      </c>
+      <c r="C83" s="6" t="s">
+        <v>618</v>
+      </c>
+      <c r="D83" s="4" t="s">
+        <v>619</v>
+      </c>
+      <c r="E83" t="s">
+        <v>620</v>
+      </c>
+      <c r="F83" s="1" t="s">
+        <v>49</v>
+      </c>
+      <c r="G83" t="s">
+        <v>621</v>
+      </c>
+      <c r="H83" s="11" t="s">
+        <v>622</v>
+      </c>
+      <c r="I83" s="4" t="s">
+        <v>623</v>
+      </c>
+      <c r="J83" s="1" t="s">
+        <v>87</v>
+      </c>
+      <c r="K83" s="1">
+        <v>1950</v>
+      </c>
+      <c r="L83" s="1" t="s">
+        <v>548</v>
+      </c>
+      <c r="M83" s="1" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="84" spans="1:13" ht="16.8" x14ac:dyDescent="0.3">
+      <c r="A84" s="1" t="s">
+        <v>624</v>
+      </c>
+      <c r="B84" s="1" t="s">
+        <v>611</v>
+      </c>
+      <c r="C84" s="6" t="s">
+        <v>625</v>
+      </c>
+      <c r="D84" s="4" t="s">
+        <v>626</v>
+      </c>
+      <c r="E84" t="s">
+        <v>627</v>
+      </c>
+      <c r="F84" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="G84" t="s">
+        <v>628</v>
+      </c>
+      <c r="H84" s="11" t="s">
+        <v>630</v>
+      </c>
+      <c r="I84" s="4" t="s">
+        <v>629</v>
+      </c>
+      <c r="J84" s="1" t="s">
+        <v>87</v>
+      </c>
+      <c r="K84" s="1">
+        <v>1972</v>
+      </c>
+      <c r="L84" s="1" t="s">
+        <v>548</v>
+      </c>
+      <c r="M84" s="1" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="85" spans="1:13" ht="16.8" x14ac:dyDescent="0.3">
+      <c r="A85" s="1" t="s">
+        <v>631</v>
+      </c>
+      <c r="B85" s="1" t="s">
+        <v>632</v>
+      </c>
+      <c r="C85" s="6" t="s">
+        <v>633</v>
+      </c>
+      <c r="D85" s="4" t="s">
+        <v>634</v>
+      </c>
+      <c r="E85" t="s">
+        <v>635</v>
+      </c>
+      <c r="F85" s="1" t="s">
+        <v>49</v>
+      </c>
+      <c r="G85" t="s">
+        <v>637</v>
+      </c>
+      <c r="H85" s="11" t="s">
+        <v>638</v>
+      </c>
+      <c r="I85" s="4" t="s">
+        <v>636</v>
+      </c>
+      <c r="J85" s="1" t="s">
+        <v>87</v>
+      </c>
+      <c r="K85" s="1">
+        <v>1898</v>
+      </c>
+      <c r="L85" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="M85" s="1" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="86" spans="1:13" ht="16.8" x14ac:dyDescent="0.3">
+      <c r="A86" s="1" t="s">
+        <v>639</v>
+      </c>
+      <c r="B86" s="1" t="s">
+        <v>611</v>
+      </c>
+      <c r="C86" s="6" t="s">
+        <v>640</v>
+      </c>
+      <c r="D86" s="4" t="s">
+        <v>641</v>
+      </c>
+      <c r="E86" t="s">
+        <v>642</v>
+      </c>
+      <c r="F86" s="1" t="s">
+        <v>49</v>
+      </c>
+      <c r="G86" t="s">
+        <v>643</v>
+      </c>
+      <c r="H86" s="11" t="s">
+        <v>645</v>
+      </c>
+      <c r="I86" s="4" t="s">
+        <v>644</v>
+      </c>
+      <c r="J86" s="1" t="s">
+        <v>87</v>
+      </c>
+      <c r="L86" s="1" t="s">
+        <v>574</v>
+      </c>
+      <c r="M86" s="1" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="87" spans="1:13" ht="16.8" x14ac:dyDescent="0.3">
+      <c r="A87" s="1" t="s">
+        <v>646</v>
+      </c>
+      <c r="B87" s="1" t="s">
+        <v>611</v>
+      </c>
+      <c r="C87" s="6" t="s">
+        <v>647</v>
+      </c>
+      <c r="D87" s="4" t="s">
+        <v>648</v>
+      </c>
+      <c r="E87" t="s">
+        <v>649</v>
+      </c>
+      <c r="F87" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="G87" t="s">
+        <v>650</v>
+      </c>
+      <c r="H87" s="11" t="s">
+        <v>652</v>
+      </c>
+      <c r="I87" s="4" t="s">
+        <v>651</v>
+      </c>
+      <c r="J87" s="1" t="s">
+        <v>87</v>
+      </c>
+      <c r="K87" s="1">
+        <v>1967</v>
+      </c>
+      <c r="L87" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="M87" s="1" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="88" spans="1:13" ht="16.8" x14ac:dyDescent="0.3">
+      <c r="A88" s="1" t="s">
+        <v>653</v>
+      </c>
+      <c r="B88" s="1" t="s">
+        <v>611</v>
+      </c>
+      <c r="C88" s="6" t="s">
+        <v>654</v>
+      </c>
+      <c r="D88" s="4" t="s">
+        <v>655</v>
+      </c>
+      <c r="E88" t="s">
+        <v>656</v>
+      </c>
+      <c r="F88" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="G88" t="s">
+        <v>657</v>
+      </c>
+      <c r="H88" s="4" t="s">
+        <v>658</v>
+      </c>
+      <c r="I88" s="4" t="s">
+        <v>659</v>
+      </c>
+      <c r="J88" s="1" t="s">
+        <v>87</v>
+      </c>
+      <c r="K88" s="1">
+        <v>1989</v>
+      </c>
+      <c r="L88" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="M88" s="1" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="89" spans="1:13" ht="16.8" x14ac:dyDescent="0.3">
+      <c r="A89" s="1" t="s">
+        <v>660</v>
+      </c>
+      <c r="B89" s="1" t="s">
+        <v>611</v>
+      </c>
+      <c r="C89" s="6" t="s">
+        <v>661</v>
+      </c>
+      <c r="D89" s="4" t="s">
+        <v>662</v>
+      </c>
+      <c r="E89" t="s">
+        <v>663</v>
+      </c>
+      <c r="F89" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="G89" t="s">
+        <v>664</v>
+      </c>
+      <c r="H89" s="11" t="s">
+        <v>666</v>
+      </c>
+      <c r="I89" s="4" t="s">
+        <v>665</v>
+      </c>
+      <c r="J89" s="1" t="s">
+        <v>667</v>
+      </c>
+      <c r="K89" s="1">
+        <v>1947</v>
+      </c>
+      <c r="L89" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="M89" s="1" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="90" spans="1:13" ht="16.8" x14ac:dyDescent="0.3">
+      <c r="A90" s="1" t="s">
+        <v>668</v>
+      </c>
+      <c r="B90" s="1" t="s">
+        <v>273</v>
+      </c>
+      <c r="C90" s="6" t="s">
+        <v>669</v>
+      </c>
+      <c r="D90" s="4" t="s">
+        <v>670</v>
+      </c>
+      <c r="E90" t="s">
+        <v>671</v>
+      </c>
+      <c r="F90" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="G90" t="s">
+        <v>672</v>
+      </c>
+      <c r="H90" s="4">
+        <v>97143809355</v>
+      </c>
+      <c r="I90" s="4" t="s">
+        <v>673</v>
+      </c>
+      <c r="J90" s="1" t="s">
+        <v>667</v>
+      </c>
+      <c r="K90" s="1">
+        <v>2008</v>
+      </c>
+      <c r="L90" s="1" t="s">
+        <v>446</v>
+      </c>
+      <c r="M90" s="1" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="91" spans="1:13" ht="16.8" x14ac:dyDescent="0.3">
+      <c r="A91" s="1" t="s">
+        <v>674</v>
+      </c>
+      <c r="B91" s="1" t="s">
+        <v>611</v>
+      </c>
+      <c r="C91" s="6" t="s">
+        <v>675</v>
+      </c>
+      <c r="D91" s="4" t="s">
+        <v>676</v>
+      </c>
+      <c r="E91" t="s">
+        <v>677</v>
+      </c>
+      <c r="F91" s="1" t="s">
+        <v>79</v>
+      </c>
+      <c r="G91" t="s">
+        <v>678</v>
+      </c>
+      <c r="H91" s="11" t="s">
+        <v>680</v>
+      </c>
+      <c r="I91" s="4" t="s">
+        <v>679</v>
+      </c>
+      <c r="J91" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="K91" s="1">
+        <v>1947</v>
+      </c>
+      <c r="L91" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="M91" s="1" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="92" spans="1:13" ht="16.8" x14ac:dyDescent="0.3">
+      <c r="A92" s="1" t="s">
+        <v>681</v>
+      </c>
+      <c r="B92" s="1" t="s">
+        <v>257</v>
+      </c>
+      <c r="C92" s="6" t="s">
+        <v>682</v>
+      </c>
+      <c r="D92" s="4" t="s">
+        <v>683</v>
+      </c>
+      <c r="E92" t="s">
+        <v>684</v>
+      </c>
+      <c r="F92" s="1" t="s">
+        <v>467</v>
+      </c>
+      <c r="G92" t="s">
+        <v>685</v>
+      </c>
+      <c r="H92" s="4" t="s">
+        <v>686</v>
+      </c>
+      <c r="I92" s="4" t="s">
+        <v>687</v>
+      </c>
+      <c r="J92" s="1" t="s">
+        <v>688</v>
+      </c>
+      <c r="L92" s="1" t="s">
+        <v>446</v>
+      </c>
+      <c r="M92" s="1" t="s">
+        <v>689</v>
+      </c>
+    </row>
+    <row r="93" spans="1:13" ht="16.8" x14ac:dyDescent="0.3">
+      <c r="A93" s="1" t="s">
+        <v>690</v>
+      </c>
+      <c r="B93" s="1" t="s">
+        <v>257</v>
+      </c>
+      <c r="C93" s="6" t="s">
+        <v>691</v>
+      </c>
+      <c r="D93" s="4" t="s">
+        <v>692</v>
+      </c>
+      <c r="E93" t="s">
+        <v>693</v>
+      </c>
+      <c r="F93" s="1" t="s">
+        <v>49</v>
+      </c>
+      <c r="G93" t="s">
+        <v>694</v>
+      </c>
+      <c r="H93" s="8">
+        <v>553305301</v>
+      </c>
+      <c r="I93" s="4" t="s">
+        <v>695</v>
+      </c>
+      <c r="J93" s="1" t="s">
+        <v>696</v>
+      </c>
+      <c r="K93" s="1">
+        <v>1958</v>
+      </c>
+      <c r="L93" s="1" t="s">
+        <v>548</v>
+      </c>
+      <c r="M93" s="1" t="s">
+        <v>689</v>
+      </c>
+    </row>
+    <row r="94" spans="1:13" ht="16.8" x14ac:dyDescent="0.3">
+      <c r="A94" s="1" t="s">
+        <v>697</v>
+      </c>
+      <c r="B94" s="1" t="s">
+        <v>257</v>
+      </c>
+      <c r="C94" s="6" t="s">
+        <v>698</v>
+      </c>
+      <c r="D94" s="4" t="s">
+        <v>699</v>
+      </c>
+      <c r="E94" t="s">
+        <v>700</v>
+      </c>
+      <c r="F94" s="1" t="s">
+        <v>79</v>
+      </c>
+      <c r="G94" t="s">
+        <v>701</v>
+      </c>
+      <c r="H94" s="11" t="s">
+        <v>703</v>
+      </c>
+      <c r="I94" s="4" t="s">
+        <v>702</v>
+      </c>
+      <c r="J94" s="1" t="s">
+        <v>696</v>
+      </c>
+      <c r="K94" s="1">
+        <v>2004</v>
+      </c>
+      <c r="L94" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="M94" s="1" t="s">
+        <v>689</v>
+      </c>
+    </row>
+    <row r="95" spans="1:13" ht="16.8" x14ac:dyDescent="0.3">
+      <c r="A95" s="1" t="s">
+        <v>704</v>
+      </c>
+      <c r="B95" s="1" t="s">
+        <v>257</v>
+      </c>
+      <c r="C95" s="6" t="s">
+        <v>705</v>
+      </c>
+      <c r="D95" s="4" t="s">
+        <v>706</v>
+      </c>
+      <c r="E95" t="s">
+        <v>707</v>
+      </c>
+      <c r="F95" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="G95" t="s">
+        <v>708</v>
+      </c>
+      <c r="H95" s="4" t="s">
+        <v>709</v>
+      </c>
+      <c r="I95" s="4" t="s">
+        <v>710</v>
+      </c>
+      <c r="J95" s="1" t="s">
+        <v>696</v>
+      </c>
+      <c r="L95" s="1">
+        <v>10</v>
+      </c>
+      <c r="M95" s="1" t="s">
+        <v>689</v>
+      </c>
+    </row>
+    <row r="96" spans="1:13" ht="16.8" x14ac:dyDescent="0.3">
+      <c r="A96" s="1" t="s">
+        <v>711</v>
+      </c>
+      <c r="B96" s="1" t="s">
+        <v>257</v>
+      </c>
+      <c r="C96" s="6" t="s">
+        <v>712</v>
+      </c>
+      <c r="D96" s="4" t="s">
+        <v>713</v>
+      </c>
+      <c r="E96" t="s">
+        <v>714</v>
+      </c>
+      <c r="F96" s="1" t="s">
+        <v>546</v>
+      </c>
+      <c r="G96" t="s">
+        <v>715</v>
+      </c>
+      <c r="H96" s="8">
+        <v>1828225</v>
+      </c>
+      <c r="I96" s="4" t="s">
+        <v>716</v>
+      </c>
+      <c r="J96" s="1" t="s">
+        <v>688</v>
+      </c>
+      <c r="K96" s="1">
+        <v>2004</v>
+      </c>
+      <c r="L96" s="1" t="s">
+        <v>446</v>
+      </c>
+      <c r="M96" s="1" t="s">
+        <v>689</v>
       </c>
     </row>
   </sheetData>
@@ -5728,6 +6652,42 @@
     <hyperlink ref="I80" r:id="rId186" display="http://www.binyah.com.sa/" xr:uid="{5D874C19-9D5D-45F2-9B6A-64F34B812C53}"/>
     <hyperlink ref="D81" r:id="rId187" display="https://www.linkedin.com/in/ryan-catani-0a67317/" xr:uid="{18AC0A40-4DEB-4581-88F2-A1C0B96D42B6}"/>
     <hyperlink ref="I81" r:id="rId188" display="http://www.macegroup.com/" xr:uid="{E1542C94-51DE-4F6B-9B92-6548EE80C9E4}"/>
+    <hyperlink ref="D82" r:id="rId189" display="https://www.linkedin.com/in/leo-faelden-6340a328/" xr:uid="{AC9DFC11-FEA9-450A-ADE1-9D238BC595BD}"/>
+    <hyperlink ref="I82" r:id="rId190" display="http://www.dewan-architects.com/" xr:uid="{A68886A8-FD49-4A05-87FD-D39A8CA6F639}"/>
+    <hyperlink ref="D83" r:id="rId191" display="https://www.linkedin.com/in/akramrafie/" xr:uid="{92899CC1-72E1-4A1B-A79A-B4B570725F71}"/>
+    <hyperlink ref="I83" r:id="rId192" display="https://www.linkedin.com/company/abunayyan-holding/" xr:uid="{53005178-26AF-4E68-8F7C-10C0FD53B239}"/>
+    <hyperlink ref="D84" r:id="rId193" display="https://www.linkedin.com/in/mohammed-febin-6477a67/" xr:uid="{61421A67-1F2C-4F23-A93A-5A3F7524C6D3}"/>
+    <hyperlink ref="I84" r:id="rId194" display="http://www.alnasruae.com/" xr:uid="{2844B0E0-392D-4EBE-8C90-82F4DAAF204C}"/>
+    <hyperlink ref="D85" r:id="rId195" display="https://www.linkedin.com/in/anithaganesh/" xr:uid="{026FD3C4-3664-4984-9E1D-129A5F32A66B}"/>
+    <hyperlink ref="I85" r:id="rId196" display="http://www.bechtel.com/" xr:uid="{FA0AF543-C559-4E62-946A-9D571AF41C52}"/>
+    <hyperlink ref="D86" r:id="rId197" display="https://www.linkedin.com/in/mohammed-alqarni-398149124/" xr:uid="{DDCAFB9F-8E58-490B-8315-C74CA2F4B2DE}"/>
+    <hyperlink ref="I86" r:id="rId198" display="http://www.siscosaudi.com/" xr:uid="{C65F3FFA-B614-4A40-AC3C-9C8D45E0560D}"/>
+    <hyperlink ref="D87" r:id="rId199" display="https://www.linkedin.com/in/matthew-bennett-assoc-cipd-91335733/" xr:uid="{068A01D8-041A-4FCF-9DD8-382167C7FE81}"/>
+    <hyperlink ref="I87" r:id="rId200" display="http://www.accgroup.com/" xr:uid="{780E64DE-CC0D-4C50-8E35-8A739A8FC0C1}"/>
+    <hyperlink ref="D88" r:id="rId201" display="https://www.linkedin.com/in/iustina-antonia-blidariu/" xr:uid="{9E97B803-F9A0-4355-BAE9-CC6F388E49F7}"/>
+    <hyperlink ref="H88" r:id="rId202" display="tel:+44 (0)20 7651 0300" xr:uid="{7D317516-431A-486B-AFBA-8F8E921F418A}"/>
+    <hyperlink ref="I88" r:id="rId203" display="https://mottmac.com/" xr:uid="{DCAF4926-15AD-4E56-AE5E-C48EA49678AD}"/>
+    <hyperlink ref="D89" r:id="rId204" display="https://www.linkedin.com/in/sam-jordan-12a3b97a/" xr:uid="{DCDFC2FC-F17C-4A6E-96D4-F5CD1CE10B31}"/>
+    <hyperlink ref="I89" r:id="rId205" display="http://www.jacobs.com/" xr:uid="{6CBE9999-8EA6-4348-BAD4-D0FBD7B89003}"/>
+    <hyperlink ref="D90" r:id="rId206" display="https://www.linkedin.com/in/areebayahya/" xr:uid="{8BA504D5-3E0A-42C0-AD3B-B5D2612DA2E2}"/>
+    <hyperlink ref="H90" r:id="rId207" display="tel:+97143809355" xr:uid="{5A08CF1A-6A9C-4443-A1E9-3E628FA3BF62}"/>
+    <hyperlink ref="I90" r:id="rId208" display="http://www.poweron.ae/" xr:uid="{578703BB-5C28-4E6C-94B0-98BCB55BDCAA}"/>
+    <hyperlink ref="D91" r:id="rId209" display="https://www.linkedin.com/in/abdullanigil/" xr:uid="{E2CA0227-4325-4890-8E9A-333F4C945F76}"/>
+    <hyperlink ref="I91" r:id="rId210" display="http://www.egis-group.com/" xr:uid="{40E76329-2828-4C86-8650-61161C3ACDDF}"/>
+    <hyperlink ref="D92" r:id="rId211" display="https://www.linkedin.com/in/ahmad-sanjar-2a2a8842/" xr:uid="{5BD12866-5F0D-4D9F-86C9-1E131052046A}"/>
+    <hyperlink ref="H92" r:id="rId212" display="tel:961-7-420720" xr:uid="{011150AD-5952-4268-A35E-DCB87C000224}"/>
+    <hyperlink ref="I92" r:id="rId213" display="http://www.pu.edu.lb/" xr:uid="{8981821F-6AE2-44E4-B4E1-E9D3ECD9C9A9}"/>
+    <hyperlink ref="D93" r:id="rId214" display="https://www.linkedin.com/in/fahad-al-fawaz-8224a7127/" xr:uid="{57F8D69C-315C-4588-A6AD-FC2B0313176A}"/>
+    <hyperlink ref="H93" r:id="rId215" display="tel:0553305301" xr:uid="{09576BD7-5FA4-4732-956F-30392E15024E}"/>
+    <hyperlink ref="I93" r:id="rId216" display="http://www.edu.com.sa/" xr:uid="{CDD3BF4C-DF40-4D07-B921-77F2DA937E33}"/>
+    <hyperlink ref="D94" r:id="rId217" display="https://www.linkedin.com/in/emma-bedford-ba882513b/" xr:uid="{C90B13EC-CCA9-41B1-82AE-275ACDC36639}"/>
+    <hyperlink ref="I94" r:id="rId218" display="http://www.cognita.com/" xr:uid="{5B0D9F1A-7521-44DD-9420-DDEDDD4140AA}"/>
+    <hyperlink ref="D95" r:id="rId219" display="https://www.linkedin.com/in/caroline-habr-4387a392/" xr:uid="{4A3EBDAD-4001-4DF7-A9E8-268BFF7834F3}"/>
+    <hyperlink ref="H95" r:id="rId220" display="tel:+971 2677 7708" xr:uid="{85B8EB10-5E00-494E-9D1B-E216CBCDC044}"/>
+    <hyperlink ref="I95" r:id="rId221" display="http://www.gulfeducation.ae/" xr:uid="{0BE80AD0-B8C2-4C0A-80D5-32A174A15FE5}"/>
+    <hyperlink ref="D96" r:id="rId222" display="https://www.linkedin.com/in/jaber-al-mallah-3b89007/" xr:uid="{30A225BD-F162-48D1-A2EF-2576045F28AB}"/>
+    <hyperlink ref="H96" r:id="rId223" display="tel:1828225" xr:uid="{82AD8865-24E5-4689-9116-31D40B81B8ED}"/>
+    <hyperlink ref="I96" r:id="rId224" display="http://www.au.edu.kw/" xr:uid="{81CB9416-DE3B-44C4-92BD-84F27E39A96C}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Add day 31 progress
</commit_message>
<xml_diff>
--- a/Defining ICP/Defined Leads.xlsx
+++ b/Defining ICP/Defined Leads.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\R E E M\Documents\EVA Ops Training\Defining ICP\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E1BACC97-287E-4085-9118-13C0AF9CB401}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A6BF626A-FD42-43DF-94D4-683DC81572E2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="1152" yWindow="1284" windowWidth="17280" windowHeight="9960" xr2:uid="{DAB7335F-B748-4A40-8146-0BCBFC1873B2}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1085" uniqueCount="717">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1306" uniqueCount="846">
   <si>
     <t>Name</t>
   </si>
@@ -2189,6 +2189,393 @@
   </si>
   <si>
     <t>http://www.au.edu.kw</t>
+  </si>
+  <si>
+    <t>Karishma Joshi</t>
+  </si>
+  <si>
+    <t>Student Recruitment Manager</t>
+  </si>
+  <si>
+    <t>Navitas</t>
+  </si>
+  <si>
+    <t>Karishma Joshi | LinkedIn</t>
+  </si>
+  <si>
+    <t>Student Recruitment Manager at a global higher education provider, directly involved in student recruitment and enrollment operations.</t>
+  </si>
+  <si>
+    <t>karishma.joshi@navitas.com</t>
+  </si>
+  <si>
+    <t>+1 619-314-9600</t>
+  </si>
+  <si>
+    <t>http://www.navitas.com</t>
+  </si>
+  <si>
+    <t>Ali Ezaldeen</t>
+  </si>
+  <si>
+    <t>The American University in the Emirates (AUE)</t>
+  </si>
+  <si>
+    <t>Ali Ezaldeen | LinkedIn</t>
+  </si>
+  <si>
+    <t>Student Recruitment Manager responsible for student enrollment, admissions, and recruitment activities within a higher education institution.</t>
+  </si>
+  <si>
+    <t>ali.ezaldeen@aue.ae</t>
+  </si>
+  <si>
+    <t>http://www.aurak.ac.ae</t>
+  </si>
+  <si>
+    <t>+971 4 449 9000</t>
+  </si>
+  <si>
+    <t>Kevin O'Brien</t>
+  </si>
+  <si>
+    <t>Regional Recruitment Manager</t>
+  </si>
+  <si>
+    <t xml:space="preserve">EHL </t>
+  </si>
+  <si>
+    <t>Kevin O'Brien | LinkedIn</t>
+  </si>
+  <si>
+    <t>Regional Recruitment Manager responsible for student recruitment, enrollment growth, and recruitment strategy across multiple markets in the higher education sector.</t>
+  </si>
+  <si>
+    <t>kevin.obrien@ehl.ch</t>
+  </si>
+  <si>
+    <t>https://www.ehlgroup.com/</t>
+  </si>
+  <si>
+    <t>Lisa Paterson</t>
+  </si>
+  <si>
+    <t>Lisa Paterson | LinkedIn</t>
+  </si>
+  <si>
+    <t>Recruitment Manager overseeing end-to-end recruitment operations across Cognita Schools' GCC network, responsible for attracting, engaging, and retaining educational talent.</t>
+  </si>
+  <si>
+    <t>lisa.paterson@cognita.com</t>
+  </si>
+  <si>
+    <t>Education Management</t>
+  </si>
+  <si>
+    <t>Malika Benallal</t>
+  </si>
+  <si>
+    <t>Education Recruitment Manager</t>
+  </si>
+  <si>
+    <t>Education Recruitment Manager responsible for international student recruitment and university partnership growth across the higher education sector.</t>
+  </si>
+  <si>
+    <t>Malika Benallal | LinkedIn</t>
+  </si>
+  <si>
+    <t>Study Group</t>
+  </si>
+  <si>
+    <t>https://www.studygroup.com/</t>
+  </si>
+  <si>
+    <t>mbenallal@studygroup.com</t>
+  </si>
+  <si>
+    <t>Elena Zwitser</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Advisor </t>
+  </si>
+  <si>
+    <t>Ward Howell International</t>
+  </si>
+  <si>
+    <t>Elena Zwitser (Fedorina) | LinkedIn</t>
+  </si>
+  <si>
+    <t>HR Transformation and Executive Search advisor at a global leadership consulting and executive search firm</t>
+  </si>
+  <si>
+    <t>elena.zwitser@ward-howell.com</t>
+  </si>
+  <si>
+    <t>http://www.ward-howell.com</t>
+  </si>
+  <si>
+    <t>+49 43 152408600</t>
+  </si>
+  <si>
+    <t>Ibrahim Albidewi</t>
+  </si>
+  <si>
+    <t>Ministry of Education</t>
+  </si>
+  <si>
+    <t>Ibrahim Albidewi | LinkedIn</t>
+  </si>
+  <si>
+    <t>Senior education advisor and strategic planning expert with extensive leadership experience in the education sector.</t>
+  </si>
+  <si>
+    <t>ialbidewi@moe.gov.sa</t>
+  </si>
+  <si>
+    <t>http://www.moe.gov.sa</t>
+  </si>
+  <si>
+    <t>+966 16 324 7000</t>
+  </si>
+  <si>
+    <t>James Brown</t>
+  </si>
+  <si>
+    <t>Head of Student Recruitment</t>
+  </si>
+  <si>
+    <t>KAUST (King Abdullah University of Science and Technology)</t>
+  </si>
+  <si>
+    <t>James Brown | LinkedIn</t>
+  </si>
+  <si>
+    <t>Direct decision-maker responsible for student recruitment and enrollment strategy at a leading Saudi university. Strong fit for Recruitment CRM.</t>
+  </si>
+  <si>
+    <t>james.brown.1@kaust.edu.sa</t>
+  </si>
+  <si>
+    <t>+966 12 808 3463</t>
+  </si>
+  <si>
+    <t>https://www.kaust.edu.sa/en</t>
+  </si>
+  <si>
+    <t>Anna Traykova</t>
+  </si>
+  <si>
+    <t>Anna Traykova | LinkedIn</t>
+  </si>
+  <si>
+    <t>Leads student recruitment activities for Navitas. Directly involved in attracting and managing student pipelines and enrollment processes. Strong Recruitment CRM fit.</t>
+  </si>
+  <si>
+    <t>anna.traykova@navitas.com</t>
+  </si>
+  <si>
+    <t>Tarkan Ulas</t>
+  </si>
+  <si>
+    <t>OnCampus Global</t>
+  </si>
+  <si>
+    <t>Tarkan Ulas | LinkedIn</t>
+  </si>
+  <si>
+    <t>Manages student recruitment for OnCampus Global. Responsible for attracting and enrolling international students. Strong fit for recruitment workflow and pipeline management solutions.</t>
+  </si>
+  <si>
+    <t>tulas@oncampus.global</t>
+  </si>
+  <si>
+    <t>+44 12 2334 5698</t>
+  </si>
+  <si>
+    <t>Seham Nada</t>
+  </si>
+  <si>
+    <t>Head of Student Recruitment Unit</t>
+  </si>
+  <si>
+    <t>IBTE</t>
+  </si>
+  <si>
+    <t>Seham Nada | LinkedIn</t>
+  </si>
+  <si>
+    <t>Leads the Student Recruitment Unit at IBTE. Responsible for student acquisition, admissions, enrollment, and recruitment operations. Strong fit for Recruitment CRM solutions.</t>
+  </si>
+  <si>
+    <t>seham.n@ibte.me</t>
+  </si>
+  <si>
+    <t>+971 45 788822</t>
+  </si>
+  <si>
+    <t>https://www.ibte.me/</t>
+  </si>
+  <si>
+    <t>https://tr.ee/OnCampus</t>
+  </si>
+  <si>
+    <t>Kutiba Nusair</t>
+  </si>
+  <si>
+    <t>Masiratna</t>
+  </si>
+  <si>
+    <t>Kutiba Nusair | LinkedIn</t>
+  </si>
+  <si>
+    <t>Manages student recruitment for an education consultancy helping students secure admissions at international universities.</t>
+  </si>
+  <si>
+    <t>kutiba@masiratna.com</t>
+  </si>
+  <si>
+    <t>+966 59 236 4444</t>
+  </si>
+  <si>
+    <t>30+</t>
+  </si>
+  <si>
+    <t>Mohammad Nufaie</t>
+  </si>
+  <si>
+    <t>Alfaisal University</t>
+  </si>
+  <si>
+    <t>Mohammad Al Nufaie | LinkedIn</t>
+  </si>
+  <si>
+    <t>Responsible for student recruitment at a university. Directly involved in attracting, managing, and converting prospective students into enrolled students.</t>
+  </si>
+  <si>
+    <t>mnufaie@alfaisal.edu</t>
+  </si>
+  <si>
+    <t>http://www.alfaisal.edu</t>
+  </si>
+  <si>
+    <t>920 000570</t>
+  </si>
+  <si>
+    <t>Rim Tabaja</t>
+  </si>
+  <si>
+    <t>Lebanese American University (LAU)</t>
+  </si>
+  <si>
+    <t>Rim Tabaja | LinkedIn</t>
+  </si>
+  <si>
+    <t>Manages student recruitment activities at LAU, including local and international recruitment, high school partnerships, and student outreach initiatives.</t>
+  </si>
+  <si>
+    <t>rim.tabaja@lau.edu.lb</t>
+  </si>
+  <si>
+    <t>http://www.lau.edu.lb/</t>
+  </si>
+  <si>
+    <t>Danna Marie Herradura</t>
+  </si>
+  <si>
+    <t>Dubai Institute of Design and Innovation (DIDI)</t>
+  </si>
+  <si>
+    <t>Danna Marie Herradura | LinkedIn</t>
+  </si>
+  <si>
+    <t>Responsible for student recruitment activities at a higher education institution focused on design and innovation.</t>
+  </si>
+  <si>
+    <t>danna.herradura@didi.ac.ae</t>
+  </si>
+  <si>
+    <t>http://didi.ac.ae/</t>
+  </si>
+  <si>
+    <t>Abhishek Sachin</t>
+  </si>
+  <si>
+    <t>Admissions Manager</t>
+  </si>
+  <si>
+    <t>ALLEN Career Institute Overseas</t>
+  </si>
+  <si>
+    <t>Abhishek Sachin | LinkedIn</t>
+  </si>
+  <si>
+    <t>Admissions Manager responsible for student enrollment and admissions operations at ALLEN Career Institute Overseas.</t>
+  </si>
+  <si>
+    <t>abhishek.sachin@allenoverseas.com</t>
+  </si>
+  <si>
+    <t>(+971)567461832</t>
+  </si>
+  <si>
+    <t>https://www.allenoverseas.com/</t>
+  </si>
+  <si>
+    <t>Emily Horsford</t>
+  </si>
+  <si>
+    <t>Harrow International School Dubai</t>
+  </si>
+  <si>
+    <t>Emily Horsford | LinkedIn</t>
+  </si>
+  <si>
+    <t>Admissions Manager overseeing student admissions and enrollment operations at Harrow International School Dubai.</t>
+  </si>
+  <si>
+    <t>ehorsford@harrowdubai.ae</t>
+  </si>
+  <si>
+    <t>harrowdubai.ae</t>
+  </si>
+  <si>
+    <t>+971 50 800 2689</t>
+  </si>
+  <si>
+    <t>Joshua David</t>
+  </si>
+  <si>
+    <t>Mount Institute of Business Development (MIBD Dubai)</t>
+  </si>
+  <si>
+    <t>Joshua David | LinkedIn</t>
+  </si>
+  <si>
+    <t>Admissions Manager responsible for student recruitment, admissions, and enrollment activities at MIBD Dubai.</t>
+  </si>
+  <si>
+    <t>joshua@mountinstitute.com</t>
+  </si>
+  <si>
+    <t>Rayan Baroudi</t>
+  </si>
+  <si>
+    <t>London Business School</t>
+  </si>
+  <si>
+    <t>https://www.linkedin.com/in/rayan-baroudi-150b99179/</t>
+  </si>
+  <si>
+    <t>Admissions Manager responsible for admissions and enrollment activities at London Business School Dubai.</t>
+  </si>
+  <si>
+    <t>rbaroudi@london.edu</t>
+  </si>
+  <si>
+    <t>+44 (0)20 70007000</t>
+  </si>
+  <si>
+    <t>https://www.london.edu/</t>
   </si>
 </sst>
 </file>
@@ -2283,7 +2670,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="18">
+  <cellXfs count="19">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -2326,6 +2713,9 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -2641,10 +3031,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3B2D820C-3568-45BE-99C1-F7479358E85B}">
-  <dimension ref="A1:M96"/>
+  <dimension ref="A1:M115"/>
   <sheetFormatPr defaultRowHeight="15.6" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="21.88671875" style="2" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="23.33203125" style="2" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="35.88671875" style="1" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="57.6640625" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="67.77734375" bestFit="1" customWidth="1"/>
@@ -6458,6 +6848,761 @@
         <v>446</v>
       </c>
       <c r="M96" s="1" t="s">
+        <v>689</v>
+      </c>
+    </row>
+    <row r="97" spans="1:13" ht="16.8" x14ac:dyDescent="0.3">
+      <c r="A97" s="1" t="s">
+        <v>717</v>
+      </c>
+      <c r="B97" s="1" t="s">
+        <v>718</v>
+      </c>
+      <c r="C97" s="6" t="s">
+        <v>719</v>
+      </c>
+      <c r="D97" s="4" t="s">
+        <v>720</v>
+      </c>
+      <c r="E97" t="s">
+        <v>721</v>
+      </c>
+      <c r="F97" s="1" t="s">
+        <v>79</v>
+      </c>
+      <c r="G97" t="s">
+        <v>722</v>
+      </c>
+      <c r="H97" s="11" t="s">
+        <v>723</v>
+      </c>
+      <c r="I97" s="4" t="s">
+        <v>724</v>
+      </c>
+      <c r="J97" s="1" t="s">
+        <v>688</v>
+      </c>
+      <c r="K97" s="1">
+        <v>1994</v>
+      </c>
+      <c r="L97" s="1" t="s">
+        <v>574</v>
+      </c>
+      <c r="M97" s="1" t="s">
+        <v>689</v>
+      </c>
+    </row>
+    <row r="98" spans="1:13" ht="16.8" x14ac:dyDescent="0.3">
+      <c r="A98" s="1" t="s">
+        <v>725</v>
+      </c>
+      <c r="B98" s="1" t="s">
+        <v>718</v>
+      </c>
+      <c r="C98" s="6" t="s">
+        <v>726</v>
+      </c>
+      <c r="D98" s="4" t="s">
+        <v>727</v>
+      </c>
+      <c r="E98" t="s">
+        <v>728</v>
+      </c>
+      <c r="F98" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="G98" t="s">
+        <v>729</v>
+      </c>
+      <c r="H98" s="11" t="s">
+        <v>731</v>
+      </c>
+      <c r="I98" s="4" t="s">
+        <v>730</v>
+      </c>
+      <c r="J98" s="1" t="s">
+        <v>688</v>
+      </c>
+      <c r="K98" s="1">
+        <v>2006</v>
+      </c>
+      <c r="L98" s="1" t="s">
+        <v>446</v>
+      </c>
+      <c r="M98" s="1" t="s">
+        <v>689</v>
+      </c>
+    </row>
+    <row r="99" spans="1:13" ht="16.8" x14ac:dyDescent="0.3">
+      <c r="A99" s="1" t="s">
+        <v>732</v>
+      </c>
+      <c r="B99" s="1" t="s">
+        <v>733</v>
+      </c>
+      <c r="C99" s="6" t="s">
+        <v>734</v>
+      </c>
+      <c r="D99" s="4" t="s">
+        <v>735</v>
+      </c>
+      <c r="E99" t="s">
+        <v>736</v>
+      </c>
+      <c r="F99" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="G99" t="s">
+        <v>737</v>
+      </c>
+      <c r="I99" s="4" t="s">
+        <v>738</v>
+      </c>
+      <c r="J99" s="1" t="s">
+        <v>688</v>
+      </c>
+      <c r="K99" s="1">
+        <v>1893</v>
+      </c>
+      <c r="L99" s="1" t="s">
+        <v>446</v>
+      </c>
+      <c r="M99" s="1" t="s">
+        <v>689</v>
+      </c>
+    </row>
+    <row r="100" spans="1:13" ht="14.4" x14ac:dyDescent="0.3">
+      <c r="A100" s="1" t="s">
+        <v>739</v>
+      </c>
+      <c r="B100" s="1" t="s">
+        <v>257</v>
+      </c>
+      <c r="C100" s="1" t="s">
+        <v>698</v>
+      </c>
+      <c r="D100" s="4" t="s">
+        <v>740</v>
+      </c>
+      <c r="E100" t="s">
+        <v>741</v>
+      </c>
+      <c r="F100" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="G100" t="s">
+        <v>742</v>
+      </c>
+      <c r="H100" s="11" t="s">
+        <v>703</v>
+      </c>
+      <c r="I100" s="4" t="s">
+        <v>702</v>
+      </c>
+      <c r="J100" s="1" t="s">
+        <v>743</v>
+      </c>
+      <c r="K100" s="1">
+        <v>2004</v>
+      </c>
+      <c r="L100" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="M100" s="1" t="s">
+        <v>689</v>
+      </c>
+    </row>
+    <row r="101" spans="1:13" ht="14.4" x14ac:dyDescent="0.3">
+      <c r="A101" s="1" t="s">
+        <v>744</v>
+      </c>
+      <c r="B101" s="1" t="s">
+        <v>745</v>
+      </c>
+      <c r="C101" s="1" t="s">
+        <v>748</v>
+      </c>
+      <c r="D101" s="4" t="s">
+        <v>747</v>
+      </c>
+      <c r="E101" t="s">
+        <v>746</v>
+      </c>
+      <c r="F101" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="G101" t="s">
+        <v>750</v>
+      </c>
+      <c r="I101" s="4" t="s">
+        <v>749</v>
+      </c>
+      <c r="J101" s="1" t="s">
+        <v>688</v>
+      </c>
+      <c r="K101" s="1">
+        <v>1994</v>
+      </c>
+      <c r="L101" s="1" t="s">
+        <v>548</v>
+      </c>
+      <c r="M101" s="1" t="s">
+        <v>689</v>
+      </c>
+    </row>
+    <row r="102" spans="1:13" ht="14.4" x14ac:dyDescent="0.3">
+      <c r="A102" s="1" t="s">
+        <v>751</v>
+      </c>
+      <c r="B102" s="1" t="s">
+        <v>752</v>
+      </c>
+      <c r="C102" s="1" t="s">
+        <v>753</v>
+      </c>
+      <c r="D102" s="4" t="s">
+        <v>754</v>
+      </c>
+      <c r="E102" t="s">
+        <v>755</v>
+      </c>
+      <c r="F102" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="G102" t="s">
+        <v>756</v>
+      </c>
+      <c r="H102" s="11" t="s">
+        <v>758</v>
+      </c>
+      <c r="I102" s="4" t="s">
+        <v>757</v>
+      </c>
+      <c r="J102" s="1" t="s">
+        <v>273</v>
+      </c>
+      <c r="K102" s="1">
+        <v>1951</v>
+      </c>
+      <c r="L102" s="1" t="s">
+        <v>51</v>
+      </c>
+      <c r="M102" s="1" t="s">
+        <v>243</v>
+      </c>
+    </row>
+    <row r="103" spans="1:13" ht="14.4" x14ac:dyDescent="0.3">
+      <c r="A103" s="1" t="s">
+        <v>759</v>
+      </c>
+      <c r="B103" s="1" t="s">
+        <v>752</v>
+      </c>
+      <c r="C103" s="1" t="s">
+        <v>760</v>
+      </c>
+      <c r="D103" s="4" t="s">
+        <v>761</v>
+      </c>
+      <c r="E103" t="s">
+        <v>762</v>
+      </c>
+      <c r="F103" s="1" t="s">
+        <v>49</v>
+      </c>
+      <c r="G103" t="s">
+        <v>763</v>
+      </c>
+      <c r="H103" s="11" t="s">
+        <v>765</v>
+      </c>
+      <c r="I103" s="4" t="s">
+        <v>764</v>
+      </c>
+      <c r="J103" s="1" t="s">
+        <v>696</v>
+      </c>
+      <c r="K103" s="1">
+        <v>1926</v>
+      </c>
+      <c r="L103" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="M103" s="1" t="s">
+        <v>689</v>
+      </c>
+    </row>
+    <row r="104" spans="1:13" ht="14.4" x14ac:dyDescent="0.3">
+      <c r="A104" s="1" t="s">
+        <v>766</v>
+      </c>
+      <c r="B104" s="1" t="s">
+        <v>767</v>
+      </c>
+      <c r="C104" s="1" t="s">
+        <v>768</v>
+      </c>
+      <c r="D104" s="4" t="s">
+        <v>769</v>
+      </c>
+      <c r="E104" t="s">
+        <v>770</v>
+      </c>
+      <c r="F104" s="1" t="s">
+        <v>49</v>
+      </c>
+      <c r="G104" t="s">
+        <v>771</v>
+      </c>
+      <c r="H104" s="11" t="s">
+        <v>772</v>
+      </c>
+      <c r="I104" s="4" t="s">
+        <v>773</v>
+      </c>
+      <c r="J104" s="1" t="s">
+        <v>688</v>
+      </c>
+      <c r="K104" s="1">
+        <v>2009</v>
+      </c>
+      <c r="L104" s="1" t="s">
+        <v>548</v>
+      </c>
+      <c r="M104" s="1" t="s">
+        <v>689</v>
+      </c>
+    </row>
+    <row r="105" spans="1:13" ht="14.4" x14ac:dyDescent="0.3">
+      <c r="A105" s="1" t="s">
+        <v>774</v>
+      </c>
+      <c r="B105" s="1" t="s">
+        <v>767</v>
+      </c>
+      <c r="C105" s="1" t="s">
+        <v>719</v>
+      </c>
+      <c r="D105" s="4" t="s">
+        <v>775</v>
+      </c>
+      <c r="E105" t="s">
+        <v>776</v>
+      </c>
+      <c r="F105" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="G105" t="s">
+        <v>777</v>
+      </c>
+      <c r="H105" s="11" t="s">
+        <v>723</v>
+      </c>
+      <c r="I105" s="4" t="s">
+        <v>724</v>
+      </c>
+      <c r="J105" s="1" t="s">
+        <v>688</v>
+      </c>
+      <c r="K105" s="1">
+        <v>1994</v>
+      </c>
+      <c r="L105" s="1" t="s">
+        <v>574</v>
+      </c>
+      <c r="M105" s="1" t="s">
+        <v>689</v>
+      </c>
+    </row>
+    <row r="106" spans="1:13" ht="14.4" x14ac:dyDescent="0.3">
+      <c r="A106" s="1" t="s">
+        <v>778</v>
+      </c>
+      <c r="B106" s="1" t="s">
+        <v>718</v>
+      </c>
+      <c r="C106" s="1" t="s">
+        <v>779</v>
+      </c>
+      <c r="D106" s="4" t="s">
+        <v>780</v>
+      </c>
+      <c r="E106" s="18" t="s">
+        <v>781</v>
+      </c>
+      <c r="F106" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="G106" t="s">
+        <v>782</v>
+      </c>
+      <c r="H106" s="11" t="s">
+        <v>783</v>
+      </c>
+      <c r="I106" s="4" t="s">
+        <v>792</v>
+      </c>
+      <c r="J106" s="1" t="s">
+        <v>688</v>
+      </c>
+      <c r="L106" s="1" t="s">
+        <v>51</v>
+      </c>
+      <c r="M106" s="1" t="s">
+        <v>689</v>
+      </c>
+    </row>
+    <row r="107" spans="1:13" ht="14.4" x14ac:dyDescent="0.3">
+      <c r="A107" s="1" t="s">
+        <v>784</v>
+      </c>
+      <c r="B107" s="1" t="s">
+        <v>785</v>
+      </c>
+      <c r="C107" s="1" t="s">
+        <v>786</v>
+      </c>
+      <c r="D107" s="4" t="s">
+        <v>787</v>
+      </c>
+      <c r="E107" s="18" t="s">
+        <v>788</v>
+      </c>
+      <c r="F107" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="G107" t="s">
+        <v>789</v>
+      </c>
+      <c r="H107" s="4" t="s">
+        <v>790</v>
+      </c>
+      <c r="I107" s="4" t="s">
+        <v>791</v>
+      </c>
+      <c r="J107" s="1" t="s">
+        <v>688</v>
+      </c>
+      <c r="L107" s="1" t="s">
+        <v>470</v>
+      </c>
+      <c r="M107" s="1" t="s">
+        <v>689</v>
+      </c>
+    </row>
+    <row r="108" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A108" s="2" t="s">
+        <v>793</v>
+      </c>
+      <c r="B108" s="1" t="s">
+        <v>718</v>
+      </c>
+      <c r="C108" s="1" t="s">
+        <v>794</v>
+      </c>
+      <c r="D108" s="4" t="s">
+        <v>795</v>
+      </c>
+      <c r="E108" t="s">
+        <v>796</v>
+      </c>
+      <c r="F108" s="1" t="s">
+        <v>49</v>
+      </c>
+      <c r="G108" t="s">
+        <v>797</v>
+      </c>
+      <c r="H108" s="11" t="s">
+        <v>798</v>
+      </c>
+      <c r="J108" s="1" t="s">
+        <v>743</v>
+      </c>
+      <c r="K108" s="1">
+        <v>2010</v>
+      </c>
+      <c r="L108" s="1" t="s">
+        <v>799</v>
+      </c>
+      <c r="M108" s="1" t="s">
+        <v>689</v>
+      </c>
+    </row>
+    <row r="109" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A109" s="2" t="s">
+        <v>800</v>
+      </c>
+      <c r="B109" s="1" t="s">
+        <v>718</v>
+      </c>
+      <c r="C109" s="1" t="s">
+        <v>801</v>
+      </c>
+      <c r="D109" s="4" t="s">
+        <v>802</v>
+      </c>
+      <c r="E109" t="s">
+        <v>803</v>
+      </c>
+      <c r="F109" s="1" t="s">
+        <v>49</v>
+      </c>
+      <c r="G109" t="s">
+        <v>804</v>
+      </c>
+      <c r="H109" s="4" t="s">
+        <v>806</v>
+      </c>
+      <c r="I109" s="4" t="s">
+        <v>805</v>
+      </c>
+      <c r="J109" s="1" t="s">
+        <v>688</v>
+      </c>
+      <c r="K109" s="1">
+        <v>2008</v>
+      </c>
+      <c r="L109" s="1" t="s">
+        <v>446</v>
+      </c>
+      <c r="M109" s="1" t="s">
+        <v>689</v>
+      </c>
+    </row>
+    <row r="110" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A110" s="2" t="s">
+        <v>807</v>
+      </c>
+      <c r="B110" s="1" t="s">
+        <v>718</v>
+      </c>
+      <c r="C110" s="1" t="s">
+        <v>808</v>
+      </c>
+      <c r="D110" s="4" t="s">
+        <v>809</v>
+      </c>
+      <c r="E110" t="s">
+        <v>810</v>
+      </c>
+      <c r="F110" s="1" t="s">
+        <v>467</v>
+      </c>
+      <c r="G110" t="s">
+        <v>811</v>
+      </c>
+      <c r="H110" s="8">
+        <v>9611786456</v>
+      </c>
+      <c r="I110" s="4" t="s">
+        <v>812</v>
+      </c>
+      <c r="J110" s="1" t="s">
+        <v>688</v>
+      </c>
+      <c r="K110" s="1">
+        <v>1924</v>
+      </c>
+      <c r="L110" s="1" t="s">
+        <v>548</v>
+      </c>
+      <c r="M110" s="1" t="s">
+        <v>689</v>
+      </c>
+    </row>
+    <row r="111" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A111" s="2" t="s">
+        <v>813</v>
+      </c>
+      <c r="B111" s="1" t="s">
+        <v>718</v>
+      </c>
+      <c r="C111" s="1" t="s">
+        <v>814</v>
+      </c>
+      <c r="D111" s="4" t="s">
+        <v>815</v>
+      </c>
+      <c r="E111" t="s">
+        <v>816</v>
+      </c>
+      <c r="F111" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="G111" t="s">
+        <v>817</v>
+      </c>
+      <c r="H111" s="8">
+        <v>97145683911</v>
+      </c>
+      <c r="I111" s="4" t="s">
+        <v>818</v>
+      </c>
+      <c r="J111" s="1" t="s">
+        <v>688</v>
+      </c>
+      <c r="K111" s="1">
+        <v>2018</v>
+      </c>
+      <c r="L111" s="1" t="s">
+        <v>470</v>
+      </c>
+      <c r="M111" s="1" t="s">
+        <v>689</v>
+      </c>
+    </row>
+    <row r="112" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A112" s="2" t="s">
+        <v>819</v>
+      </c>
+      <c r="B112" s="1" t="s">
+        <v>820</v>
+      </c>
+      <c r="C112" s="1" t="s">
+        <v>821</v>
+      </c>
+      <c r="D112" s="4" t="s">
+        <v>822</v>
+      </c>
+      <c r="E112" t="s">
+        <v>823</v>
+      </c>
+      <c r="F112" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="G112" t="s">
+        <v>824</v>
+      </c>
+      <c r="H112" s="4" t="s">
+        <v>825</v>
+      </c>
+      <c r="I112" s="4" t="s">
+        <v>826</v>
+      </c>
+      <c r="J112" s="1" t="s">
+        <v>743</v>
+      </c>
+      <c r="K112" s="1">
+        <v>1988</v>
+      </c>
+      <c r="L112" s="1" t="s">
+        <v>470</v>
+      </c>
+      <c r="M112" s="1" t="s">
+        <v>689</v>
+      </c>
+    </row>
+    <row r="113" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A113" s="2" t="s">
+        <v>827</v>
+      </c>
+      <c r="B113" s="1" t="s">
+        <v>820</v>
+      </c>
+      <c r="C113" s="1" t="s">
+        <v>828</v>
+      </c>
+      <c r="D113" s="4" t="s">
+        <v>829</v>
+      </c>
+      <c r="E113" t="s">
+        <v>830</v>
+      </c>
+      <c r="F113" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="G113" t="s">
+        <v>831</v>
+      </c>
+      <c r="H113" s="11" t="s">
+        <v>833</v>
+      </c>
+      <c r="I113" s="4" t="s">
+        <v>832</v>
+      </c>
+      <c r="J113" s="1" t="s">
+        <v>696</v>
+      </c>
+      <c r="L113" s="1" t="s">
+        <v>470</v>
+      </c>
+      <c r="M113" s="1" t="s">
+        <v>689</v>
+      </c>
+    </row>
+    <row r="114" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A114" s="2" t="s">
+        <v>834</v>
+      </c>
+      <c r="B114" s="1" t="s">
+        <v>820</v>
+      </c>
+      <c r="C114" s="1" t="s">
+        <v>835</v>
+      </c>
+      <c r="D114" s="4" t="s">
+        <v>836</v>
+      </c>
+      <c r="E114" t="s">
+        <v>837</v>
+      </c>
+      <c r="F114" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="G114" t="s">
+        <v>838</v>
+      </c>
+      <c r="J114" s="1" t="s">
+        <v>696</v>
+      </c>
+      <c r="K114" s="1">
+        <v>2023</v>
+      </c>
+      <c r="L114" s="1" t="s">
+        <v>484</v>
+      </c>
+      <c r="M114" s="1" t="s">
+        <v>689</v>
+      </c>
+    </row>
+    <row r="115" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A115" s="2" t="s">
+        <v>839</v>
+      </c>
+      <c r="B115" s="1" t="s">
+        <v>820</v>
+      </c>
+      <c r="C115" s="1" t="s">
+        <v>840</v>
+      </c>
+      <c r="D115" s="4" t="s">
+        <v>841</v>
+      </c>
+      <c r="E115" t="s">
+        <v>842</v>
+      </c>
+      <c r="F115" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="G115" t="s">
+        <v>843</v>
+      </c>
+      <c r="H115" s="4" t="s">
+        <v>844</v>
+      </c>
+      <c r="I115" s="4" t="s">
+        <v>845</v>
+      </c>
+      <c r="J115" s="1" t="s">
+        <v>696</v>
+      </c>
+      <c r="K115" s="1">
+        <v>1964</v>
+      </c>
+      <c r="L115" s="1" t="s">
+        <v>51</v>
+      </c>
+      <c r="M115" s="1" t="s">
         <v>689</v>
       </c>
     </row>
@@ -6688,6 +7833,48 @@
     <hyperlink ref="D96" r:id="rId222" display="https://www.linkedin.com/in/jaber-al-mallah-3b89007/" xr:uid="{30A225BD-F162-48D1-A2EF-2576045F28AB}"/>
     <hyperlink ref="H96" r:id="rId223" display="tel:1828225" xr:uid="{82AD8865-24E5-4689-9116-31D40B81B8ED}"/>
     <hyperlink ref="I96" r:id="rId224" display="http://www.au.edu.kw/" xr:uid="{81CB9416-DE3B-44C4-92BD-84F27E39A96C}"/>
+    <hyperlink ref="D97" r:id="rId225" display="https://www.linkedin.com/in/karishma-joshi-914457190/" xr:uid="{B49E3D21-CAD0-428D-B6A7-ADFD9FA97D30}"/>
+    <hyperlink ref="I97" r:id="rId226" display="http://www.navitas.com/" xr:uid="{69A38D87-835C-4812-A39B-677257EBEE52}"/>
+    <hyperlink ref="D98" r:id="rId227" display="https://www.linkedin.com/in/ali-ezaldeen/" xr:uid="{501AADF1-DD32-40A5-B52D-82C4323AECF4}"/>
+    <hyperlink ref="I98" r:id="rId228" display="http://www.aurak.ac.ae/" xr:uid="{9E21094C-98CA-4D4A-B024-5DCEE8F28E41}"/>
+    <hyperlink ref="D99" r:id="rId229" display="https://www.linkedin.com/in/kevin-o-brien-321aaa27/" xr:uid="{C8F2F700-4C60-4C47-A451-6DA46C80F16F}"/>
+    <hyperlink ref="I99" r:id="rId230" xr:uid="{2E1916A4-A5BF-46CB-A6A7-9442A964B3AB}"/>
+    <hyperlink ref="D100" r:id="rId231" display="https://www.linkedin.com/in/lisa-paterson-4231a01b0/" xr:uid="{B85B6AF7-8CAE-4009-A9DD-5DDD6B5FB076}"/>
+    <hyperlink ref="I100" r:id="rId232" display="http://www.cognita.com/" xr:uid="{1EAD4FF3-853E-47C9-97FA-54AA7EE8CF88}"/>
+    <hyperlink ref="D101" r:id="rId233" display="https://www.linkedin.com/in/malika-benallal-a51b24150/" xr:uid="{8E5D0A7D-51E0-4733-8D65-AD1FAE1A4AED}"/>
+    <hyperlink ref="I101" r:id="rId234" xr:uid="{B88970E4-E07D-44DA-A57B-53B7BE50A0CA}"/>
+    <hyperlink ref="D102" r:id="rId235" display="https://www.linkedin.com/in/fedorina/" xr:uid="{F7911B1A-F8D1-4BD0-8B5A-E2B30C4A4B30}"/>
+    <hyperlink ref="I102" r:id="rId236" display="http://www.ward-howell.com/" xr:uid="{7E0A9104-CDDB-459F-BD98-EFB6A84F0E2E}"/>
+    <hyperlink ref="D103" r:id="rId237" display="https://www.linkedin.com/in/ibrahimalbidewi/" xr:uid="{60C23A25-E74E-4646-A6CF-2DFE3ED1CDED}"/>
+    <hyperlink ref="I103" r:id="rId238" display="http://www.moe.gov.sa/" xr:uid="{9C0043BC-35C4-445E-A6C5-5FBFECF2F6EE}"/>
+    <hyperlink ref="D104" r:id="rId239" display="https://www.linkedin.com/in/jb2026/" xr:uid="{656D6926-32C8-4ECC-B78F-463E74F6FACE}"/>
+    <hyperlink ref="I104" r:id="rId240" xr:uid="{A7653D34-5518-4370-95CF-E5B5A3F6F445}"/>
+    <hyperlink ref="D105" r:id="rId241" display="https://www.linkedin.com/in/annatraykova/" xr:uid="{9A90AEA0-35F8-4965-98F0-C104F730AD06}"/>
+    <hyperlink ref="I105" r:id="rId242" display="http://www.navitas.com/" xr:uid="{76807DD0-1C85-48EE-AF6B-2459F09ABA0A}"/>
+    <hyperlink ref="D106" r:id="rId243" display="https://www.linkedin.com/in/tarkan-ulas-49857069/" xr:uid="{A47E8C8E-000F-4881-9F68-E11B28CB62AF}"/>
+    <hyperlink ref="D107" r:id="rId244" display="https://www.linkedin.com/in/seham-nada-7215151b3/" xr:uid="{5B0F78B7-6384-499B-83D5-FAE0285586B4}"/>
+    <hyperlink ref="H107" r:id="rId245" display="tel:+971 45 788822" xr:uid="{16031B8F-DB29-46BD-B64E-83634BE7EEBC}"/>
+    <hyperlink ref="I107" r:id="rId246" xr:uid="{4B209AB2-CD8E-4F0F-A272-4CC6264A66F3}"/>
+    <hyperlink ref="I106" r:id="rId247" xr:uid="{1DD8FF70-E172-476F-BD1D-D2CB45C07739}"/>
+    <hyperlink ref="D108" r:id="rId248" display="https://www.linkedin.com/in/kutiba-nusair-82966564/" xr:uid="{9257BED0-2415-4B13-AC84-8129CC271A1C}"/>
+    <hyperlink ref="D109" r:id="rId249" display="https://www.linkedin.com/in/mohammad-al-nufaie-26252b88/" xr:uid="{ECBDD1AE-0840-42D3-89D5-30DB27E3571D}"/>
+    <hyperlink ref="I109" r:id="rId250" display="http://www.alfaisal.edu/" xr:uid="{AFE87D8C-EDFD-4CAA-878A-A19F1AA141AC}"/>
+    <hyperlink ref="H109" r:id="rId251" display="tel:920 000570" xr:uid="{710A4142-BDDC-4D9E-96A0-7C40EF1CAC29}"/>
+    <hyperlink ref="D110" r:id="rId252" display="https://www.linkedin.com/in/rim-tabaja-6664ba105/" xr:uid="{E4A35E5E-DC26-4C37-A76B-855EB12B47D1}"/>
+    <hyperlink ref="H110" r:id="rId253" display="tel:9611786456" xr:uid="{50FDD505-811E-48B8-830E-CD0F40BC6E57}"/>
+    <hyperlink ref="I110" r:id="rId254" xr:uid="{982873DD-85F0-4B67-9A25-38388C6A9618}"/>
+    <hyperlink ref="D111" r:id="rId255" display="https://www.linkedin.com/in/danna-herradura/" xr:uid="{B3CF92EC-3866-42BA-8542-488AE2B16FFB}"/>
+    <hyperlink ref="H111" r:id="rId256" display="tel:+97145683911" xr:uid="{5DE37C97-8702-41CC-95A9-CD7CC12BC57C}"/>
+    <hyperlink ref="I111" r:id="rId257" xr:uid="{EAEA7CD6-E0E7-46C9-A1E5-97A190408739}"/>
+    <hyperlink ref="D112" r:id="rId258" display="https://www.linkedin.com/in/abhishek-sachin-8362b4169/" xr:uid="{0B935AA2-6ED7-46DD-839B-BE862CC777F8}"/>
+    <hyperlink ref="H112" r:id="rId259" display="tel:(+971)567461832" xr:uid="{5628A06E-D838-45A2-AD29-D5218E4CC123}"/>
+    <hyperlink ref="I112" r:id="rId260" xr:uid="{ADBD3E39-8992-4E6F-894F-68FA77B1B219}"/>
+    <hyperlink ref="D113" r:id="rId261" display="https://www.linkedin.com/in/emily-horsford-440a0375/" xr:uid="{EBDF6101-291A-4C1B-982D-34DB12568016}"/>
+    <hyperlink ref="I113" r:id="rId262" display="https://harrowdubai.ae/" xr:uid="{7F402EE2-14A7-4A88-AF60-4D5622A39256}"/>
+    <hyperlink ref="D114" r:id="rId263" display="https://www.linkedin.com/in/joshua-david-mibd/" xr:uid="{82A1C4B8-83F5-4F4B-8A74-159E8964C573}"/>
+    <hyperlink ref="D115" r:id="rId264" xr:uid="{12630422-7BF2-49B8-9243-5285A6D21E18}"/>
+    <hyperlink ref="H115" r:id="rId265" display="tel:+44 (0)20 70007000" xr:uid="{AD62242C-6F8D-4C6C-9382-3939A28C788C}"/>
+    <hyperlink ref="I115" r:id="rId266" xr:uid="{247AE263-1B19-4870-962B-C2545D2A9E90}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Add day 32 progress
</commit_message>
<xml_diff>
--- a/Defining ICP/Defined Leads.xlsx
+++ b/Defining ICP/Defined Leads.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\R E E M\Documents\EVA Ops Training\Defining ICP\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A6BF626A-FD42-43DF-94D4-683DC81572E2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1F80A39E-6033-4465-B47B-CA223A2E55E9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="1152" yWindow="1284" windowWidth="17280" windowHeight="9960" xr2:uid="{DAB7335F-B748-4A40-8146-0BCBFC1873B2}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1306" uniqueCount="846">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1365" uniqueCount="881">
   <si>
     <t>Name</t>
   </si>
@@ -2576,6 +2576,111 @@
   </si>
   <si>
     <t>https://www.london.edu/</t>
+  </si>
+  <si>
+    <t>Manar El Halabi</t>
+  </si>
+  <si>
+    <t>ESA Business School</t>
+  </si>
+  <si>
+    <t>Manar El Halabi | LinkedIn</t>
+  </si>
+  <si>
+    <t>Head of Admissions at ESA Business School overseeing admissions operations, enrollment management, and student recruitment activities.</t>
+  </si>
+  <si>
+    <t>elhalabi.m@esa.edu.lb</t>
+  </si>
+  <si>
+    <t>http://www.esa.edu.lb/</t>
+  </si>
+  <si>
+    <t>+961 1 373 373</t>
+  </si>
+  <si>
+    <t>Ilona Arakilo</t>
+  </si>
+  <si>
+    <t>Head of Admissions</t>
+  </si>
+  <si>
+    <t>Edways</t>
+  </si>
+  <si>
+    <t>Ilona Arakilo | LinkedIn</t>
+  </si>
+  <si>
+    <t>Head of Admissions at Edways, responsible for managing school admissions and enrollment support services for families across Dubai.</t>
+  </si>
+  <si>
+    <t>ilona@edways.com</t>
+  </si>
+  <si>
+    <t>+971 58 298 5331</t>
+  </si>
+  <si>
+    <t>www.edways.com</t>
+  </si>
+  <si>
+    <t>Sara Zeineddine</t>
+  </si>
+  <si>
+    <t>East International University</t>
+  </si>
+  <si>
+    <t>Sara Zeineddine | LinkedIn</t>
+  </si>
+  <si>
+    <t>Admissions Manager at East International University responsible for admissions operations, student recruitment, application processing, and enrollment management.</t>
+  </si>
+  <si>
+    <t>szeineddine@azmuniversity.edu.lb</t>
+  </si>
+  <si>
+    <t>eiu.edu.lb</t>
+  </si>
+  <si>
+    <t>Sophie Aden</t>
+  </si>
+  <si>
+    <t>Athena Global Education</t>
+  </si>
+  <si>
+    <t>Sophie Aden | LinkedIn</t>
+  </si>
+  <si>
+    <t>Admissions Manager at Athena Global Education responsible for student admissions, enrollment management, applicant tracking, and admissions operations.</t>
+  </si>
+  <si>
+    <t>sophie@uniathena.com</t>
+  </si>
+  <si>
+    <t>https://uniathena.com/</t>
+  </si>
+  <si>
+    <t>+971 55 879 5492</t>
+  </si>
+  <si>
+    <t>Lama Musallam</t>
+  </si>
+  <si>
+    <t>GEMS Metropole School – Al Waha</t>
+  </si>
+  <si>
+    <t>Lama Musallam | LinkedIn</t>
+  </si>
+  <si>
+    <t>Admissions Manager at GEMS Metropole School – Al Waha overseeing student enrollment, admissions processes, applicant tracking, and family engagement activities.</t>
+  </si>
+  <si>
+    <t>l.musallam_mtw@gemsedu.com</t>
+  </si>
+  <si>
+    <t>+971 4 526 6555</t>
+  </si>
+  <si>
+    <t>https://www.gemsmetropoleschool-alwaha.com/</t>
   </si>
 </sst>
 </file>
@@ -3031,7 +3136,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3B2D820C-3568-45BE-99C1-F7479358E85B}">
-  <dimension ref="A1:M115"/>
+  <dimension ref="A1:M120"/>
   <sheetFormatPr defaultRowHeight="15.6" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="23.33203125" style="2" bestFit="1" customWidth="1"/>
@@ -3042,7 +3147,7 @@
     <col min="6" max="6" width="12.77734375" style="1" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="46.5546875" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="18.44140625" style="11" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="42.109375" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="47.88671875" bestFit="1" customWidth="1"/>
     <col min="10" max="10" width="25.77734375" style="1" bestFit="1" customWidth="1"/>
     <col min="11" max="11" width="11.77734375" style="1" customWidth="1"/>
     <col min="12" max="12" width="11" style="1" bestFit="1" customWidth="1"/>
@@ -7603,6 +7708,211 @@
         <v>51</v>
       </c>
       <c r="M115" s="1" t="s">
+        <v>689</v>
+      </c>
+    </row>
+    <row r="116" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A116" s="2" t="s">
+        <v>846</v>
+      </c>
+      <c r="B116" s="1" t="s">
+        <v>820</v>
+      </c>
+      <c r="C116" s="1" t="s">
+        <v>847</v>
+      </c>
+      <c r="D116" s="4" t="s">
+        <v>848</v>
+      </c>
+      <c r="E116" t="s">
+        <v>849</v>
+      </c>
+      <c r="F116" s="1" t="s">
+        <v>467</v>
+      </c>
+      <c r="G116" t="s">
+        <v>850</v>
+      </c>
+      <c r="H116" s="11" t="s">
+        <v>852</v>
+      </c>
+      <c r="I116" s="4" t="s">
+        <v>851</v>
+      </c>
+      <c r="J116" s="1" t="s">
+        <v>688</v>
+      </c>
+      <c r="K116" s="1">
+        <v>1996</v>
+      </c>
+      <c r="L116" s="1" t="s">
+        <v>470</v>
+      </c>
+      <c r="M116" s="1" t="s">
+        <v>689</v>
+      </c>
+    </row>
+    <row r="117" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A117" s="2" t="s">
+        <v>853</v>
+      </c>
+      <c r="B117" s="1" t="s">
+        <v>854</v>
+      </c>
+      <c r="C117" s="1" t="s">
+        <v>855</v>
+      </c>
+      <c r="D117" s="4" t="s">
+        <v>856</v>
+      </c>
+      <c r="E117" t="s">
+        <v>857</v>
+      </c>
+      <c r="F117" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="G117" t="s">
+        <v>858</v>
+      </c>
+      <c r="H117" s="4" t="s">
+        <v>859</v>
+      </c>
+      <c r="I117" s="4" t="s">
+        <v>860</v>
+      </c>
+      <c r="J117" s="1" t="s">
+        <v>696</v>
+      </c>
+      <c r="K117" s="1">
+        <v>2023</v>
+      </c>
+      <c r="L117" s="1" t="s">
+        <v>518</v>
+      </c>
+      <c r="M117" s="1" t="s">
+        <v>689</v>
+      </c>
+    </row>
+    <row r="118" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A118" s="2" t="s">
+        <v>861</v>
+      </c>
+      <c r="B118" s="1" t="s">
+        <v>820</v>
+      </c>
+      <c r="C118" s="1" t="s">
+        <v>862</v>
+      </c>
+      <c r="D118" s="4" t="s">
+        <v>863</v>
+      </c>
+      <c r="E118" t="s">
+        <v>864</v>
+      </c>
+      <c r="F118" s="1" t="s">
+        <v>467</v>
+      </c>
+      <c r="G118" t="s">
+        <v>865</v>
+      </c>
+      <c r="H118" s="8">
+        <v>6446571</v>
+      </c>
+      <c r="I118" s="4" t="s">
+        <v>866</v>
+      </c>
+      <c r="J118" s="1" t="s">
+        <v>688</v>
+      </c>
+      <c r="K118" s="1">
+        <v>2015</v>
+      </c>
+      <c r="L118" s="1" t="s">
+        <v>446</v>
+      </c>
+      <c r="M118" s="1" t="s">
+        <v>689</v>
+      </c>
+    </row>
+    <row r="119" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A119" s="2" t="s">
+        <v>867</v>
+      </c>
+      <c r="B119" s="1" t="s">
+        <v>820</v>
+      </c>
+      <c r="C119" s="1" t="s">
+        <v>868</v>
+      </c>
+      <c r="D119" s="4" t="s">
+        <v>869</v>
+      </c>
+      <c r="E119" t="s">
+        <v>870</v>
+      </c>
+      <c r="F119" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="G119" t="s">
+        <v>871</v>
+      </c>
+      <c r="H119" s="11" t="s">
+        <v>873</v>
+      </c>
+      <c r="I119" s="4" t="s">
+        <v>872</v>
+      </c>
+      <c r="J119" s="1" t="s">
+        <v>688</v>
+      </c>
+      <c r="K119" s="1">
+        <v>2019</v>
+      </c>
+      <c r="L119" s="1" t="s">
+        <v>470</v>
+      </c>
+      <c r="M119" s="1" t="s">
+        <v>689</v>
+      </c>
+    </row>
+    <row r="120" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A120" s="2" t="s">
+        <v>874</v>
+      </c>
+      <c r="B120" s="1" t="s">
+        <v>820</v>
+      </c>
+      <c r="C120" s="1" t="s">
+        <v>875</v>
+      </c>
+      <c r="D120" s="4" t="s">
+        <v>876</v>
+      </c>
+      <c r="E120" t="s">
+        <v>877</v>
+      </c>
+      <c r="F120" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="G120" t="s">
+        <v>878</v>
+      </c>
+      <c r="H120" s="11" t="s">
+        <v>879</v>
+      </c>
+      <c r="I120" s="4" t="s">
+        <v>880</v>
+      </c>
+      <c r="J120" s="1" t="s">
+        <v>696</v>
+      </c>
+      <c r="K120" s="1">
+        <v>2023</v>
+      </c>
+      <c r="L120" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="M120" s="1" t="s">
         <v>689</v>
       </c>
     </row>
@@ -7875,6 +8185,17 @@
     <hyperlink ref="D115" r:id="rId264" xr:uid="{12630422-7BF2-49B8-9243-5285A6D21E18}"/>
     <hyperlink ref="H115" r:id="rId265" display="tel:+44 (0)20 70007000" xr:uid="{AD62242C-6F8D-4C6C-9382-3939A28C788C}"/>
     <hyperlink ref="I115" r:id="rId266" xr:uid="{247AE263-1B19-4870-962B-C2545D2A9E90}"/>
+    <hyperlink ref="D116" r:id="rId267" display="https://www.linkedin.com/in/manar-el-halabi-3853bb97/" xr:uid="{FE9F8F38-DB82-49D5-970B-1D5962409965}"/>
+    <hyperlink ref="I116" r:id="rId268" xr:uid="{4968D991-A526-416B-A447-2D5CA9114C71}"/>
+    <hyperlink ref="D117" r:id="rId269" display="https://www.linkedin.com/in/ilona-arakilo-a40816125/" xr:uid="{0716C298-EAD6-48FE-AF23-A91B93BD63F1}"/>
+    <hyperlink ref="H117" r:id="rId270" display="tel:+971 58 298 5331" xr:uid="{1375BA65-4F19-4594-9DD1-28E129FEA6B5}"/>
+    <hyperlink ref="I117" r:id="rId271" display="https://www.edways.com/" xr:uid="{08DB9DEC-47FD-45AC-BAFE-8EED38B1F101}"/>
+    <hyperlink ref="D118" r:id="rId272" display="https://www.linkedin.com/in/sara-zeineddine-4440b321b/" xr:uid="{999DAEC2-297D-4D76-ACF4-D4CF3CE08FB2}"/>
+    <hyperlink ref="H118" r:id="rId273" display="tel:06446571" xr:uid="{8B6D4D2C-E318-40D1-ADCB-43449192776C}"/>
+    <hyperlink ref="I118" r:id="rId274" display="https://eiu.edu.lb/" xr:uid="{8780CC80-AC2A-4C69-AC79-CF14B703B1DA}"/>
+    <hyperlink ref="D119" r:id="rId275" display="https://www.linkedin.com/in/sophie-aden-baa9121a8/" xr:uid="{B894DBD8-2EB2-45B9-A293-F00639806413}"/>
+    <hyperlink ref="I119" r:id="rId276" xr:uid="{8242B6AE-5BE3-48E8-B74E-F01C00CE7649}"/>
+    <hyperlink ref="D120" r:id="rId277" display="https://www.linkedin.com/in/lama-musallam-3a11b6aa/" xr:uid="{B6154992-5153-487D-91B3-4F124E70D2B7}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>